<commit_message>
Update forest data - 2026-02-23 12:34
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2592" uniqueCount="1307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2617" uniqueCount="1319">
   <si>
     <t>link</t>
   </si>
@@ -3939,6 +3939,42 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/preilu-pag/cckmx.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/ambelu-pag/bkxli.html</t>
+  </si>
+  <si>
+    <t>64 500 €</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/asunes-pag/ihdfn.html</t>
+  </si>
+  <si>
+    <t>1.95 ha.</t>
+  </si>
+  <si>
+    <t>60460010036</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/skaistas-pag/ljohg.html</t>
+  </si>
+  <si>
+    <t>105 000 €</t>
+  </si>
+  <si>
+    <t>69880090057</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/talsi-and-reg/vandzenes-pag/ienlj.html</t>
+  </si>
+  <si>
+    <t>88940050107</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/tukums-and-reg/dzukstes-pag/fpkoj.html</t>
+  </si>
+  <si>
+    <t>90480060028</t>
   </si>
 </sst>
 </file>
@@ -4351,7 +4387,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F514"/>
+  <dimension ref="A1:F517"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -14640,6 +14676,66 @@
       </c>
       <c r="F514" s="2">
         <v>46072.54166666667</v>
+      </c>
+    </row>
+    <row r="515" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A515" s="3" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B515" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C515" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D515" s="4" t="s">
+        <v>1303</v>
+      </c>
+      <c r="E515" s="4" t="s">
+        <v>1304</v>
+      </c>
+      <c r="F515" s="2">
+        <v>46072.90694444445</v>
+      </c>
+    </row>
+    <row r="516" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A516" s="3" t="s">
+        <v>1305</v>
+      </c>
+      <c r="B516" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C516" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D516" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E516" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F516" s="2">
+        <v>46073.47083333333</v>
+      </c>
+    </row>
+    <row r="517" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A517" s="3" t="s">
+        <v>1306</v>
+      </c>
+      <c r="B517" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="C517" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D517" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E517" s="4" t="s">
+        <v>1301</v>
+      </c>
+      <c r="F517" s="2">
+        <v>46072.83888888889</v>
       </c>
     </row>
   </sheetData>
@@ -15157,6 +15253,9 @@
     <hyperlink ref="A512" r:id="rId511"/>
     <hyperlink ref="A513" r:id="rId512"/>
     <hyperlink ref="A514" r:id="rId513"/>
+    <hyperlink ref="A515" r:id="rId514"/>
+    <hyperlink ref="A516" r:id="rId515"/>
+    <hyperlink ref="A517" r:id="rId516"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -15168,7 +15267,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -15201,62 +15300,102 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1302</v>
+        <v>1307</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>88</v>
+        <v>1308</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>28</v>
+        <v>74</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>1303</v>
+        <v>162</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1304</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46072.90694444445</v>
+        <v>46073.68541666667</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1305</v>
+        <v>1309</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>106</v>
+        <v>707</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>124</v>
+        <v>146</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>135</v>
+        <v>1310</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>25</v>
+        <v>1311</v>
       </c>
       <c r="F3" s="2">
-        <v>46073.47083333333</v>
+        <v>46074.5375</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>1306</v>
+        <v>1312</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>467</v>
+        <v>1313</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>284</v>
+        <v>146</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>36</v>
+        <v>699</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>1301</v>
+        <v>1314</v>
       </c>
       <c r="F4" s="2">
-        <v>46072.83888888889</v>
+        <v>46073.71319444444</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1315</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>843</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1316</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46074.736805555556</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>1317</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>1318</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46076.59166666667</v>
       </c>
     </row>
   </sheetData>
@@ -15264,6 +15403,8 @@
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
     <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+    <hyperlink ref="A6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-02-24 12:35
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2617" uniqueCount="1319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2627" uniqueCount="1322">
   <si>
     <t>link</t>
   </si>
@@ -3975,6 +3975,15 @@
   </si>
   <si>
     <t>90480060028</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/limbadzi-and-reg/ainazu-l-t/icmki.html</t>
+  </si>
+  <si>
+    <t>66250030323</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/tukums-and-reg/dzukstes-pag/gfjjm.html</t>
   </si>
 </sst>
 </file>
@@ -4387,7 +4396,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F517"/>
+  <dimension ref="A1:F522"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -14736,6 +14745,106 @@
       </c>
       <c r="F517" s="2">
         <v>46072.83888888889</v>
+      </c>
+    </row>
+    <row r="518" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A518" s="3" t="s">
+        <v>1307</v>
+      </c>
+      <c r="B518" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C518" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D518" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="E518" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F518" s="2">
+        <v>46073.68541666667</v>
+      </c>
+    </row>
+    <row r="519" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A519" s="3" t="s">
+        <v>1309</v>
+      </c>
+      <c r="B519" s="4" t="s">
+        <v>707</v>
+      </c>
+      <c r="C519" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D519" s="4" t="s">
+        <v>1310</v>
+      </c>
+      <c r="E519" s="4" t="s">
+        <v>1311</v>
+      </c>
+      <c r="F519" s="2">
+        <v>46074.5375</v>
+      </c>
+    </row>
+    <row r="520" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A520" s="3" t="s">
+        <v>1312</v>
+      </c>
+      <c r="B520" s="4" t="s">
+        <v>1313</v>
+      </c>
+      <c r="C520" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D520" s="4" t="s">
+        <v>699</v>
+      </c>
+      <c r="E520" s="4" t="s">
+        <v>1314</v>
+      </c>
+      <c r="F520" s="2">
+        <v>46073.71319444444</v>
+      </c>
+    </row>
+    <row r="521" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A521" s="3" t="s">
+        <v>1315</v>
+      </c>
+      <c r="B521" s="4" t="s">
+        <v>843</v>
+      </c>
+      <c r="C521" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="D521" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E521" s="4" t="s">
+        <v>1316</v>
+      </c>
+      <c r="F521" s="2">
+        <v>46074.736805555556</v>
+      </c>
+    </row>
+    <row r="522" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A522" s="3" t="s">
+        <v>1317</v>
+      </c>
+      <c r="B522" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="C522" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D522" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E522" s="4" t="s">
+        <v>1318</v>
+      </c>
+      <c r="F522" s="2">
+        <v>46076.59166666667</v>
       </c>
     </row>
   </sheetData>
@@ -15256,6 +15365,11 @@
     <hyperlink ref="A515" r:id="rId514"/>
     <hyperlink ref="A516" r:id="rId515"/>
     <hyperlink ref="A517" r:id="rId516"/>
+    <hyperlink ref="A518" r:id="rId517"/>
+    <hyperlink ref="A519" r:id="rId518"/>
+    <hyperlink ref="A520" r:id="rId519"/>
+    <hyperlink ref="A521" r:id="rId520"/>
+    <hyperlink ref="A522" r:id="rId521"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -15267,7 +15381,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -15300,111 +15414,48 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1307</v>
+        <v>1319</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1308</v>
+        <v>116</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>74</v>
+        <v>208</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>162</v>
+        <v>930</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>25</v>
+        <v>1320</v>
       </c>
       <c r="F2" s="2">
-        <v>46073.68541666667</v>
+        <v>46076.69305555556</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1309</v>
+        <v>1321</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>707</v>
+        <v>533</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>146</v>
+        <v>376</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>1310</v>
+        <v>169</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1311</v>
+        <v>1318</v>
       </c>
       <c r="F3" s="2">
-        <v>46074.5375</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1312</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>1313</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>699</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1314</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46073.71319444444</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1315</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>843</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>356</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1316</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46074.736805555556</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>1317</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>533</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>376</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>1318</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46076.59166666667</v>
+        <v>46077.410416666666</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-02-25 12:34
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2627" uniqueCount="1322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2632" uniqueCount="1324">
   <si>
     <t>link</t>
   </si>
@@ -3984,6 +3984,12 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/tukums-and-reg/dzukstes-pag/gfjjm.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/liepaja-and-reg/aizputes-pag/beolce.html</t>
+  </si>
+  <si>
+    <t>64420060044</t>
   </si>
 </sst>
 </file>
@@ -4396,7 +4402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F522"/>
+  <dimension ref="A1:F524"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -14845,6 +14851,46 @@
       </c>
       <c r="F522" s="2">
         <v>46076.59166666667</v>
+      </c>
+    </row>
+    <row r="523" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A523" s="3" t="s">
+        <v>1319</v>
+      </c>
+      <c r="B523" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C523" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D523" s="4" t="s">
+        <v>930</v>
+      </c>
+      <c r="E523" s="4" t="s">
+        <v>1320</v>
+      </c>
+      <c r="F523" s="2">
+        <v>46076.69305555556</v>
+      </c>
+    </row>
+    <row r="524" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A524" s="3" t="s">
+        <v>1321</v>
+      </c>
+      <c r="B524" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="C524" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D524" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E524" s="4" t="s">
+        <v>1318</v>
+      </c>
+      <c r="F524" s="2">
+        <v>46077.410416666666</v>
       </c>
     </row>
   </sheetData>
@@ -15370,6 +15416,8 @@
     <hyperlink ref="A520" r:id="rId519"/>
     <hyperlink ref="A521" r:id="rId520"/>
     <hyperlink ref="A522" r:id="rId521"/>
+    <hyperlink ref="A523" r:id="rId522"/>
+    <hyperlink ref="A524" r:id="rId523"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -15381,7 +15429,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -15414,48 +15462,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1319</v>
+        <v>1322</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>116</v>
+        <v>217</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>208</v>
+        <v>190</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>930</v>
+        <v>67</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1320</v>
+        <v>1323</v>
       </c>
       <c r="F2" s="2">
-        <v>46076.69305555556</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1321</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>533</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>376</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1318</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46077.410416666666</v>
+        <v>46077.69583333333</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-02-26 12:35
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2632" uniqueCount="1324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2667" uniqueCount="1340">
   <si>
     <t>link</t>
   </si>
@@ -3990,6 +3990,54 @@
   </si>
   <si>
     <t>64420060044</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/dubnas-pag/phffg.html</t>
+  </si>
+  <si>
+    <t>22 050 €</t>
+  </si>
+  <si>
+    <t>44520030223</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/dobele-and-reg/iles-pag/mjnbl.html</t>
+  </si>
+  <si>
+    <t>66 150 €</t>
+  </si>
+  <si>
+    <t>46640020168</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/andrupenes-pag/jinjp.html</t>
+  </si>
+  <si>
+    <t>78 750 €</t>
+  </si>
+  <si>
+    <t>31 ha.</t>
+  </si>
+  <si>
+    <t>60420010026</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ludza-and-reg/merdzenes-pag/dpxic.html</t>
+  </si>
+  <si>
+    <t>68720070080</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/upmalas-pag/ioglc.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/rozkalnu-pag/mnbll.html</t>
+  </si>
+  <si>
+    <t>76640020109</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/kaunatas-pag/oxook.html</t>
   </si>
 </sst>
 </file>
@@ -4402,7 +4450,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F524"/>
+  <dimension ref="A1:F525"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -14891,6 +14939,26 @@
       </c>
       <c r="F524" s="2">
         <v>46077.410416666666</v>
+      </c>
+    </row>
+    <row r="525" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A525" s="3" t="s">
+        <v>1322</v>
+      </c>
+      <c r="B525" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="C525" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="D525" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E525" s="4" t="s">
+        <v>1323</v>
+      </c>
+      <c r="F525" s="2">
+        <v>46077.69583333333</v>
       </c>
     </row>
   </sheetData>
@@ -15418,6 +15486,7 @@
     <hyperlink ref="A522" r:id="rId521"/>
     <hyperlink ref="A523" r:id="rId522"/>
     <hyperlink ref="A524" r:id="rId523"/>
+    <hyperlink ref="A525" r:id="rId524"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -15429,7 +15498,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -15462,27 +15531,153 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1322</v>
+        <v>1324</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>217</v>
+        <v>1325</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>190</v>
+        <v>74</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>67</v>
+        <v>154</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1323</v>
+        <v>1326</v>
       </c>
       <c r="F2" s="2">
-        <v>46077.69583333333</v>
+        <v>46079.52083333333</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1327</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>1328</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1329</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46079.52777777778</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1330</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>1331</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>1332</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1333</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46079.53680555556</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1334</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1335</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46078.745833333334</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>1336</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>1175</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46079.36458333333</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>1337</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46079.3625</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>1339</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" s="2">
+        <v>46079.4625</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+    <hyperlink ref="A6" r:id="rId5"/>
+    <hyperlink ref="A7" r:id="rId6"/>
+    <hyperlink ref="A8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-02-27 12:30
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2667" uniqueCount="1340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2682" uniqueCount="1347">
   <si>
     <t>link</t>
   </si>
@@ -4038,6 +4038,27 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/kaunatas-pag/oxook.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/berzpils-pag/kfhhh.html</t>
+  </si>
+  <si>
+    <t>9 600 €</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/gulbene-and-reg/rankas-pag/dcxdx.html</t>
+  </si>
+  <si>
+    <t>1.55 ha.</t>
+  </si>
+  <si>
+    <t>50840030030</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jelgava-and-reg/kalnciems/cgjmhd.html</t>
+  </si>
+  <si>
+    <t>79 500 €</t>
   </si>
 </sst>
 </file>
@@ -4450,7 +4471,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F525"/>
+  <dimension ref="A1:F532"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -14959,6 +14980,146 @@
       </c>
       <c r="F525" s="2">
         <v>46077.69583333333</v>
+      </c>
+    </row>
+    <row r="526" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A526" s="3" t="s">
+        <v>1324</v>
+      </c>
+      <c r="B526" s="4" t="s">
+        <v>1325</v>
+      </c>
+      <c r="C526" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D526" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="E526" s="4" t="s">
+        <v>1326</v>
+      </c>
+      <c r="F526" s="2">
+        <v>46079.52083333333</v>
+      </c>
+    </row>
+    <row r="527" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A527" s="3" t="s">
+        <v>1327</v>
+      </c>
+      <c r="B527" s="4" t="s">
+        <v>1328</v>
+      </c>
+      <c r="C527" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D527" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E527" s="4" t="s">
+        <v>1329</v>
+      </c>
+      <c r="F527" s="2">
+        <v>46079.52777777778</v>
+      </c>
+    </row>
+    <row r="528" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A528" s="3" t="s">
+        <v>1330</v>
+      </c>
+      <c r="B528" s="4" t="s">
+        <v>1331</v>
+      </c>
+      <c r="C528" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D528" s="4" t="s">
+        <v>1332</v>
+      </c>
+      <c r="E528" s="4" t="s">
+        <v>1333</v>
+      </c>
+      <c r="F528" s="2">
+        <v>46079.53680555556</v>
+      </c>
+    </row>
+    <row r="529" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A529" s="3" t="s">
+        <v>1334</v>
+      </c>
+      <c r="B529" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C529" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D529" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E529" s="4" t="s">
+        <v>1335</v>
+      </c>
+      <c r="F529" s="2">
+        <v>46078.745833333334</v>
+      </c>
+    </row>
+    <row r="530" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A530" s="3" t="s">
+        <v>1336</v>
+      </c>
+      <c r="B530" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="C530" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D530" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E530" s="4" t="s">
+        <v>1175</v>
+      </c>
+      <c r="F530" s="2">
+        <v>46079.36458333333</v>
+      </c>
+    </row>
+    <row r="531" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A531" s="3" t="s">
+        <v>1337</v>
+      </c>
+      <c r="B531" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="C531" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D531" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E531" s="4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="F531" s="2">
+        <v>46079.3625</v>
+      </c>
+    </row>
+    <row r="532" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A532" s="3" t="s">
+        <v>1339</v>
+      </c>
+      <c r="B532" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C532" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D532" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E532" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F532" s="2">
+        <v>46079.4625</v>
       </c>
     </row>
   </sheetData>
@@ -15487,6 +15648,13 @@
     <hyperlink ref="A523" r:id="rId522"/>
     <hyperlink ref="A524" r:id="rId523"/>
     <hyperlink ref="A525" r:id="rId524"/>
+    <hyperlink ref="A526" r:id="rId525"/>
+    <hyperlink ref="A527" r:id="rId526"/>
+    <hyperlink ref="A528" r:id="rId527"/>
+    <hyperlink ref="A529" r:id="rId528"/>
+    <hyperlink ref="A530" r:id="rId529"/>
+    <hyperlink ref="A531" r:id="rId530"/>
+    <hyperlink ref="A532" r:id="rId531"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -15498,7 +15666,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -15531,142 +15699,62 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1324</v>
+        <v>1340</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1325</v>
+        <v>1341</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>74</v>
+        <v>28</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>154</v>
+        <v>186</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1326</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46079.52083333333</v>
+        <v>46080.57708333334</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1327</v>
+        <v>1342</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>1328</v>
+        <v>988</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>44</v>
+        <v>1343</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1329</v>
+        <v>1344</v>
       </c>
       <c r="F3" s="2">
-        <v>46079.52777777778</v>
+        <v>46080.513194444444</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>1330</v>
+        <v>1345</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>1331</v>
+        <v>1346</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>146</v>
+        <v>518</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>1332</v>
+        <v>67</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>1333</v>
+        <v>560</v>
       </c>
       <c r="F4" s="2">
-        <v>46079.53680555556</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1334</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1335</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46078.745833333334</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>1336</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>1175</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46079.36458333333</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>1337</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>1338</v>
-      </c>
-      <c r="F7" s="2">
-        <v>46079.3625</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>1339</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F8" s="2">
-        <v>46079.4625</v>
+        <v>46079.617361111115</v>
       </c>
     </row>
   </sheetData>
@@ -15674,10 +15762,6 @@
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
     <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A6" r:id="rId5"/>
-    <hyperlink ref="A7" r:id="rId6"/>
-    <hyperlink ref="A8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-03-02 12:32
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2682" uniqueCount="1347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2717" uniqueCount="1362">
   <si>
     <t>link</t>
   </si>
@@ -4059,6 +4059,51 @@
   </si>
   <si>
     <t>79 500 €</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/ambelu-pag/epjkp.html</t>
+  </si>
+  <si>
+    <t>44420050067</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/kalupes-pag/bpoklc.html</t>
+  </si>
+  <si>
+    <t>44620060021</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jelgava-and-reg/other/bxnndx.html</t>
+  </si>
+  <si>
+    <t>5.54 ha.</t>
+  </si>
+  <si>
+    <t>54780020011</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/ezernieku-pag/bdhnb.html</t>
+  </si>
+  <si>
+    <t>60560040240</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ludza-and-reg/istras-pag/boxkl.html</t>
+  </si>
+  <si>
+    <t>5.23 ha.</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ogre-and-reg/birzgales-pag/coiik.html</t>
+  </si>
+  <si>
+    <t>74440100020</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/struzanu-pag/bliixi.html</t>
+  </si>
+  <si>
+    <t>78940010006</t>
   </si>
 </sst>
 </file>
@@ -4471,7 +4516,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F532"/>
+  <dimension ref="A1:F535"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -15120,6 +15165,66 @@
       </c>
       <c r="F532" s="2">
         <v>46079.4625</v>
+      </c>
+    </row>
+    <row r="533" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A533" s="3" t="s">
+        <v>1340</v>
+      </c>
+      <c r="B533" s="4" t="s">
+        <v>1341</v>
+      </c>
+      <c r="C533" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D533" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E533" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F533" s="2">
+        <v>46080.57708333334</v>
+      </c>
+    </row>
+    <row r="534" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A534" s="3" t="s">
+        <v>1342</v>
+      </c>
+      <c r="B534" s="4" t="s">
+        <v>988</v>
+      </c>
+      <c r="C534" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D534" s="4" t="s">
+        <v>1343</v>
+      </c>
+      <c r="E534" s="4" t="s">
+        <v>1344</v>
+      </c>
+      <c r="F534" s="2">
+        <v>46080.513194444444</v>
+      </c>
+    </row>
+    <row r="535" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A535" s="3" t="s">
+        <v>1345</v>
+      </c>
+      <c r="B535" s="4" t="s">
+        <v>1346</v>
+      </c>
+      <c r="C535" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="D535" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E535" s="4" t="s">
+        <v>560</v>
+      </c>
+      <c r="F535" s="2">
+        <v>46079.617361111115</v>
       </c>
     </row>
   </sheetData>
@@ -15655,6 +15760,9 @@
     <hyperlink ref="A530" r:id="rId529"/>
     <hyperlink ref="A531" r:id="rId530"/>
     <hyperlink ref="A532" r:id="rId531"/>
+    <hyperlink ref="A533" r:id="rId532"/>
+    <hyperlink ref="A534" r:id="rId533"/>
+    <hyperlink ref="A535" r:id="rId534"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -15666,7 +15774,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -15699,62 +15807,142 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1340</v>
+        <v>1347</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1341</v>
+        <v>497</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>28</v>
+        <v>74</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>186</v>
+        <v>36</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>25</v>
+        <v>1348</v>
       </c>
       <c r="F2" s="2">
-        <v>46080.57708333334</v>
+        <v>46081.87569444445</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1342</v>
+        <v>1349</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>988</v>
+        <v>437</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>124</v>
+        <v>74</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>1343</v>
+        <v>154</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1344</v>
+        <v>1350</v>
       </c>
       <c r="F3" s="2">
-        <v>46080.513194444444</v>
+        <v>46081.586805555555</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>1345</v>
+        <v>1351</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>1346</v>
+        <v>31</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>518</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>67</v>
+        <v>1352</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>560</v>
+        <v>1353</v>
       </c>
       <c r="F4" s="2">
-        <v>46079.617361111115</v>
+        <v>46080.80069444445</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1354</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>1163</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1355</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46081.884722222225</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>1356</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>816</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>1357</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46081.620833333334</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>1358</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>1359</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46083.433333333334</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>1360</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>1361</v>
+      </c>
+      <c r="F8" s="2">
+        <v>46081.896527777775</v>
       </c>
     </row>
   </sheetData>
@@ -15762,6 +15950,10 @@
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
     <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+    <hyperlink ref="A6" r:id="rId5"/>
+    <hyperlink ref="A7" r:id="rId6"/>
+    <hyperlink ref="A8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-03-03 12:32
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2717" uniqueCount="1362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2732" uniqueCount="1368">
   <si>
     <t>link</t>
   </si>
@@ -4104,6 +4104,24 @@
   </si>
   <si>
     <t>78940010006</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/jaunaluksnes-pag/njkfd.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/lazdukalna-pag/coifx.html</t>
+  </si>
+  <si>
+    <t>14000 m²</t>
+  </si>
+  <si>
+    <t>38640080372</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/ligatnes-pag/dxemc.html</t>
+  </si>
+  <si>
+    <t>42620040875</t>
   </si>
 </sst>
 </file>
@@ -4516,7 +4534,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F535"/>
+  <dimension ref="A1:F542"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -15225,6 +15243,146 @@
       </c>
       <c r="F535" s="2">
         <v>46079.617361111115</v>
+      </c>
+    </row>
+    <row r="536" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A536" s="3" t="s">
+        <v>1347</v>
+      </c>
+      <c r="B536" s="4" t="s">
+        <v>497</v>
+      </c>
+      <c r="C536" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D536" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E536" s="4" t="s">
+        <v>1348</v>
+      </c>
+      <c r="F536" s="2">
+        <v>46081.87569444445</v>
+      </c>
+    </row>
+    <row r="537" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A537" s="3" t="s">
+        <v>1349</v>
+      </c>
+      <c r="B537" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="C537" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D537" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="E537" s="4" t="s">
+        <v>1350</v>
+      </c>
+      <c r="F537" s="2">
+        <v>46081.586805555555</v>
+      </c>
+    </row>
+    <row r="538" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A538" s="3" t="s">
+        <v>1351</v>
+      </c>
+      <c r="B538" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C538" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="D538" s="4" t="s">
+        <v>1352</v>
+      </c>
+      <c r="E538" s="4" t="s">
+        <v>1353</v>
+      </c>
+      <c r="F538" s="2">
+        <v>46080.80069444445</v>
+      </c>
+    </row>
+    <row r="539" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A539" s="3" t="s">
+        <v>1354</v>
+      </c>
+      <c r="B539" s="4" t="s">
+        <v>1163</v>
+      </c>
+      <c r="C539" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D539" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E539" s="4" t="s">
+        <v>1355</v>
+      </c>
+      <c r="F539" s="2">
+        <v>46081.884722222225</v>
+      </c>
+    </row>
+    <row r="540" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A540" s="3" t="s">
+        <v>1356</v>
+      </c>
+      <c r="B540" s="4" t="s">
+        <v>816</v>
+      </c>
+      <c r="C540" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D540" s="4" t="s">
+        <v>1357</v>
+      </c>
+      <c r="E540" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F540" s="2">
+        <v>46081.620833333334</v>
+      </c>
+    </row>
+    <row r="541" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A541" s="3" t="s">
+        <v>1358</v>
+      </c>
+      <c r="B541" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C541" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="D541" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E541" s="4" t="s">
+        <v>1359</v>
+      </c>
+      <c r="F541" s="2">
+        <v>46083.433333333334</v>
+      </c>
+    </row>
+    <row r="542" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A542" s="3" t="s">
+        <v>1360</v>
+      </c>
+      <c r="B542" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="C542" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D542" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E542" s="4" t="s">
+        <v>1361</v>
+      </c>
+      <c r="F542" s="2">
+        <v>46081.896527777775</v>
       </c>
     </row>
   </sheetData>
@@ -15763,6 +15921,13 @@
     <hyperlink ref="A533" r:id="rId532"/>
     <hyperlink ref="A534" r:id="rId533"/>
     <hyperlink ref="A535" r:id="rId534"/>
+    <hyperlink ref="A536" r:id="rId535"/>
+    <hyperlink ref="A537" r:id="rId536"/>
+    <hyperlink ref="A538" r:id="rId537"/>
+    <hyperlink ref="A539" r:id="rId538"/>
+    <hyperlink ref="A540" r:id="rId539"/>
+    <hyperlink ref="A541" r:id="rId540"/>
+    <hyperlink ref="A542" r:id="rId541"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -15774,7 +15939,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -15807,142 +15972,62 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1347</v>
+        <v>1362</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>497</v>
+        <v>25</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>74</v>
+        <v>435</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1348</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46081.87569444445</v>
+        <v>46084.19791666667</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1349</v>
+        <v>1363</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>437</v>
+        <v>536</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>74</v>
+        <v>28</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>154</v>
+        <v>1364</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1350</v>
+        <v>1365</v>
       </c>
       <c r="F3" s="2">
-        <v>46081.586805555555</v>
+        <v>46083.740277777775</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>1351</v>
+        <v>1366</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>31</v>
+        <v>112</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>518</v>
+        <v>63</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>1352</v>
+        <v>272</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>1353</v>
+        <v>1367</v>
       </c>
       <c r="F4" s="2">
-        <v>46080.80069444445</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1354</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>1163</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1355</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46081.884722222225</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>1356</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>816</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>1357</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46081.620833333334</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>1358</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>275</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>1359</v>
-      </c>
-      <c r="F7" s="2">
-        <v>46083.433333333334</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>1360</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>268</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>1361</v>
-      </c>
-      <c r="F8" s="2">
-        <v>46081.896527777775</v>
+        <v>46083.898611111115</v>
       </c>
     </row>
   </sheetData>
@@ -15950,10 +16035,6 @@
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
     <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A6" r:id="rId5"/>
-    <hyperlink ref="A7" r:id="rId6"/>
-    <hyperlink ref="A8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-03-04 12:29
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2732" uniqueCount="1368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2747" uniqueCount="1375">
   <si>
     <t>link</t>
   </si>
@@ -4122,6 +4122,27 @@
   </si>
   <si>
     <t>42620040875</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/alsviku-pag/eflef.html</t>
+  </si>
+  <si>
+    <t>36420060128</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/marsnenu-pag/jxcnd.html</t>
+  </si>
+  <si>
+    <t>42640020047</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/silmalas-pag/menog.html</t>
+  </si>
+  <si>
+    <t>4.87 ha.</t>
+  </si>
+  <si>
+    <t>78880120151</t>
   </si>
 </sst>
 </file>
@@ -4534,7 +4555,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F542"/>
+  <dimension ref="A1:F545"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -15383,6 +15404,66 @@
       </c>
       <c r="F542" s="2">
         <v>46081.896527777775</v>
+      </c>
+    </row>
+    <row r="543" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A543" s="3" t="s">
+        <v>1362</v>
+      </c>
+      <c r="B543" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C543" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D543" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E543" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F543" s="2">
+        <v>46084.19791666667</v>
+      </c>
+    </row>
+    <row r="544" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A544" s="3" t="s">
+        <v>1363</v>
+      </c>
+      <c r="B544" s="4" t="s">
+        <v>536</v>
+      </c>
+      <c r="C544" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D544" s="4" t="s">
+        <v>1364</v>
+      </c>
+      <c r="E544" s="4" t="s">
+        <v>1365</v>
+      </c>
+      <c r="F544" s="2">
+        <v>46083.740277777775</v>
+      </c>
+    </row>
+    <row r="545" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A545" s="3" t="s">
+        <v>1366</v>
+      </c>
+      <c r="B545" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C545" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D545" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E545" s="4" t="s">
+        <v>1367</v>
+      </c>
+      <c r="F545" s="2">
+        <v>46083.898611111115</v>
       </c>
     </row>
   </sheetData>
@@ -15928,6 +16009,9 @@
     <hyperlink ref="A540" r:id="rId539"/>
     <hyperlink ref="A541" r:id="rId540"/>
     <hyperlink ref="A542" r:id="rId541"/>
+    <hyperlink ref="A543" r:id="rId542"/>
+    <hyperlink ref="A544" r:id="rId543"/>
+    <hyperlink ref="A545" r:id="rId544"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -15972,62 +16056,62 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1362</v>
+        <v>1368</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>25</v>
+        <v>88</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>435</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>25</v>
+        <v>1369</v>
       </c>
       <c r="F2" s="2">
-        <v>46084.19791666667</v>
+        <v>46085.49861111111</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1363</v>
+        <v>1370</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>536</v>
+        <v>274</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>28</v>
+        <v>63</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>1364</v>
+        <v>162</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1365</v>
+        <v>1371</v>
       </c>
       <c r="F3" s="2">
-        <v>46083.740277777775</v>
+        <v>46085.48611111111</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>1366</v>
+        <v>1372</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>112</v>
+        <v>31</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>63</v>
+        <v>294</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>272</v>
+        <v>1373</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>1367</v>
+        <v>1374</v>
       </c>
       <c r="F4" s="2">
-        <v>46083.898611111115</v>
+        <v>46084.92361111111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-03-05 12:32
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -4555,7 +4555,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F545"/>
+  <dimension ref="A1:F548"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -15464,6 +15464,66 @@
       </c>
       <c r="F545" s="2">
         <v>46083.898611111115</v>
+      </c>
+    </row>
+    <row r="546" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A546" s="3" t="s">
+        <v>1368</v>
+      </c>
+      <c r="B546" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C546" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D546" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E546" s="4" t="s">
+        <v>1369</v>
+      </c>
+      <c r="F546" s="2">
+        <v>46085.49861111111</v>
+      </c>
+    </row>
+    <row r="547" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A547" s="3" t="s">
+        <v>1370</v>
+      </c>
+      <c r="B547" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="C547" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D547" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="E547" s="4" t="s">
+        <v>1371</v>
+      </c>
+      <c r="F547" s="2">
+        <v>46085.48611111111</v>
+      </c>
+    </row>
+    <row r="548" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A548" s="3" t="s">
+        <v>1372</v>
+      </c>
+      <c r="B548" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C548" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D548" s="4" t="s">
+        <v>1373</v>
+      </c>
+      <c r="E548" s="4" t="s">
+        <v>1374</v>
+      </c>
+      <c r="F548" s="2">
+        <v>46084.92361111111</v>
       </c>
     </row>
   </sheetData>
@@ -16012,6 +16072,9 @@
     <hyperlink ref="A543" r:id="rId542"/>
     <hyperlink ref="A544" r:id="rId543"/>
     <hyperlink ref="A545" r:id="rId544"/>
+    <hyperlink ref="A546" r:id="rId545"/>
+    <hyperlink ref="A547" r:id="rId546"/>
+    <hyperlink ref="A548" r:id="rId547"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -16023,7 +16086,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16054,72 +16117,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>1368</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>1369</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46085.49861111111</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1370</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>274</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1371</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46085.48611111111</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1372</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>1373</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1374</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46084.92361111111</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-03-06 12:28
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2747" uniqueCount="1375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2762" uniqueCount="1382">
   <si>
     <t>link</t>
   </si>
@@ -4143,6 +4143,27 @@
   </si>
   <si>
     <t>78880120151</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/salas-pag/honox.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/saldus-and-reg/zirnu-pag/jxpff.html</t>
+  </si>
+  <si>
+    <t>10.34 ha.</t>
+  </si>
+  <si>
+    <t>84960060342</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/saldus-and-reg/zirnu-pag/eojox.html</t>
+  </si>
+  <si>
+    <t>10.96 ha.</t>
+  </si>
+  <si>
+    <t>84960060340</t>
   </si>
 </sst>
 </file>
@@ -16086,7 +16107,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16117,7 +16138,72 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>1375</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46087.42361111111</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1376</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>1377</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1378</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46086.92708333333</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1379</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>1380</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1381</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46086.882638888885</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-03-09 12:32
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2762" uniqueCount="1382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2797" uniqueCount="1396">
   <si>
     <t>link</t>
   </si>
@@ -4164,6 +4164,48 @@
   </si>
   <si>
     <t>84960060340</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/annas-pag/odkip.html</t>
+  </si>
+  <si>
+    <t>36440040254</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/annas-pag/mdkol.html</t>
+  </si>
+  <si>
+    <t>36440020111</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/bauska-and-reg/iecavas-nov/akebh.html</t>
+  </si>
+  <si>
+    <t>40640060628</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/atasienes-pag/hklhl.html</t>
+  </si>
+  <si>
+    <t>56460120038</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/limbadzi-and-reg/braslavas-pag/ienfb.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valmiera-and-reg/mazsalaca/hmilg.html</t>
+  </si>
+  <si>
+    <t>96310030104</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ventspils-and-reg/targales-pag/dnpgh.html</t>
+  </si>
+  <si>
+    <t>7739 m²</t>
+  </si>
+  <si>
+    <t>98660020143</t>
   </si>
 </sst>
 </file>
@@ -4576,7 +4618,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F548"/>
+  <dimension ref="A1:F551"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -15545,6 +15587,66 @@
       </c>
       <c r="F548" s="2">
         <v>46084.92361111111</v>
+      </c>
+    </row>
+    <row r="549" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A549" s="3" t="s">
+        <v>1375</v>
+      </c>
+      <c r="B549" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="C549" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D549" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E549" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F549" s="2">
+        <v>46087.42361111111</v>
+      </c>
+    </row>
+    <row r="550" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A550" s="3" t="s">
+        <v>1376</v>
+      </c>
+      <c r="B550" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="C550" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="D550" s="4" t="s">
+        <v>1377</v>
+      </c>
+      <c r="E550" s="4" t="s">
+        <v>1378</v>
+      </c>
+      <c r="F550" s="2">
+        <v>46086.92708333333</v>
+      </c>
+    </row>
+    <row r="551" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A551" s="3" t="s">
+        <v>1379</v>
+      </c>
+      <c r="B551" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C551" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="D551" s="4" t="s">
+        <v>1380</v>
+      </c>
+      <c r="E551" s="4" t="s">
+        <v>1381</v>
+      </c>
+      <c r="F551" s="2">
+        <v>46086.882638888885</v>
       </c>
     </row>
   </sheetData>
@@ -16096,6 +16198,9 @@
     <hyperlink ref="A546" r:id="rId545"/>
     <hyperlink ref="A547" r:id="rId546"/>
     <hyperlink ref="A548" r:id="rId547"/>
+    <hyperlink ref="A549" r:id="rId548"/>
+    <hyperlink ref="A550" r:id="rId549"/>
+    <hyperlink ref="A551" r:id="rId550"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -16107,7 +16212,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16140,62 +16245,142 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1375</v>
+        <v>1382</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>274</v>
+        <v>497</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>127</v>
+        <v>435</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>186</v>
+        <v>1247</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>25</v>
+        <v>1383</v>
       </c>
       <c r="F2" s="2">
-        <v>46087.42361111111</v>
+        <v>46090.54375</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1376</v>
+        <v>1384</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>290</v>
+        <v>380</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>346</v>
+        <v>435</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>1377</v>
+        <v>154</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1378</v>
+        <v>1385</v>
       </c>
       <c r="F3" s="2">
-        <v>46086.92708333333</v>
+        <v>46090.53958333333</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>1379</v>
+        <v>1386</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>70</v>
+        <v>576</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>346</v>
+        <v>48</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>1380</v>
+        <v>272</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>1381</v>
+        <v>1387</v>
       </c>
       <c r="F4" s="2">
-        <v>46086.882638888885</v>
+        <v>46087.83333333333</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1388</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>355</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1389</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46090.56388888889</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>1390</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46088.74375</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>1391</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>1392</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46088.46527777778</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>1393</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>1394</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>1395</v>
+      </c>
+      <c r="F8" s="2">
+        <v>46089.53958333333</v>
       </c>
     </row>
   </sheetData>
@@ -16203,6 +16388,10 @@
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
     <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+    <hyperlink ref="A6" r:id="rId5"/>
+    <hyperlink ref="A7" r:id="rId6"/>
+    <hyperlink ref="A8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-03-10 12:32
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -4618,7 +4618,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F551"/>
+  <dimension ref="A1:F558"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -15647,6 +15647,146 @@
       </c>
       <c r="F551" s="2">
         <v>46086.882638888885</v>
+      </c>
+    </row>
+    <row r="552" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A552" s="3" t="s">
+        <v>1382</v>
+      </c>
+      <c r="B552" s="4" t="s">
+        <v>497</v>
+      </c>
+      <c r="C552" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D552" s="4" t="s">
+        <v>1247</v>
+      </c>
+      <c r="E552" s="4" t="s">
+        <v>1383</v>
+      </c>
+      <c r="F552" s="2">
+        <v>46090.54375</v>
+      </c>
+    </row>
+    <row r="553" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A553" s="3" t="s">
+        <v>1384</v>
+      </c>
+      <c r="B553" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="C553" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D553" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="E553" s="4" t="s">
+        <v>1385</v>
+      </c>
+      <c r="F553" s="2">
+        <v>46090.53958333333</v>
+      </c>
+    </row>
+    <row r="554" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A554" s="3" t="s">
+        <v>1386</v>
+      </c>
+      <c r="B554" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="C554" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D554" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E554" s="4" t="s">
+        <v>1387</v>
+      </c>
+      <c r="F554" s="2">
+        <v>46087.83333333333</v>
+      </c>
+    </row>
+    <row r="555" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A555" s="3" t="s">
+        <v>1388</v>
+      </c>
+      <c r="B555" s="4" t="s">
+        <v>355</v>
+      </c>
+      <c r="C555" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D555" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E555" s="4" t="s">
+        <v>1389</v>
+      </c>
+      <c r="F555" s="2">
+        <v>46090.56388888889</v>
+      </c>
+    </row>
+    <row r="556" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A556" s="3" t="s">
+        <v>1390</v>
+      </c>
+      <c r="B556" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C556" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D556" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E556" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F556" s="2">
+        <v>46088.74375</v>
+      </c>
+    </row>
+    <row r="557" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A557" s="3" t="s">
+        <v>1391</v>
+      </c>
+      <c r="B557" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="C557" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D557" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E557" s="4" t="s">
+        <v>1392</v>
+      </c>
+      <c r="F557" s="2">
+        <v>46088.46527777778</v>
+      </c>
+    </row>
+    <row r="558" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A558" s="3" t="s">
+        <v>1393</v>
+      </c>
+      <c r="B558" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C558" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D558" s="4" t="s">
+        <v>1394</v>
+      </c>
+      <c r="E558" s="4" t="s">
+        <v>1395</v>
+      </c>
+      <c r="F558" s="2">
+        <v>46089.53958333333</v>
       </c>
     </row>
   </sheetData>
@@ -16201,6 +16341,13 @@
     <hyperlink ref="A549" r:id="rId548"/>
     <hyperlink ref="A550" r:id="rId549"/>
     <hyperlink ref="A551" r:id="rId550"/>
+    <hyperlink ref="A552" r:id="rId551"/>
+    <hyperlink ref="A553" r:id="rId552"/>
+    <hyperlink ref="A554" r:id="rId553"/>
+    <hyperlink ref="A555" r:id="rId554"/>
+    <hyperlink ref="A556" r:id="rId555"/>
+    <hyperlink ref="A557" r:id="rId556"/>
+    <hyperlink ref="A558" r:id="rId557"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -16212,7 +16359,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16243,156 +16390,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>1382</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>497</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>1247</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>1383</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46090.54375</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1384</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>380</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1385</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46090.53958333333</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1386</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>576</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1387</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46087.83333333333</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1388</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>355</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1389</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46090.56388888889</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>1390</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46088.74375</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>1391</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>274</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>1392</v>
-      </c>
-      <c r="F7" s="2">
-        <v>46088.46527777778</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>1393</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>404</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>1394</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>1395</v>
-      </c>
-      <c r="F8" s="2">
-        <v>46089.53958333333</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A6" r:id="rId5"/>
-    <hyperlink ref="A7" r:id="rId6"/>
-    <hyperlink ref="A8" r:id="rId7"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-03-11 12:31
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2797" uniqueCount="1396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2827" uniqueCount="1411">
   <si>
     <t>link</t>
   </si>
@@ -4206,6 +4206,51 @@
   </si>
   <si>
     <t>98660020143</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/ziemera-pag/dmixh.html</t>
+  </si>
+  <si>
+    <t>47 €</t>
+  </si>
+  <si>
+    <t>1000 m²</t>
+  </si>
+  <si>
+    <t>36960020036</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/indras-pag/pgbbh.html</t>
+  </si>
+  <si>
+    <t>60620040936</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ludza-and-reg/blontu-pag/hldkl.html</t>
+  </si>
+  <si>
+    <t>46 €</t>
+  </si>
+  <si>
+    <t>68440050091</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/aizkalnes-pag/mibme.html</t>
+  </si>
+  <si>
+    <t>76440050023</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/silmalas-pag/llljp.html</t>
+  </si>
+  <si>
+    <t>78880050054</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/tukums-and-reg/kandava/eojec.html</t>
+  </si>
+  <si>
+    <t>90620060027</t>
   </si>
 </sst>
 </file>
@@ -16359,7 +16404,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16390,7 +16435,135 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>1396</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>1397</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>1398</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>1399</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46092.59930555556</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1400</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>843</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1401</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46092.54236111111</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1402</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>1403</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1404</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46092.54513888889</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1405</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1406</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46091.649305555555</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>1407</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>501</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>1343</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>1408</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46091.89166666666</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>1409</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>1410</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46091.62986111111</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+    <hyperlink ref="A6" r:id="rId5"/>
+    <hyperlink ref="A7" r:id="rId6"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-03-12 12:31
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2827" uniqueCount="1411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2832" uniqueCount="1412">
   <si>
     <t>link</t>
   </si>
@@ -4251,6 +4251,9 @@
   </si>
   <si>
     <t>90620060027</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/atasienes-pag/lkdxj.html</t>
   </si>
 </sst>
 </file>
@@ -4663,7 +4666,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F558"/>
+  <dimension ref="A1:F564"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -15832,6 +15835,126 @@
       </c>
       <c r="F558" s="2">
         <v>46089.53958333333</v>
+      </c>
+    </row>
+    <row r="559" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A559" s="3" t="s">
+        <v>1396</v>
+      </c>
+      <c r="B559" s="4" t="s">
+        <v>1397</v>
+      </c>
+      <c r="C559" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D559" s="4" t="s">
+        <v>1398</v>
+      </c>
+      <c r="E559" s="4" t="s">
+        <v>1399</v>
+      </c>
+      <c r="F559" s="2">
+        <v>46092.59930555556</v>
+      </c>
+    </row>
+    <row r="560" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A560" s="3" t="s">
+        <v>1400</v>
+      </c>
+      <c r="B560" s="4" t="s">
+        <v>843</v>
+      </c>
+      <c r="C560" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D560" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E560" s="4" t="s">
+        <v>1401</v>
+      </c>
+      <c r="F560" s="2">
+        <v>46092.54236111111</v>
+      </c>
+    </row>
+    <row r="561" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A561" s="3" t="s">
+        <v>1402</v>
+      </c>
+      <c r="B561" s="4" t="s">
+        <v>1403</v>
+      </c>
+      <c r="C561" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D561" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E561" s="4" t="s">
+        <v>1404</v>
+      </c>
+      <c r="F561" s="2">
+        <v>46092.54513888889</v>
+      </c>
+    </row>
+    <row r="562" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A562" s="3" t="s">
+        <v>1405</v>
+      </c>
+      <c r="B562" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="C562" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D562" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E562" s="4" t="s">
+        <v>1406</v>
+      </c>
+      <c r="F562" s="2">
+        <v>46091.649305555555</v>
+      </c>
+    </row>
+    <row r="563" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A563" s="3" t="s">
+        <v>1407</v>
+      </c>
+      <c r="B563" s="4" t="s">
+        <v>501</v>
+      </c>
+      <c r="C563" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D563" s="4" t="s">
+        <v>1343</v>
+      </c>
+      <c r="E563" s="4" t="s">
+        <v>1408</v>
+      </c>
+      <c r="F563" s="2">
+        <v>46091.89166666666</v>
+      </c>
+    </row>
+    <row r="564" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A564" s="3" t="s">
+        <v>1409</v>
+      </c>
+      <c r="B564" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C564" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D564" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="E564" s="4" t="s">
+        <v>1410</v>
+      </c>
+      <c r="F564" s="2">
+        <v>46091.62986111111</v>
       </c>
     </row>
   </sheetData>
@@ -16393,6 +16516,12 @@
     <hyperlink ref="A556" r:id="rId555"/>
     <hyperlink ref="A557" r:id="rId556"/>
     <hyperlink ref="A558" r:id="rId557"/>
+    <hyperlink ref="A559" r:id="rId558"/>
+    <hyperlink ref="A560" r:id="rId559"/>
+    <hyperlink ref="A561" r:id="rId560"/>
+    <hyperlink ref="A562" r:id="rId561"/>
+    <hyperlink ref="A563" r:id="rId562"/>
+    <hyperlink ref="A564" r:id="rId563"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -16404,7 +16533,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16437,132 +16566,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1396</v>
+        <v>1411</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1397</v>
+        <v>52</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>435</v>
+        <v>127</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>1398</v>
+        <v>186</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1399</v>
+        <v>1389</v>
       </c>
       <c r="F2" s="2">
-        <v>46092.59930555556</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1400</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>843</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1401</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46092.54236111111</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1402</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>1403</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1404</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46092.54513888889</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1405</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>467</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1406</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46091.649305555555</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>1407</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>501</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>1343</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>1408</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46091.89166666666</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>1409</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>376</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>1410</v>
-      </c>
-      <c r="F7" s="2">
-        <v>46091.62986111111</v>
+        <v>46092.75</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A6" r:id="rId5"/>
-    <hyperlink ref="A7" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-03-13 12:30
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -4666,7 +4666,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F564"/>
+  <dimension ref="A1:F565"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -15955,6 +15955,26 @@
       </c>
       <c r="F564" s="2">
         <v>46091.62986111111</v>
+      </c>
+    </row>
+    <row r="565" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A565" s="3" t="s">
+        <v>1411</v>
+      </c>
+      <c r="B565" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C565" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D565" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E565" s="4" t="s">
+        <v>1389</v>
+      </c>
+      <c r="F565" s="2">
+        <v>46092.75</v>
       </c>
     </row>
   </sheetData>
@@ -16522,6 +16542,7 @@
     <hyperlink ref="A562" r:id="rId561"/>
     <hyperlink ref="A563" r:id="rId562"/>
     <hyperlink ref="A564" r:id="rId563"/>
+    <hyperlink ref="A565" r:id="rId564"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -16533,7 +16554,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16564,30 +16585,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>1411</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>1389</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46092.75</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-03-16 12:41
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2832" uniqueCount="1412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2847" uniqueCount="1419">
   <si>
     <t>link</t>
   </si>
@@ -4254,6 +4254,27 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/atasienes-pag/lkdxj.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/demenes-pag/adhnp.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/kastulinas-pag/khxil.html</t>
+  </si>
+  <si>
+    <t>60720020081</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/feimanu-pag/pfijm.html</t>
+  </si>
+  <si>
+    <t>80 €</t>
+  </si>
+  <si>
+    <t>2.40 ha.</t>
+  </si>
+  <si>
+    <t>78520090172</t>
   </si>
 </sst>
 </file>
@@ -16554,7 +16575,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16585,7 +16606,72 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>1412</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>549</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>972</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46095.57638888889</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1413</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1414</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46094.79861111111</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1415</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>1416</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>1417</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1418</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46097.35277777778</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-03-17 12:40
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -4687,7 +4687,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F565"/>
+  <dimension ref="A1:F568"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -15996,6 +15996,66 @@
       </c>
       <c r="F565" s="2">
         <v>46092.75</v>
+      </c>
+    </row>
+    <row r="566" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A566" s="3" t="s">
+        <v>1412</v>
+      </c>
+      <c r="B566" s="4" t="s">
+        <v>549</v>
+      </c>
+      <c r="C566" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D566" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E566" s="4" t="s">
+        <v>972</v>
+      </c>
+      <c r="F566" s="2">
+        <v>46095.57638888889</v>
+      </c>
+    </row>
+    <row r="567" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A567" s="3" t="s">
+        <v>1413</v>
+      </c>
+      <c r="B567" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C567" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D567" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E567" s="4" t="s">
+        <v>1414</v>
+      </c>
+      <c r="F567" s="2">
+        <v>46094.79861111111</v>
+      </c>
+    </row>
+    <row r="568" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A568" s="3" t="s">
+        <v>1415</v>
+      </c>
+      <c r="B568" s="4" t="s">
+        <v>1416</v>
+      </c>
+      <c r="C568" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D568" s="4" t="s">
+        <v>1417</v>
+      </c>
+      <c r="E568" s="4" t="s">
+        <v>1418</v>
+      </c>
+      <c r="F568" s="2">
+        <v>46097.35277777778</v>
       </c>
     </row>
   </sheetData>
@@ -16564,6 +16624,9 @@
     <hyperlink ref="A563" r:id="rId562"/>
     <hyperlink ref="A564" r:id="rId563"/>
     <hyperlink ref="A565" r:id="rId564"/>
+    <hyperlink ref="A566" r:id="rId565"/>
+    <hyperlink ref="A567" r:id="rId566"/>
+    <hyperlink ref="A568" r:id="rId567"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -16575,7 +16638,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16606,72 +16669,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>1412</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>549</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>972</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46095.57638888889</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1413</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1414</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46094.79861111111</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1415</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>1416</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>1417</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1418</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46097.35277777778</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-03-19 12:34
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2847" uniqueCount="1419">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2852" uniqueCount="1420">
   <si>
     <t>link</t>
   </si>
@@ -4275,6 +4275,9 @@
   </si>
   <si>
     <t>78520090172</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/aluksne/kcxpe.html</t>
   </si>
 </sst>
 </file>
@@ -16638,7 +16641,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16669,7 +16672,30 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>1419</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>1241</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>831</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46100.32361111111</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-03-20 12:31
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2852" uniqueCount="1420">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2857" uniqueCount="1423">
   <si>
     <t>link</t>
   </si>
@@ -4278,6 +4278,15 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/aluksne/kcxpe.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/gulbene-and-reg/lejasciema-pag/jlndd.html</t>
+  </si>
+  <si>
+    <t>17.30 ha.</t>
+  </si>
+  <si>
+    <t>50640190230</t>
   </si>
 </sst>
 </file>
@@ -4690,7 +4699,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F568"/>
+  <dimension ref="A1:F569"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16059,6 +16068,26 @@
       </c>
       <c r="F568" s="2">
         <v>46097.35277777778</v>
+      </c>
+    </row>
+    <row r="569" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A569" s="3" t="s">
+        <v>1419</v>
+      </c>
+      <c r="B569" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C569" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D569" s="4" t="s">
+        <v>1241</v>
+      </c>
+      <c r="E569" s="4" t="s">
+        <v>831</v>
+      </c>
+      <c r="F569" s="2">
+        <v>46100.32361111111</v>
       </c>
     </row>
   </sheetData>
@@ -16630,6 +16659,7 @@
     <hyperlink ref="A566" r:id="rId565"/>
     <hyperlink ref="A567" r:id="rId566"/>
     <hyperlink ref="A568" r:id="rId567"/>
+    <hyperlink ref="A569" r:id="rId568"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -16674,22 +16704,22 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1419</v>
+        <v>1420</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>23</v>
+        <v>745</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>435</v>
+        <v>124</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>1241</v>
+        <v>1421</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>831</v>
+        <v>1422</v>
       </c>
       <c r="F2" s="2">
-        <v>46100.32361111111</v>
+        <v>46101.45625</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-03-23 12:37
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2857" uniqueCount="1423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2862" uniqueCount="1424">
   <si>
     <t>link</t>
   </si>
@@ -4287,6 +4287,9 @@
   </si>
   <si>
     <t>50640190230</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/praulienas-pag/cgbig.html</t>
   </si>
 </sst>
 </file>
@@ -4699,7 +4702,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F569"/>
+  <dimension ref="A1:F570"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16088,6 +16091,26 @@
       </c>
       <c r="F569" s="2">
         <v>46100.32361111111</v>
+      </c>
+    </row>
+    <row r="570" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A570" s="3" t="s">
+        <v>1420</v>
+      </c>
+      <c r="B570" s="4" t="s">
+        <v>745</v>
+      </c>
+      <c r="C570" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D570" s="4" t="s">
+        <v>1421</v>
+      </c>
+      <c r="E570" s="4" t="s">
+        <v>1422</v>
+      </c>
+      <c r="F570" s="2">
+        <v>46101.45625</v>
       </c>
     </row>
   </sheetData>
@@ -16660,6 +16683,7 @@
     <hyperlink ref="A567" r:id="rId566"/>
     <hyperlink ref="A568" r:id="rId567"/>
     <hyperlink ref="A569" r:id="rId568"/>
+    <hyperlink ref="A570" r:id="rId569"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -16704,22 +16728,22 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1420</v>
+        <v>1423</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>745</v>
+        <v>31</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>124</v>
+        <v>256</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>1421</v>
+        <v>911</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1422</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46101.45625</v>
+        <v>46104.41875</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-03-24 12:41
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2862" uniqueCount="1424">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2902" uniqueCount="1444">
   <si>
     <t>link</t>
   </si>
@@ -4290,6 +4290,66 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/praulienas-pag/cgbig.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aizkraukle-and-reg/klintaines-pag/chjng.html</t>
+  </si>
+  <si>
+    <t>32580080102</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/skilbenu-pag/bhhfnk.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/rugaju-pag/exfmg.html</t>
+  </si>
+  <si>
+    <t>3.84 ha.</t>
+  </si>
+  <si>
+    <t>38740120715</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/ziguru-pag/mifgk.html</t>
+  </si>
+  <si>
+    <t>38980030292</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ludza-and-reg/istras-pag/nbcnx.html</t>
+  </si>
+  <si>
+    <t>41 500 €</t>
+  </si>
+  <si>
+    <t>68600018023</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/preili/ghfoi.html</t>
+  </si>
+  <si>
+    <t>37 000 €</t>
+  </si>
+  <si>
+    <t>8.60 ha.</t>
+  </si>
+  <si>
+    <t>76420100182</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/preili/ggxom.html</t>
+  </si>
+  <si>
+    <t>20.70 ha.</t>
+  </si>
+  <si>
+    <t>76580040204</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/tukums-and-reg/irlavas-pag/cgkfnf.html</t>
+  </si>
+  <si>
+    <t>90540020060</t>
   </si>
 </sst>
 </file>
@@ -4702,7 +4762,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F570"/>
+  <dimension ref="A1:F571"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16111,6 +16171,26 @@
       </c>
       <c r="F570" s="2">
         <v>46101.45625</v>
+      </c>
+    </row>
+    <row r="571" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A571" s="3" t="s">
+        <v>1423</v>
+      </c>
+      <c r="B571" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C571" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D571" s="4" t="s">
+        <v>911</v>
+      </c>
+      <c r="E571" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F571" s="2">
+        <v>46104.41875</v>
       </c>
     </row>
   </sheetData>
@@ -16684,6 +16764,7 @@
     <hyperlink ref="A568" r:id="rId567"/>
     <hyperlink ref="A569" r:id="rId568"/>
     <hyperlink ref="A570" r:id="rId569"/>
+    <hyperlink ref="A571" r:id="rId570"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -16695,7 +16776,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16728,27 +16809,174 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1423</v>
+        <v>1424</v>
       </c>
       <c r="B2" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>659</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>1425</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46104.6125</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1426</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>911</v>
-      </c>
-      <c r="E2" s="4" t="s">
+      <c r="C3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="2">
-        <v>46104.41875</v>
+      <c r="F3" s="2">
+        <v>46105.584027777775</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1427</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>1428</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1429</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46104.92916666667</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1430</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1431</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46104.91805555555</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>1432</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>1433</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>1434</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46104.72361111111</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>1435</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>1436</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>1437</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>1438</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46105.566666666666</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>1439</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>1440</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>1441</v>
+      </c>
+      <c r="F8" s="2">
+        <v>46104.944444444445</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>1442</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>1443</v>
+      </c>
+      <c r="F9" s="2">
+        <v>46105.51388888889</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+    <hyperlink ref="A6" r:id="rId5"/>
+    <hyperlink ref="A7" r:id="rId6"/>
+    <hyperlink ref="A8" r:id="rId7"/>
+    <hyperlink ref="A9" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-03-25 12:38
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2902" uniqueCount="1444">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2932" uniqueCount="1457">
   <si>
     <t>link</t>
   </si>
@@ -4350,6 +4350,45 @@
   </si>
   <si>
     <t>90540020060</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aizkraukle-and-reg/valles-pag/cfdjp.html</t>
+  </si>
+  <si>
+    <t>32900110082</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/sventes-pag/mnhcg.html</t>
+  </si>
+  <si>
+    <t>44880060172</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/aizkalnes-pag/hcflo.html</t>
+  </si>
+  <si>
+    <t>76440030194</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/maltas-pag/lfgpd.html</t>
+  </si>
+  <si>
+    <t>78700060038</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/saldus-and-reg/zanas-pag/jniex.html</t>
+  </si>
+  <si>
+    <t>0.89 ha.</t>
+  </si>
+  <si>
+    <t>84940010052</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/talsi-and-reg/dundagas-pag/bxmfb.html</t>
+  </si>
+  <si>
+    <t>88500320025</t>
   </si>
 </sst>
 </file>
@@ -4762,7 +4801,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F571"/>
+  <dimension ref="A1:F579"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16191,6 +16230,166 @@
       </c>
       <c r="F571" s="2">
         <v>46104.41875</v>
+      </c>
+    </row>
+    <row r="572" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A572" s="3" t="s">
+        <v>1424</v>
+      </c>
+      <c r="B572" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C572" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D572" s="4" t="s">
+        <v>659</v>
+      </c>
+      <c r="E572" s="4" t="s">
+        <v>1425</v>
+      </c>
+      <c r="F572" s="2">
+        <v>46104.6125</v>
+      </c>
+    </row>
+    <row r="573" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A573" s="3" t="s">
+        <v>1426</v>
+      </c>
+      <c r="B573" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C573" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D573" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E573" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F573" s="2">
+        <v>46105.584027777775</v>
+      </c>
+    </row>
+    <row r="574" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A574" s="3" t="s">
+        <v>1427</v>
+      </c>
+      <c r="B574" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C574" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D574" s="4" t="s">
+        <v>1428</v>
+      </c>
+      <c r="E574" s="4" t="s">
+        <v>1429</v>
+      </c>
+      <c r="F574" s="2">
+        <v>46104.92916666667</v>
+      </c>
+    </row>
+    <row r="575" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A575" s="3" t="s">
+        <v>1430</v>
+      </c>
+      <c r="B575" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C575" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D575" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E575" s="4" t="s">
+        <v>1431</v>
+      </c>
+      <c r="F575" s="2">
+        <v>46104.91805555555</v>
+      </c>
+    </row>
+    <row r="576" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A576" s="3" t="s">
+        <v>1432</v>
+      </c>
+      <c r="B576" s="4" t="s">
+        <v>1433</v>
+      </c>
+      <c r="C576" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D576" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="E576" s="4" t="s">
+        <v>1434</v>
+      </c>
+      <c r="F576" s="2">
+        <v>46104.72361111111</v>
+      </c>
+    </row>
+    <row r="577" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A577" s="3" t="s">
+        <v>1435</v>
+      </c>
+      <c r="B577" s="4" t="s">
+        <v>1436</v>
+      </c>
+      <c r="C577" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D577" s="4" t="s">
+        <v>1437</v>
+      </c>
+      <c r="E577" s="4" t="s">
+        <v>1438</v>
+      </c>
+      <c r="F577" s="2">
+        <v>46105.566666666666</v>
+      </c>
+    </row>
+    <row r="578" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A578" s="3" t="s">
+        <v>1439</v>
+      </c>
+      <c r="B578" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="C578" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D578" s="4" t="s">
+        <v>1440</v>
+      </c>
+      <c r="E578" s="4" t="s">
+        <v>1441</v>
+      </c>
+      <c r="F578" s="2">
+        <v>46104.944444444445</v>
+      </c>
+    </row>
+    <row r="579" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A579" s="3" t="s">
+        <v>1442</v>
+      </c>
+      <c r="B579" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="C579" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D579" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E579" s="4" t="s">
+        <v>1443</v>
+      </c>
+      <c r="F579" s="2">
+        <v>46105.51388888889</v>
       </c>
     </row>
   </sheetData>
@@ -16765,6 +16964,14 @@
     <hyperlink ref="A569" r:id="rId568"/>
     <hyperlink ref="A570" r:id="rId569"/>
     <hyperlink ref="A571" r:id="rId570"/>
+    <hyperlink ref="A572" r:id="rId571"/>
+    <hyperlink ref="A573" r:id="rId572"/>
+    <hyperlink ref="A574" r:id="rId573"/>
+    <hyperlink ref="A575" r:id="rId574"/>
+    <hyperlink ref="A576" r:id="rId575"/>
+    <hyperlink ref="A577" r:id="rId576"/>
+    <hyperlink ref="A578" r:id="rId577"/>
+    <hyperlink ref="A579" r:id="rId578"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -16776,7 +16983,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16809,7 +17016,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1424</v>
+        <v>1444</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>43</v>
@@ -16818,153 +17025,113 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>659</v>
+        <v>36</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1425</v>
+        <v>1445</v>
       </c>
       <c r="F2" s="2">
-        <v>46104.6125</v>
+        <v>46106.58541666667</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1426</v>
+        <v>1446</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>31</v>
+        <v>116</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>28</v>
+        <v>74</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>186</v>
+        <v>82</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>25</v>
+        <v>1447</v>
       </c>
       <c r="F3" s="2">
-        <v>46105.584027777775</v>
+        <v>46106.575694444444</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>1427</v>
+        <v>1448</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>43</v>
+        <v>204</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>28</v>
+        <v>284</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>1428</v>
+        <v>85</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>1429</v>
+        <v>1449</v>
       </c>
       <c r="F4" s="2">
-        <v>46104.92916666667</v>
+        <v>46106.47916666667</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>1430</v>
+        <v>1450</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>204</v>
+        <v>927</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>28</v>
+        <v>294</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>59</v>
+        <v>82</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>1431</v>
+        <v>1451</v>
       </c>
       <c r="F5" s="2">
-        <v>46104.91805555555</v>
+        <v>46105.68125</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>1432</v>
+        <v>1452</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>1433</v>
+        <v>576</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>234</v>
+        <v>346</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>154</v>
+        <v>1453</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>1434</v>
+        <v>1454</v>
       </c>
       <c r="F6" s="2">
-        <v>46104.72361111111</v>
+        <v>46106.42152777778</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>1435</v>
+        <v>1455</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>1436</v>
+        <v>221</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>284</v>
+        <v>356</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>1437</v>
+        <v>186</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>1438</v>
+        <v>1456</v>
       </c>
       <c r="F7" s="2">
-        <v>46105.566666666666</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>1439</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>437</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>1440</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>1441</v>
-      </c>
-      <c r="F8" s="2">
-        <v>46104.944444444445</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>1442</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>376</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>1443</v>
-      </c>
-      <c r="F9" s="2">
-        <v>46105.51388888889</v>
+        <v>46105.61666666667</v>
       </c>
     </row>
   </sheetData>
@@ -16975,8 +17142,6 @@
     <hyperlink ref="A5" r:id="rId4"/>
     <hyperlink ref="A6" r:id="rId5"/>
     <hyperlink ref="A7" r:id="rId6"/>
-    <hyperlink ref="A8" r:id="rId7"/>
-    <hyperlink ref="A9" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-03-26 12:45
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2932" uniqueCount="1457">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2957" uniqueCount="1468">
   <si>
     <t>link</t>
   </si>
@@ -4389,6 +4389,39 @@
   </si>
   <si>
     <t>88500320025</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/alsviku-pag/ipehh.html</t>
+  </si>
+  <si>
+    <t>36420140324</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/pededzes-pag/flcix.html</t>
+  </si>
+  <si>
+    <t>98 000 €</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/gulbene-and-reg/ligo-pag/dnihd.html</t>
+  </si>
+  <si>
+    <t>5076003007</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ogre-and-reg/suntazu-pag/bkkmg.html</t>
+  </si>
+  <si>
+    <t>74880040011</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/pusas-pag/bbccd.html</t>
+  </si>
+  <si>
+    <t>5.50 ha.</t>
+  </si>
+  <si>
+    <t>78800030252</t>
   </si>
 </sst>
 </file>
@@ -4801,7 +4834,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F579"/>
+  <dimension ref="A1:F585"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16390,6 +16423,126 @@
       </c>
       <c r="F579" s="2">
         <v>46105.51388888889</v>
+      </c>
+    </row>
+    <row r="580" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A580" s="3" t="s">
+        <v>1444</v>
+      </c>
+      <c r="B580" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C580" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D580" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E580" s="4" t="s">
+        <v>1445</v>
+      </c>
+      <c r="F580" s="2">
+        <v>46106.58541666667</v>
+      </c>
+    </row>
+    <row r="581" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A581" s="3" t="s">
+        <v>1446</v>
+      </c>
+      <c r="B581" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C581" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D581" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E581" s="4" t="s">
+        <v>1447</v>
+      </c>
+      <c r="F581" s="2">
+        <v>46106.575694444444</v>
+      </c>
+    </row>
+    <row r="582" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A582" s="3" t="s">
+        <v>1448</v>
+      </c>
+      <c r="B582" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C582" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D582" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E582" s="4" t="s">
+        <v>1449</v>
+      </c>
+      <c r="F582" s="2">
+        <v>46106.47916666667</v>
+      </c>
+    </row>
+    <row r="583" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A583" s="3" t="s">
+        <v>1450</v>
+      </c>
+      <c r="B583" s="4" t="s">
+        <v>927</v>
+      </c>
+      <c r="C583" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D583" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E583" s="4" t="s">
+        <v>1451</v>
+      </c>
+      <c r="F583" s="2">
+        <v>46105.68125</v>
+      </c>
+    </row>
+    <row r="584" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A584" s="3" t="s">
+        <v>1452</v>
+      </c>
+      <c r="B584" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="C584" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="D584" s="4" t="s">
+        <v>1453</v>
+      </c>
+      <c r="E584" s="4" t="s">
+        <v>1454</v>
+      </c>
+      <c r="F584" s="2">
+        <v>46106.42152777778</v>
+      </c>
+    </row>
+    <row r="585" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A585" s="3" t="s">
+        <v>1455</v>
+      </c>
+      <c r="B585" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="C585" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="D585" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E585" s="4" t="s">
+        <v>1456</v>
+      </c>
+      <c r="F585" s="2">
+        <v>46105.61666666667</v>
       </c>
     </row>
   </sheetData>
@@ -16972,6 +17125,12 @@
     <hyperlink ref="A577" r:id="rId576"/>
     <hyperlink ref="A578" r:id="rId577"/>
     <hyperlink ref="A579" r:id="rId578"/>
+    <hyperlink ref="A580" r:id="rId579"/>
+    <hyperlink ref="A581" r:id="rId580"/>
+    <hyperlink ref="A582" r:id="rId581"/>
+    <hyperlink ref="A583" r:id="rId582"/>
+    <hyperlink ref="A584" r:id="rId583"/>
+    <hyperlink ref="A585" r:id="rId584"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -16983,7 +17142,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17016,122 +17175,102 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1444</v>
+        <v>1457</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>43</v>
+        <v>843</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>8</v>
+        <v>435</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>36</v>
+        <v>272</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1445</v>
+        <v>1458</v>
       </c>
       <c r="F2" s="2">
-        <v>46106.58541666667</v>
+        <v>46106.95277777778</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1446</v>
+        <v>1459</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>116</v>
+        <v>1460</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>74</v>
+        <v>435</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>82</v>
+        <v>209</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1447</v>
+        <v>25</v>
       </c>
       <c r="F3" s="2">
-        <v>46106.575694444444</v>
+        <v>46106.879166666666</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>1448</v>
+        <v>1461</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>204</v>
+        <v>102</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>284</v>
+        <v>124</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>85</v>
+        <v>13</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>1449</v>
+        <v>1462</v>
       </c>
       <c r="F4" s="2">
-        <v>46106.47916666667</v>
+        <v>46106.836111111115</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>1450</v>
+        <v>1463</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>927</v>
+        <v>217</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>294</v>
+        <v>275</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>82</v>
+        <v>209</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>1451</v>
+        <v>1464</v>
       </c>
       <c r="F5" s="2">
-        <v>46105.68125</v>
+        <v>46107.57847222222</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>1452</v>
+        <v>1465</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>576</v>
+        <v>31</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>346</v>
+        <v>294</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>1453</v>
+        <v>1466</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>1454</v>
+        <v>1467</v>
       </c>
       <c r="F6" s="2">
-        <v>46106.42152777778</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>1455</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>356</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>1456</v>
-      </c>
-      <c r="F7" s="2">
-        <v>46105.61666666667</v>
+        <v>46106.631944444445</v>
       </c>
     </row>
   </sheetData>
@@ -17141,7 +17280,6 @@
     <hyperlink ref="A4" r:id="rId3"/>
     <hyperlink ref="A5" r:id="rId4"/>
     <hyperlink ref="A6" r:id="rId5"/>
-    <hyperlink ref="A7" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-03-27 12:35
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2957" uniqueCount="1468">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2962" uniqueCount="1470">
   <si>
     <t>link</t>
   </si>
@@ -4422,6 +4422,12 @@
   </si>
   <si>
     <t>78800030252</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/vectilzas-pag/mknpd.html</t>
+  </si>
+  <si>
+    <t>38900040041</t>
   </si>
 </sst>
 </file>
@@ -4834,7 +4840,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F585"/>
+  <dimension ref="A1:F590"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16543,6 +16549,106 @@
       </c>
       <c r="F585" s="2">
         <v>46105.61666666667</v>
+      </c>
+    </row>
+    <row r="586" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A586" s="3" t="s">
+        <v>1457</v>
+      </c>
+      <c r="B586" s="4" t="s">
+        <v>843</v>
+      </c>
+      <c r="C586" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D586" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E586" s="4" t="s">
+        <v>1458</v>
+      </c>
+      <c r="F586" s="2">
+        <v>46106.95277777778</v>
+      </c>
+    </row>
+    <row r="587" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A587" s="3" t="s">
+        <v>1459</v>
+      </c>
+      <c r="B587" s="4" t="s">
+        <v>1460</v>
+      </c>
+      <c r="C587" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D587" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="E587" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F587" s="2">
+        <v>46106.879166666666</v>
+      </c>
+    </row>
+    <row r="588" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A588" s="3" t="s">
+        <v>1461</v>
+      </c>
+      <c r="B588" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C588" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D588" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E588" s="4" t="s">
+        <v>1462</v>
+      </c>
+      <c r="F588" s="2">
+        <v>46106.836111111115</v>
+      </c>
+    </row>
+    <row r="589" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A589" s="3" t="s">
+        <v>1463</v>
+      </c>
+      <c r="B589" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="C589" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="D589" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="E589" s="4" t="s">
+        <v>1464</v>
+      </c>
+      <c r="F589" s="2">
+        <v>46107.57847222222</v>
+      </c>
+    </row>
+    <row r="590" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A590" s="3" t="s">
+        <v>1465</v>
+      </c>
+      <c r="B590" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C590" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D590" s="4" t="s">
+        <v>1466</v>
+      </c>
+      <c r="E590" s="4" t="s">
+        <v>1467</v>
+      </c>
+      <c r="F590" s="2">
+        <v>46106.631944444445</v>
       </c>
     </row>
   </sheetData>
@@ -17131,6 +17237,11 @@
     <hyperlink ref="A583" r:id="rId582"/>
     <hyperlink ref="A584" r:id="rId583"/>
     <hyperlink ref="A585" r:id="rId584"/>
+    <hyperlink ref="A586" r:id="rId585"/>
+    <hyperlink ref="A587" r:id="rId586"/>
+    <hyperlink ref="A588" r:id="rId587"/>
+    <hyperlink ref="A589" r:id="rId588"/>
+    <hyperlink ref="A590" r:id="rId589"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -17142,7 +17253,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17175,111 +17286,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1457</v>
+        <v>1468</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>843</v>
+        <v>27</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>435</v>
+        <v>28</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>272</v>
+        <v>209</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1458</v>
+        <v>1469</v>
       </c>
       <c r="F2" s="2">
-        <v>46106.95277777778</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1459</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>1460</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46106.879166666666</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1461</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1462</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46106.836111111115</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1463</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>275</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1464</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46107.57847222222</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>1465</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>1466</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>1467</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46106.631944444445</v>
+        <v>46107.87847222222</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-03-30 12:46
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2962" uniqueCount="1470">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2992" uniqueCount="1483">
   <si>
     <t>link</t>
   </si>
@@ -4428,6 +4428,45 @@
   </si>
   <si>
     <t>38900040041</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/rugaju-pag/gegnf.html</t>
+  </si>
+  <si>
+    <t>3 700 €</t>
+  </si>
+  <si>
+    <t>38740120593</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/baltinavas-pag/lkdbn.html</t>
+  </si>
+  <si>
+    <t>38440050008</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kuldiga-and-reg/kuldiga/enibi.html</t>
+  </si>
+  <si>
+    <t>62540020077</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kuldiga-and-reg/kuldiga/cghlg.html</t>
+  </si>
+  <si>
+    <t>26720030094</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ventspils-and-reg/uzavas-pag/nodfh.html</t>
+  </si>
+  <si>
+    <t>98780040031</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ventspils-and-reg/varves-pag/bckje.html</t>
+  </si>
+  <si>
+    <t>98840110015</t>
   </si>
 </sst>
 </file>
@@ -4840,7 +4879,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F590"/>
+  <dimension ref="A1:F591"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16649,6 +16688,26 @@
       </c>
       <c r="F590" s="2">
         <v>46106.631944444445</v>
+      </c>
+    </row>
+    <row r="591" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A591" s="3" t="s">
+        <v>1468</v>
+      </c>
+      <c r="B591" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C591" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D591" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="E591" s="4" t="s">
+        <v>1469</v>
+      </c>
+      <c r="F591" s="2">
+        <v>46107.87847222222</v>
       </c>
     </row>
   </sheetData>
@@ -17242,6 +17301,7 @@
     <hyperlink ref="A588" r:id="rId587"/>
     <hyperlink ref="A589" r:id="rId588"/>
     <hyperlink ref="A590" r:id="rId589"/>
+    <hyperlink ref="A591" r:id="rId590"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -17253,7 +17313,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17286,27 +17346,132 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1468</v>
+        <v>1470</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>27</v>
+        <v>1471</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>28</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>209</v>
+        <v>82</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1469</v>
+        <v>1472</v>
       </c>
       <c r="F2" s="2">
-        <v>46107.87847222222</v>
+        <v>46111.43194444444</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1473</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1474</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46110.47777777778</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1475</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1476</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46111.649305555555</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1477</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1478</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46109.35833333334</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>1479</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>1480</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46109.361805555556</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>1481</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>1482</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46109.35416666667</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+    <hyperlink ref="A6" r:id="rId5"/>
+    <hyperlink ref="A7" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-03-31 12:45
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -4879,7 +4879,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F591"/>
+  <dimension ref="A1:F597"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16708,6 +16708,126 @@
       </c>
       <c r="F591" s="2">
         <v>46107.87847222222</v>
+      </c>
+    </row>
+    <row r="592" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A592" s="3" t="s">
+        <v>1470</v>
+      </c>
+      <c r="B592" s="4" t="s">
+        <v>1471</v>
+      </c>
+      <c r="C592" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D592" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E592" s="4" t="s">
+        <v>1472</v>
+      </c>
+      <c r="F592" s="2">
+        <v>46111.43194444444</v>
+      </c>
+    </row>
+    <row r="593" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A593" s="3" t="s">
+        <v>1473</v>
+      </c>
+      <c r="B593" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C593" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D593" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E593" s="4" t="s">
+        <v>1474</v>
+      </c>
+      <c r="F593" s="2">
+        <v>46110.47777777778</v>
+      </c>
+    </row>
+    <row r="594" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A594" s="3" t="s">
+        <v>1475</v>
+      </c>
+      <c r="B594" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C594" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="D594" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E594" s="4" t="s">
+        <v>1476</v>
+      </c>
+      <c r="F594" s="2">
+        <v>46111.649305555555</v>
+      </c>
+    </row>
+    <row r="595" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A595" s="3" t="s">
+        <v>1477</v>
+      </c>
+      <c r="B595" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C595" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="D595" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E595" s="4" t="s">
+        <v>1478</v>
+      </c>
+      <c r="F595" s="2">
+        <v>46109.35833333334</v>
+      </c>
+    </row>
+    <row r="596" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A596" s="3" t="s">
+        <v>1479</v>
+      </c>
+      <c r="B596" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C596" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D596" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E596" s="4" t="s">
+        <v>1480</v>
+      </c>
+      <c r="F596" s="2">
+        <v>46109.361805555556</v>
+      </c>
+    </row>
+    <row r="597" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A597" s="3" t="s">
+        <v>1481</v>
+      </c>
+      <c r="B597" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C597" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D597" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E597" s="4" t="s">
+        <v>1482</v>
+      </c>
+      <c r="F597" s="2">
+        <v>46109.35416666667</v>
       </c>
     </row>
   </sheetData>
@@ -17302,6 +17422,12 @@
     <hyperlink ref="A589" r:id="rId588"/>
     <hyperlink ref="A590" r:id="rId589"/>
     <hyperlink ref="A591" r:id="rId590"/>
+    <hyperlink ref="A592" r:id="rId591"/>
+    <hyperlink ref="A593" r:id="rId592"/>
+    <hyperlink ref="A594" r:id="rId593"/>
+    <hyperlink ref="A595" r:id="rId594"/>
+    <hyperlink ref="A596" r:id="rId595"/>
+    <hyperlink ref="A597" r:id="rId596"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -17313,7 +17439,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17344,135 +17470,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>1470</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>1471</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>1472</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46111.43194444444</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1473</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1474</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46110.47777777778</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1475</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>424</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1476</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46111.649305555555</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1477</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>424</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1478</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46109.35833333334</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>1479</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>404</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>1480</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46109.361805555556</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>1481</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>404</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>1482</v>
-      </c>
-      <c r="F7" s="2">
-        <v>46109.35416666667</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A6" r:id="rId5"/>
-    <hyperlink ref="A7" r:id="rId6"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-04-01 12:48
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2992" uniqueCount="1483">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3002" uniqueCount="1486">
   <si>
     <t>link</t>
   </si>
@@ -4467,6 +4467,15 @@
   </si>
   <si>
     <t>98840110015</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/indras-pag/lfnpc.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/talsi-and-reg/vandzenes-pag/ookni.html</t>
+  </si>
+  <si>
+    <t>88940080323</t>
   </si>
 </sst>
 </file>
@@ -17439,7 +17448,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17470,7 +17479,51 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>1483</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>1401</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46113.47708333333</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1484</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1485</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46113.375</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-04-02 12:42
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3002" uniqueCount="1486">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3017" uniqueCount="1495">
   <si>
     <t>link</t>
   </si>
@@ -4476,6 +4476,33 @@
   </si>
   <si>
     <t>88940080323</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/bauska-and-reg/vecumnieku-pag/bghld.html</t>
+  </si>
+  <si>
+    <t>20 001 €</t>
+  </si>
+  <si>
+    <t>40940121263</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/atasienes-pag/hkldk.html</t>
+  </si>
+  <si>
+    <t>18 001 €</t>
+  </si>
+  <si>
+    <t>56760020017</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ludza-and-reg/rundenu-pag/mnmci.html</t>
+  </si>
+  <si>
+    <t>30 001 €</t>
+  </si>
+  <si>
+    <t>68920060100</t>
   </si>
 </sst>
 </file>
@@ -4888,7 +4915,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F597"/>
+  <dimension ref="A1:F599"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16837,6 +16864,46 @@
       </c>
       <c r="F597" s="2">
         <v>46109.35416666667</v>
+      </c>
+    </row>
+    <row r="598" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A598" s="3" t="s">
+        <v>1483</v>
+      </c>
+      <c r="B598" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C598" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D598" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E598" s="4" t="s">
+        <v>1401</v>
+      </c>
+      <c r="F598" s="2">
+        <v>46113.47708333333</v>
+      </c>
+    </row>
+    <row r="599" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A599" s="3" t="s">
+        <v>1484</v>
+      </c>
+      <c r="B599" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C599" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="D599" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E599" s="4" t="s">
+        <v>1485</v>
+      </c>
+      <c r="F599" s="2">
+        <v>46113.375</v>
       </c>
     </row>
   </sheetData>
@@ -17437,6 +17504,8 @@
     <hyperlink ref="A595" r:id="rId594"/>
     <hyperlink ref="A596" r:id="rId595"/>
     <hyperlink ref="A597" r:id="rId596"/>
+    <hyperlink ref="A598" r:id="rId597"/>
+    <hyperlink ref="A599" r:id="rId598"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -17448,7 +17517,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17481,48 +17550,69 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1483</v>
+        <v>1486</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>47</v>
+        <v>1487</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>146</v>
+        <v>48</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>85</v>
+        <v>186</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1401</v>
+        <v>1488</v>
       </c>
       <c r="F2" s="2">
-        <v>46113.47708333333</v>
+        <v>46113.91458333333</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1484</v>
+        <v>1489</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>43</v>
+        <v>1490</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>356</v>
+        <v>127</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>36</v>
+        <v>85</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1485</v>
+        <v>1491</v>
       </c>
       <c r="F3" s="2">
-        <v>46113.375</v>
+        <v>46113.92291666666</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1492</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>1493</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1494</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46113.93611111111</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-04-03 12:35
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3017" uniqueCount="1495">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3027" uniqueCount="1500">
   <si>
     <t>link</t>
   </si>
@@ -4503,6 +4503,21 @@
   </si>
   <si>
     <t>68920060100</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/liepas-pag/ephdg.html</t>
+  </si>
+  <si>
+    <t>18.54 ha.</t>
+  </si>
+  <si>
+    <t>42600050083</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/vecsalienas-pag/mcnie.html</t>
+  </si>
+  <si>
+    <t>44960050019</t>
   </si>
 </sst>
 </file>
@@ -4915,7 +4930,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F599"/>
+  <dimension ref="A1:F602"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16904,6 +16919,66 @@
       </c>
       <c r="F599" s="2">
         <v>46113.375</v>
+      </c>
+    </row>
+    <row r="600" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A600" s="3" t="s">
+        <v>1486</v>
+      </c>
+      <c r="B600" s="4" t="s">
+        <v>1487</v>
+      </c>
+      <c r="C600" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D600" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E600" s="4" t="s">
+        <v>1488</v>
+      </c>
+      <c r="F600" s="2">
+        <v>46113.91458333333</v>
+      </c>
+    </row>
+    <row r="601" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A601" s="3" t="s">
+        <v>1489</v>
+      </c>
+      <c r="B601" s="4" t="s">
+        <v>1490</v>
+      </c>
+      <c r="C601" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D601" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E601" s="4" t="s">
+        <v>1491</v>
+      </c>
+      <c r="F601" s="2">
+        <v>46113.92291666666</v>
+      </c>
+    </row>
+    <row r="602" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A602" s="3" t="s">
+        <v>1492</v>
+      </c>
+      <c r="B602" s="4" t="s">
+        <v>1493</v>
+      </c>
+      <c r="C602" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D602" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="E602" s="4" t="s">
+        <v>1494</v>
+      </c>
+      <c r="F602" s="2">
+        <v>46113.93611111111</v>
       </c>
     </row>
   </sheetData>
@@ -17506,6 +17581,9 @@
     <hyperlink ref="A597" r:id="rId596"/>
     <hyperlink ref="A598" r:id="rId597"/>
     <hyperlink ref="A599" r:id="rId598"/>
+    <hyperlink ref="A600" r:id="rId599"/>
+    <hyperlink ref="A601" r:id="rId600"/>
+    <hyperlink ref="A602" r:id="rId601"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -17517,7 +17595,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17550,69 +17628,48 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1486</v>
+        <v>1495</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1487</v>
+        <v>781</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>186</v>
+        <v>1496</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1488</v>
+        <v>1497</v>
       </c>
       <c r="F2" s="2">
-        <v>46113.91458333333</v>
+        <v>46115.57361111111</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1489</v>
+        <v>1498</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>1490</v>
+        <v>88</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>127</v>
+        <v>74</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>85</v>
+        <v>13</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1491</v>
+        <v>1499</v>
       </c>
       <c r="F3" s="2">
-        <v>46113.92291666666</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1492</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>1493</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1494</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46113.93611111111</v>
+        <v>46114.67361111111</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-04-06 12:41
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3027" uniqueCount="1500">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3037" uniqueCount="1507">
   <si>
     <t>link</t>
   </si>
@@ -4518,6 +4518,27 @@
   </si>
   <si>
     <t>44960050019</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aizkraukle-and-reg/mazzalves-pag/jfbek.html</t>
+  </si>
+  <si>
+    <t>9 700 €</t>
+  </si>
+  <si>
+    <t>32660050001</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ogre-and-reg/birzgales-pag/fbjfe.html</t>
+  </si>
+  <si>
+    <t>29 999 €</t>
+  </si>
+  <si>
+    <t>3.20 ha.</t>
+  </si>
+  <si>
+    <t>74440020097</t>
   </si>
 </sst>
 </file>
@@ -4930,7 +4951,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F602"/>
+  <dimension ref="A1:F604"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -16979,6 +17000,46 @@
       </c>
       <c r="F602" s="2">
         <v>46113.93611111111</v>
+      </c>
+    </row>
+    <row r="603" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A603" s="3" t="s">
+        <v>1495</v>
+      </c>
+      <c r="B603" s="4" t="s">
+        <v>781</v>
+      </c>
+      <c r="C603" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D603" s="4" t="s">
+        <v>1496</v>
+      </c>
+      <c r="E603" s="4" t="s">
+        <v>1497</v>
+      </c>
+      <c r="F603" s="2">
+        <v>46115.57361111111</v>
+      </c>
+    </row>
+    <row r="604" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A604" s="3" t="s">
+        <v>1498</v>
+      </c>
+      <c r="B604" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C604" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D604" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E604" s="4" t="s">
+        <v>1499</v>
+      </c>
+      <c r="F604" s="2">
+        <v>46114.67361111111</v>
       </c>
     </row>
   </sheetData>
@@ -17584,6 +17645,8 @@
     <hyperlink ref="A600" r:id="rId599"/>
     <hyperlink ref="A601" r:id="rId600"/>
     <hyperlink ref="A602" r:id="rId601"/>
+    <hyperlink ref="A603" r:id="rId602"/>
+    <hyperlink ref="A604" r:id="rId603"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -17628,42 +17691,42 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1495</v>
+        <v>1500</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>781</v>
+        <v>1501</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>63</v>
+        <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>1496</v>
+        <v>186</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1497</v>
+        <v>1502</v>
       </c>
       <c r="F2" s="2">
-        <v>46115.57361111111</v>
+        <v>46116.6375</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1498</v>
+        <v>1503</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>88</v>
+        <v>1504</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>74</v>
+        <v>275</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>13</v>
+        <v>1505</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1499</v>
+        <v>1506</v>
       </c>
       <c r="F3" s="2">
-        <v>46114.67361111111</v>
+        <v>46117.00625</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-04-07 12:52
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3037" uniqueCount="1507">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3047" uniqueCount="1511">
   <si>
     <t>link</t>
   </si>
@@ -4539,6 +4539,18 @@
   </si>
   <si>
     <t>74440020097</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/salienas-pag/bccgjg.html</t>
+  </si>
+  <si>
+    <t>10 200 €</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/saldus-and-reg/gaiku-pag/dbodi.html</t>
+  </si>
+  <si>
+    <t>84520010104</t>
   </si>
 </sst>
 </file>
@@ -4951,7 +4963,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F604"/>
+  <dimension ref="A1:F606"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17040,6 +17052,46 @@
       </c>
       <c r="F604" s="2">
         <v>46114.67361111111</v>
+      </c>
+    </row>
+    <row r="605" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A605" s="3" t="s">
+        <v>1500</v>
+      </c>
+      <c r="B605" s="4" t="s">
+        <v>1501</v>
+      </c>
+      <c r="C605" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D605" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E605" s="4" t="s">
+        <v>1502</v>
+      </c>
+      <c r="F605" s="2">
+        <v>46116.6375</v>
+      </c>
+    </row>
+    <row r="606" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A606" s="3" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B606" s="4" t="s">
+        <v>1504</v>
+      </c>
+      <c r="C606" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="D606" s="4" t="s">
+        <v>1505</v>
+      </c>
+      <c r="E606" s="4" t="s">
+        <v>1506</v>
+      </c>
+      <c r="F606" s="2">
+        <v>46117.00625</v>
       </c>
     </row>
   </sheetData>
@@ -17647,6 +17699,8 @@
     <hyperlink ref="A602" r:id="rId601"/>
     <hyperlink ref="A603" r:id="rId602"/>
     <hyperlink ref="A604" r:id="rId603"/>
+    <hyperlink ref="A605" r:id="rId604"/>
+    <hyperlink ref="A606" r:id="rId605"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -17691,42 +17745,42 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1500</v>
+        <v>1507</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1501</v>
+        <v>1508</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>8</v>
+        <v>74</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>186</v>
+        <v>272</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1502</v>
+        <v>1131</v>
       </c>
       <c r="F2" s="2">
-        <v>46116.6375</v>
+        <v>46118.65694444445</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1503</v>
+        <v>1509</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>1504</v>
+        <v>217</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>275</v>
+        <v>346</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>1505</v>
+        <v>903</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1506</v>
+        <v>1510</v>
       </c>
       <c r="F3" s="2">
-        <v>46117.00625</v>
+        <v>46119.5875</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-04-08 12:51
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3047" uniqueCount="1511">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3057" uniqueCount="1517">
   <si>
     <t>link</t>
   </si>
@@ -4551,6 +4551,24 @@
   </si>
   <si>
     <t>84520010104</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/cesis/ddmdi.html</t>
+  </si>
+  <si>
+    <t>2686 m²</t>
+  </si>
+  <si>
+    <t>42720060303</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/indras-pag/mepic.html</t>
+  </si>
+  <si>
+    <t>23 100 €</t>
+  </si>
+  <si>
+    <t>60620050145</t>
   </si>
 </sst>
 </file>
@@ -4963,7 +4981,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F606"/>
+  <dimension ref="A1:F608"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17092,6 +17110,46 @@
       </c>
       <c r="F606" s="2">
         <v>46117.00625</v>
+      </c>
+    </row>
+    <row r="607" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A607" s="3" t="s">
+        <v>1507</v>
+      </c>
+      <c r="B607" s="4" t="s">
+        <v>1508</v>
+      </c>
+      <c r="C607" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D607" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E607" s="4" t="s">
+        <v>1131</v>
+      </c>
+      <c r="F607" s="2">
+        <v>46118.65694444445</v>
+      </c>
+    </row>
+    <row r="608" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A608" s="3" t="s">
+        <v>1509</v>
+      </c>
+      <c r="B608" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="C608" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="D608" s="4" t="s">
+        <v>903</v>
+      </c>
+      <c r="E608" s="4" t="s">
+        <v>1510</v>
+      </c>
+      <c r="F608" s="2">
+        <v>46119.5875</v>
       </c>
     </row>
   </sheetData>
@@ -17701,6 +17759,8 @@
     <hyperlink ref="A604" r:id="rId603"/>
     <hyperlink ref="A605" r:id="rId604"/>
     <hyperlink ref="A606" r:id="rId605"/>
+    <hyperlink ref="A607" r:id="rId606"/>
+    <hyperlink ref="A608" r:id="rId607"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -17745,42 +17805,42 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1507</v>
+        <v>1511</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1508</v>
+        <v>204</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>272</v>
+        <v>1512</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1131</v>
+        <v>1513</v>
       </c>
       <c r="F2" s="2">
-        <v>46118.65694444445</v>
+        <v>46120.54236111111</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1509</v>
+        <v>1514</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>217</v>
+        <v>1515</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>346</v>
+        <v>146</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>903</v>
+        <v>13</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1510</v>
+        <v>1516</v>
       </c>
       <c r="F3" s="2">
-        <v>46119.5875</v>
+        <v>46120.51944444445</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-04-09 12:54
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3057" uniqueCount="1517">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3062" uniqueCount="1519">
   <si>
     <t>link</t>
   </si>
@@ -4569,6 +4569,12 @@
   </si>
   <si>
     <t>60620050145</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/sausnejas-pag/hjhbp.html</t>
+  </si>
+  <si>
+    <t>69 300 €</t>
   </si>
 </sst>
 </file>
@@ -4981,7 +4987,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F608"/>
+  <dimension ref="A1:F610"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17150,6 +17156,46 @@
       </c>
       <c r="F608" s="2">
         <v>46119.5875</v>
+      </c>
+    </row>
+    <row r="609" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A609" s="3" t="s">
+        <v>1511</v>
+      </c>
+      <c r="B609" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C609" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D609" s="4" t="s">
+        <v>1512</v>
+      </c>
+      <c r="E609" s="4" t="s">
+        <v>1513</v>
+      </c>
+      <c r="F609" s="2">
+        <v>46120.54236111111</v>
+      </c>
+    </row>
+    <row r="610" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A610" s="3" t="s">
+        <v>1514</v>
+      </c>
+      <c r="B610" s="4" t="s">
+        <v>1515</v>
+      </c>
+      <c r="C610" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D610" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E610" s="4" t="s">
+        <v>1516</v>
+      </c>
+      <c r="F610" s="2">
+        <v>46120.51944444445</v>
       </c>
     </row>
   </sheetData>
@@ -17761,6 +17807,8 @@
     <hyperlink ref="A606" r:id="rId605"/>
     <hyperlink ref="A607" r:id="rId606"/>
     <hyperlink ref="A608" r:id="rId607"/>
+    <hyperlink ref="A609" r:id="rId608"/>
+    <hyperlink ref="A610" r:id="rId609"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -17772,7 +17820,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17805,48 +17853,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1511</v>
+        <v>1517</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>204</v>
+        <v>1518</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>63</v>
+        <v>256</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>1512</v>
+        <v>103</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1513</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46120.54236111111</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1514</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>1515</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1516</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46120.51944444445</v>
+        <v>46120.709027777775</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-04-10 12:41
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3062" uniqueCount="1519">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3067" uniqueCount="1522">
   <si>
     <t>link</t>
   </si>
@@ -4575,6 +4575,15 @@
   </si>
   <si>
     <t>69 300 €</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/tabores-pag/ndmbn.html</t>
+  </si>
+  <si>
+    <t>0.94 ha.</t>
+  </si>
+  <si>
+    <t>44920030592</t>
   </si>
 </sst>
 </file>
@@ -4987,7 +4996,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F610"/>
+  <dimension ref="A1:F611"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17196,6 +17205,26 @@
       </c>
       <c r="F610" s="2">
         <v>46120.51944444445</v>
+      </c>
+    </row>
+    <row r="611" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A611" s="3" t="s">
+        <v>1517</v>
+      </c>
+      <c r="B611" s="4" t="s">
+        <v>1518</v>
+      </c>
+      <c r="C611" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D611" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E611" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F611" s="2">
+        <v>46120.709027777775</v>
       </c>
     </row>
   </sheetData>
@@ -17809,6 +17838,7 @@
     <hyperlink ref="A608" r:id="rId607"/>
     <hyperlink ref="A609" r:id="rId608"/>
     <hyperlink ref="A610" r:id="rId609"/>
+    <hyperlink ref="A611" r:id="rId610"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -17853,22 +17883,22 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1517</v>
+        <v>1519</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1518</v>
+        <v>1115</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>256</v>
+        <v>74</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>103</v>
+        <v>1520</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>25</v>
+        <v>1521</v>
       </c>
       <c r="F2" s="2">
-        <v>46120.709027777775</v>
+        <v>46121.669444444444</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-04-13 12:56
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3067" uniqueCount="1522">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3087" uniqueCount="1529">
   <si>
     <t>link</t>
   </si>
@@ -4584,6 +4584,27 @@
   </si>
   <si>
     <t>44920030592</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/lazdulejas-pag/cbpih.html</t>
+  </si>
+  <si>
+    <t>38660040339</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/varaklanu-pag/diejf.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/aglonas-pag/cdokm.html</t>
+  </si>
+  <si>
+    <t>7642-004-0221</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/saldus-and-reg/blidenes-pag/mmdcc.html</t>
+  </si>
+  <si>
+    <t>8444 004 0011</t>
   </si>
 </sst>
 </file>
@@ -4996,7 +5017,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F611"/>
+  <dimension ref="A1:F612"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17225,6 +17246,26 @@
       </c>
       <c r="F611" s="2">
         <v>46120.709027777775</v>
+      </c>
+    </row>
+    <row r="612" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A612" s="3" t="s">
+        <v>1519</v>
+      </c>
+      <c r="B612" s="4" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C612" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D612" s="4" t="s">
+        <v>1520</v>
+      </c>
+      <c r="E612" s="4" t="s">
+        <v>1521</v>
+      </c>
+      <c r="F612" s="2">
+        <v>46121.669444444444</v>
       </c>
     </row>
   </sheetData>
@@ -17839,6 +17880,7 @@
     <hyperlink ref="A609" r:id="rId608"/>
     <hyperlink ref="A610" r:id="rId609"/>
     <hyperlink ref="A611" r:id="rId610"/>
+    <hyperlink ref="A612" r:id="rId611"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -17850,7 +17892,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17883,27 +17925,90 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1519</v>
+        <v>1522</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1115</v>
+        <v>131</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>74</v>
+        <v>28</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>1520</v>
+        <v>36</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1521</v>
+        <v>1523</v>
       </c>
       <c r="F2" s="2">
-        <v>46121.669444444444</v>
+        <v>46123.46041666667</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1524</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46124.75555555556</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1525</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>816</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1526</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46122.72986111111</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1527</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1528</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46125.59583333333</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-04-14 12:55
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -5017,7 +5017,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F612"/>
+  <dimension ref="A1:F616"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17266,6 +17266,86 @@
       </c>
       <c r="F612" s="2">
         <v>46121.669444444444</v>
+      </c>
+    </row>
+    <row r="613" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A613" s="3" t="s">
+        <v>1522</v>
+      </c>
+      <c r="B613" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C613" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D613" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E613" s="4" t="s">
+        <v>1523</v>
+      </c>
+      <c r="F613" s="2">
+        <v>46123.46041666667</v>
+      </c>
+    </row>
+    <row r="614" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A614" s="3" t="s">
+        <v>1524</v>
+      </c>
+      <c r="B614" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C614" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D614" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E614" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F614" s="2">
+        <v>46124.75555555556</v>
+      </c>
+    </row>
+    <row r="615" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A615" s="3" t="s">
+        <v>1525</v>
+      </c>
+      <c r="B615" s="4" t="s">
+        <v>816</v>
+      </c>
+      <c r="C615" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D615" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E615" s="4" t="s">
+        <v>1526</v>
+      </c>
+      <c r="F615" s="2">
+        <v>46122.72986111111</v>
+      </c>
+    </row>
+    <row r="616" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A616" s="3" t="s">
+        <v>1527</v>
+      </c>
+      <c r="B616" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C616" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="D616" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E616" s="4" t="s">
+        <v>1528</v>
+      </c>
+      <c r="F616" s="2">
+        <v>46125.59583333333</v>
       </c>
     </row>
   </sheetData>
@@ -17881,6 +17961,10 @@
     <hyperlink ref="A610" r:id="rId609"/>
     <hyperlink ref="A611" r:id="rId610"/>
     <hyperlink ref="A612" r:id="rId611"/>
+    <hyperlink ref="A613" r:id="rId612"/>
+    <hyperlink ref="A614" r:id="rId613"/>
+    <hyperlink ref="A615" r:id="rId614"/>
+    <hyperlink ref="A616" r:id="rId615"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -17892,7 +17976,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17923,93 +18007,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>1522</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>1523</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46123.46041666667</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1524</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46124.75555555556</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1525</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>816</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1526</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46122.72986111111</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1527</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>346</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1528</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46125.59583333333</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-04-17 12:51
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3087" uniqueCount="1529">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3102" uniqueCount="1536">
   <si>
     <t>link</t>
   </si>
@@ -4605,6 +4605,27 @@
   </si>
   <si>
     <t>8444 004 0011</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/bauska-and-reg/vecumnieku-pag/kgnoj.html</t>
+  </si>
+  <si>
+    <t>40940180037</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/andrupenes-pag/jnegx.html</t>
+  </si>
+  <si>
+    <t>6042-007-0218</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/limbadzi-and-reg/liepupes-pag/ckdfc.html</t>
+  </si>
+  <si>
+    <t>145 800 €</t>
+  </si>
+  <si>
+    <t>66600130224</t>
   </si>
 </sst>
 </file>
@@ -17976,7 +17997,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18007,7 +18028,72 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>1529</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>1530</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46129.4625</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1531</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>1417</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1532</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46128.825</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1533</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>1534</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1535</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46129.44861111111</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-04-20 13:00
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3102" uniqueCount="1536">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3117" uniqueCount="1543">
   <si>
     <t>link</t>
   </si>
@@ -4626,6 +4626,27 @@
   </si>
   <si>
     <t>66600130224</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/liepaja-and-reg/vergales-pag/kopil.html</t>
+  </si>
+  <si>
+    <t>150 000 €</t>
+  </si>
+  <si>
+    <t>64960010063</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/limbadzi-and-reg/alojas-l-t/kxfgb.html</t>
+  </si>
+  <si>
+    <t>66270030084</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/madona/kpdng.html</t>
+  </si>
+  <si>
+    <t>70860080049</t>
   </si>
 </sst>
 </file>
@@ -5038,7 +5059,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F616"/>
+  <dimension ref="A1:F619"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17367,6 +17388,66 @@
       </c>
       <c r="F616" s="2">
         <v>46125.59583333333</v>
+      </c>
+    </row>
+    <row r="617" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A617" s="3" t="s">
+        <v>1529</v>
+      </c>
+      <c r="B617" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C617" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D617" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E617" s="4" t="s">
+        <v>1530</v>
+      </c>
+      <c r="F617" s="2">
+        <v>46129.4625</v>
+      </c>
+    </row>
+    <row r="618" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A618" s="3" t="s">
+        <v>1531</v>
+      </c>
+      <c r="B618" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="C618" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D618" s="4" t="s">
+        <v>1417</v>
+      </c>
+      <c r="E618" s="4" t="s">
+        <v>1532</v>
+      </c>
+      <c r="F618" s="2">
+        <v>46128.825</v>
+      </c>
+    </row>
+    <row r="619" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A619" s="3" t="s">
+        <v>1533</v>
+      </c>
+      <c r="B619" s="4" t="s">
+        <v>1534</v>
+      </c>
+      <c r="C619" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D619" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E619" s="4" t="s">
+        <v>1535</v>
+      </c>
+      <c r="F619" s="2">
+        <v>46129.44861111111</v>
       </c>
     </row>
   </sheetData>
@@ -17986,6 +18067,9 @@
     <hyperlink ref="A614" r:id="rId613"/>
     <hyperlink ref="A615" r:id="rId614"/>
     <hyperlink ref="A616" r:id="rId615"/>
+    <hyperlink ref="A617" r:id="rId616"/>
+    <hyperlink ref="A618" r:id="rId617"/>
+    <hyperlink ref="A619" r:id="rId618"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -18030,62 +18114,62 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1529</v>
+        <v>1536</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>62</v>
+        <v>1537</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>48</v>
+        <v>190</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>67</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1530</v>
+        <v>1538</v>
       </c>
       <c r="F2" s="2">
-        <v>46129.4625</v>
+        <v>46130.56597222222</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1531</v>
+        <v>1539</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>246</v>
+        <v>337</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>146</v>
+        <v>208</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>1417</v>
+        <v>1007</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1532</v>
+        <v>1540</v>
       </c>
       <c r="F3" s="2">
-        <v>46128.825</v>
+        <v>46131.64722222222</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>1533</v>
+        <v>1541</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>1534</v>
+        <v>274</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>208</v>
+        <v>256</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>75</v>
+        <v>162</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>1535</v>
+        <v>1542</v>
       </c>
       <c r="F4" s="2">
-        <v>46129.44861111111</v>
+        <v>46130.63888888889</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-04-21 12:55
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3117" uniqueCount="1543">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3127" uniqueCount="1549">
   <si>
     <t>link</t>
   </si>
@@ -4647,6 +4647,24 @@
   </si>
   <si>
     <t>70860080049</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/bauska-and-reg/vecumnieku-pag/kifdn.html</t>
+  </si>
+  <si>
+    <t>128 000 €</t>
+  </si>
+  <si>
+    <t>27.60 ha.</t>
+  </si>
+  <si>
+    <t>40940130023; .47</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/limbadzi-and-reg/liepupes-pag/fenmx.html</t>
+  </si>
+  <si>
+    <t>135 800 €</t>
   </si>
 </sst>
 </file>
@@ -5059,7 +5077,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F619"/>
+  <dimension ref="A1:F622"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17448,6 +17466,66 @@
       </c>
       <c r="F619" s="2">
         <v>46129.44861111111</v>
+      </c>
+    </row>
+    <row r="620" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A620" s="3" t="s">
+        <v>1536</v>
+      </c>
+      <c r="B620" s="4" t="s">
+        <v>1537</v>
+      </c>
+      <c r="C620" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="D620" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E620" s="4" t="s">
+        <v>1538</v>
+      </c>
+      <c r="F620" s="2">
+        <v>46130.56597222222</v>
+      </c>
+    </row>
+    <row r="621" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A621" s="3" t="s">
+        <v>1539</v>
+      </c>
+      <c r="B621" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="C621" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D621" s="4" t="s">
+        <v>1007</v>
+      </c>
+      <c r="E621" s="4" t="s">
+        <v>1540</v>
+      </c>
+      <c r="F621" s="2">
+        <v>46131.64722222222</v>
+      </c>
+    </row>
+    <row r="622" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A622" s="3" t="s">
+        <v>1541</v>
+      </c>
+      <c r="B622" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="C622" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D622" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="E622" s="4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="F622" s="2">
+        <v>46130.63888888889</v>
       </c>
     </row>
   </sheetData>
@@ -18070,6 +18148,9 @@
     <hyperlink ref="A617" r:id="rId616"/>
     <hyperlink ref="A618" r:id="rId617"/>
     <hyperlink ref="A619" r:id="rId618"/>
+    <hyperlink ref="A620" r:id="rId619"/>
+    <hyperlink ref="A621" r:id="rId620"/>
+    <hyperlink ref="A622" r:id="rId621"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -18081,7 +18162,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18114,69 +18195,48 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1536</v>
+        <v>1543</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1537</v>
+        <v>1544</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>190</v>
+        <v>48</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>67</v>
+        <v>1545</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1538</v>
+        <v>1546</v>
       </c>
       <c r="F2" s="2">
-        <v>46130.56597222222</v>
+        <v>46133.60902777778</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1539</v>
+        <v>1547</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>337</v>
+        <v>1548</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>208</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>1007</v>
+        <v>75</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1540</v>
+        <v>1535</v>
       </c>
       <c r="F3" s="2">
-        <v>46131.64722222222</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1541</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>274</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1542</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46130.63888888889</v>
+        <v>46133.62777777778</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-04-22 12:55
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3127" uniqueCount="1549">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3137" uniqueCount="1553">
   <si>
     <t>link</t>
   </si>
@@ -4665,6 +4665,18 @@
   </si>
   <si>
     <t>135 800 €</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/kalna-pag/adilf.html</t>
+  </si>
+  <si>
+    <t>56660060200</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/rites-pag/kglbh.html</t>
+  </si>
+  <si>
+    <t>7.37 ha.</t>
   </si>
 </sst>
 </file>
@@ -5077,7 +5089,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F622"/>
+  <dimension ref="A1:F624"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17526,6 +17538,46 @@
       </c>
       <c r="F622" s="2">
         <v>46130.63888888889</v>
+      </c>
+    </row>
+    <row r="623" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A623" s="3" t="s">
+        <v>1543</v>
+      </c>
+      <c r="B623" s="4" t="s">
+        <v>1544</v>
+      </c>
+      <c r="C623" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D623" s="4" t="s">
+        <v>1545</v>
+      </c>
+      <c r="E623" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="F623" s="2">
+        <v>46133.60902777778</v>
+      </c>
+    </row>
+    <row r="624" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A624" s="3" t="s">
+        <v>1547</v>
+      </c>
+      <c r="B624" s="4" t="s">
+        <v>1548</v>
+      </c>
+      <c r="C624" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D624" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E624" s="4" t="s">
+        <v>1535</v>
+      </c>
+      <c r="F624" s="2">
+        <v>46133.62777777778</v>
       </c>
     </row>
   </sheetData>
@@ -18151,6 +18203,8 @@
     <hyperlink ref="A620" r:id="rId619"/>
     <hyperlink ref="A621" r:id="rId620"/>
     <hyperlink ref="A622" r:id="rId621"/>
+    <hyperlink ref="A623" r:id="rId622"/>
+    <hyperlink ref="A624" r:id="rId623"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -18195,42 +18249,42 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1543</v>
+        <v>1549</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1544</v>
+        <v>88</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>48</v>
+        <v>127</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>1545</v>
+        <v>82</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1546</v>
+        <v>1550</v>
       </c>
       <c r="F2" s="2">
-        <v>46133.60902777778</v>
+        <v>46134.49166666667</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1547</v>
+        <v>1551</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>1548</v>
+        <v>271</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>208</v>
+        <v>127</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>75</v>
+        <v>1552</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1535</v>
+        <v>25</v>
       </c>
       <c r="F3" s="2">
-        <v>46133.62777777778</v>
+        <v>46134.351388888885</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-04-23 12:55
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3137" uniqueCount="1553">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3147" uniqueCount="1556">
   <si>
     <t>link</t>
   </si>
@@ -4677,6 +4677,15 @@
   </si>
   <si>
     <t>7.37 ha.</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/lazdukalna-pag/dlxfh.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/raiskuma-pag/hihce.html</t>
+  </si>
+  <si>
+    <t>47240060117</t>
   </si>
 </sst>
 </file>
@@ -5089,7 +5098,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F624"/>
+  <dimension ref="A1:F626"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17578,6 +17587,46 @@
       </c>
       <c r="F624" s="2">
         <v>46133.62777777778</v>
+      </c>
+    </row>
+    <row r="625" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A625" s="3" t="s">
+        <v>1549</v>
+      </c>
+      <c r="B625" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C625" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D625" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E625" s="4" t="s">
+        <v>1550</v>
+      </c>
+      <c r="F625" s="2">
+        <v>46134.49166666667</v>
+      </c>
+    </row>
+    <row r="626" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A626" s="3" t="s">
+        <v>1551</v>
+      </c>
+      <c r="B626" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="C626" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D626" s="4" t="s">
+        <v>1552</v>
+      </c>
+      <c r="E626" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F626" s="2">
+        <v>46134.351388888885</v>
       </c>
     </row>
   </sheetData>
@@ -18205,6 +18254,8 @@
     <hyperlink ref="A622" r:id="rId621"/>
     <hyperlink ref="A623" r:id="rId622"/>
     <hyperlink ref="A624" r:id="rId623"/>
+    <hyperlink ref="A625" r:id="rId624"/>
+    <hyperlink ref="A626" r:id="rId625"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -18249,42 +18300,42 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1549</v>
+        <v>1553</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>88</v>
+        <v>204</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>127</v>
+        <v>28</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>82</v>
+        <v>162</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1550</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46134.49166666667</v>
+        <v>46135.43888888889</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1551</v>
+        <v>1554</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>271</v>
+        <v>106</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>127</v>
+        <v>63</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>1552</v>
+        <v>24</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>25</v>
+        <v>1555</v>
       </c>
       <c r="F3" s="2">
-        <v>46134.351388888885</v>
+        <v>46134.822222222225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-04-24 12:53
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3147" uniqueCount="1556">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3162" uniqueCount="1564">
   <si>
     <t>link</t>
   </si>
@@ -4686,6 +4686,30 @@
   </si>
   <si>
     <t>47240060117</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/susaju-pag/nlhon.html</t>
+  </si>
+  <si>
+    <t>170 000 €</t>
+  </si>
+  <si>
+    <t>26 ha.</t>
+  </si>
+  <si>
+    <t>38780130015</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/bikernieku-pag/poodp.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/rozupes-pag/mgcfi.html</t>
+  </si>
+  <si>
+    <t>23 ha.</t>
+  </si>
+  <si>
+    <t>76660090393</t>
   </si>
 </sst>
 </file>
@@ -5098,7 +5122,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F626"/>
+  <dimension ref="A1:F628"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17627,6 +17651,46 @@
       </c>
       <c r="F626" s="2">
         <v>46134.351388888885</v>
+      </c>
+    </row>
+    <row r="627" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A627" s="3" t="s">
+        <v>1553</v>
+      </c>
+      <c r="B627" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C627" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D627" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="E627" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F627" s="2">
+        <v>46135.43888888889</v>
+      </c>
+    </row>
+    <row r="628" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A628" s="3" t="s">
+        <v>1554</v>
+      </c>
+      <c r="B628" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C628" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D628" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E628" s="4" t="s">
+        <v>1555</v>
+      </c>
+      <c r="F628" s="2">
+        <v>46134.822222222225</v>
       </c>
     </row>
   </sheetData>
@@ -18256,6 +18320,8 @@
     <hyperlink ref="A624" r:id="rId623"/>
     <hyperlink ref="A625" r:id="rId624"/>
     <hyperlink ref="A626" r:id="rId625"/>
+    <hyperlink ref="A627" r:id="rId626"/>
+    <hyperlink ref="A628" r:id="rId627"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -18267,7 +18333,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18300,48 +18366,69 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1553</v>
+        <v>1556</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>204</v>
+        <v>1557</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>28</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>162</v>
+        <v>1558</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>25</v>
+        <v>1559</v>
       </c>
       <c r="F2" s="2">
-        <v>46135.43888888889</v>
+        <v>46136.39583333333</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1554</v>
+        <v>1560</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>106</v>
+        <v>134</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1555</v>
+        <v>25</v>
       </c>
       <c r="F3" s="2">
-        <v>46134.822222222225</v>
+        <v>46136.27777777778</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1561</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>1562</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1563</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46135.736805555556</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-04-27 13:13
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3162" uniqueCount="1564">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3187" uniqueCount="1572">
   <si>
     <t>link</t>
   </si>
@@ -4710,6 +4710,30 @@
   </si>
   <si>
     <t>76660090393</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/gulbene-and-reg/stamerienas-pag/egenn.html</t>
+  </si>
+  <si>
+    <t>50880030055</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/aronas-pag/jbkpi.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/griskanu-pag/edclk.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/sakstagala-pag/ehjjn.html</t>
+  </si>
+  <si>
+    <t>78860070038</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/other/hxlkn.html</t>
+  </si>
+  <si>
+    <t>120 €</t>
   </si>
 </sst>
 </file>
@@ -5122,7 +5146,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F628"/>
+  <dimension ref="A1:F631"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17691,6 +17715,66 @@
       </c>
       <c r="F628" s="2">
         <v>46134.822222222225</v>
+      </c>
+    </row>
+    <row r="629" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A629" s="3" t="s">
+        <v>1556</v>
+      </c>
+      <c r="B629" s="4" t="s">
+        <v>1557</v>
+      </c>
+      <c r="C629" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D629" s="4" t="s">
+        <v>1558</v>
+      </c>
+      <c r="E629" s="4" t="s">
+        <v>1559</v>
+      </c>
+      <c r="F629" s="2">
+        <v>46136.39583333333</v>
+      </c>
+    </row>
+    <row r="630" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A630" s="3" t="s">
+        <v>1560</v>
+      </c>
+      <c r="B630" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="C630" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D630" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E630" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F630" s="2">
+        <v>46136.27777777778</v>
+      </c>
+    </row>
+    <row r="631" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A631" s="3" t="s">
+        <v>1561</v>
+      </c>
+      <c r="B631" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C631" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D631" s="4" t="s">
+        <v>1562</v>
+      </c>
+      <c r="E631" s="4" t="s">
+        <v>1563</v>
+      </c>
+      <c r="F631" s="2">
+        <v>46135.736805555556</v>
       </c>
     </row>
   </sheetData>
@@ -18322,6 +18406,9 @@
     <hyperlink ref="A626" r:id="rId625"/>
     <hyperlink ref="A627" r:id="rId626"/>
     <hyperlink ref="A628" r:id="rId627"/>
+    <hyperlink ref="A629" r:id="rId628"/>
+    <hyperlink ref="A630" r:id="rId629"/>
+    <hyperlink ref="A631" r:id="rId630"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -18333,7 +18420,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18366,62 +18453,102 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1556</v>
+        <v>1564</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1557</v>
+        <v>91</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>28</v>
+        <v>124</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>1558</v>
+        <v>135</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1559</v>
+        <v>1565</v>
       </c>
       <c r="F2" s="2">
-        <v>46136.39583333333</v>
+        <v>46139.33263888889</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1560</v>
+        <v>1566</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>134</v>
+        <v>70</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>74</v>
+        <v>256</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>25</v>
       </c>
       <c r="F3" s="2">
-        <v>46136.27777777778</v>
+        <v>46137.52569444444</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>1561</v>
+        <v>1567</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>102</v>
+        <v>204</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>284</v>
+        <v>294</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>1562</v>
+        <v>59</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>1563</v>
+        <v>820</v>
       </c>
       <c r="F4" s="2">
-        <v>46135.736805555556</v>
+        <v>46139.35625</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1568</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1569</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46137.56736111111</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>1570</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>1571</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46139.601388888885</v>
       </c>
     </row>
   </sheetData>
@@ -18429,6 +18556,8 @@
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
     <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+    <hyperlink ref="A6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-04-28 13:23
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -5146,7 +5146,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F631"/>
+  <dimension ref="A1:F636"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17775,6 +17775,106 @@
       </c>
       <c r="F631" s="2">
         <v>46135.736805555556</v>
+      </c>
+    </row>
+    <row r="632" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A632" s="3" t="s">
+        <v>1564</v>
+      </c>
+      <c r="B632" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C632" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D632" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E632" s="4" t="s">
+        <v>1565</v>
+      </c>
+      <c r="F632" s="2">
+        <v>46139.33263888889</v>
+      </c>
+    </row>
+    <row r="633" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A633" s="3" t="s">
+        <v>1566</v>
+      </c>
+      <c r="B633" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C633" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D633" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E633" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F633" s="2">
+        <v>46137.52569444444</v>
+      </c>
+    </row>
+    <row r="634" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A634" s="3" t="s">
+        <v>1567</v>
+      </c>
+      <c r="B634" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C634" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D634" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E634" s="4" t="s">
+        <v>820</v>
+      </c>
+      <c r="F634" s="2">
+        <v>46139.35625</v>
+      </c>
+    </row>
+    <row r="635" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A635" s="3" t="s">
+        <v>1568</v>
+      </c>
+      <c r="B635" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C635" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D635" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E635" s="4" t="s">
+        <v>1569</v>
+      </c>
+      <c r="F635" s="2">
+        <v>46137.56736111111</v>
+      </c>
+    </row>
+    <row r="636" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A636" s="3" t="s">
+        <v>1570</v>
+      </c>
+      <c r="B636" s="4" t="s">
+        <v>1571</v>
+      </c>
+      <c r="C636" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D636" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E636" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F636" s="2">
+        <v>46139.601388888885</v>
       </c>
     </row>
   </sheetData>
@@ -18409,6 +18509,11 @@
     <hyperlink ref="A629" r:id="rId628"/>
     <hyperlink ref="A630" r:id="rId629"/>
     <hyperlink ref="A631" r:id="rId630"/>
+    <hyperlink ref="A632" r:id="rId631"/>
+    <hyperlink ref="A633" r:id="rId632"/>
+    <hyperlink ref="A634" r:id="rId633"/>
+    <hyperlink ref="A635" r:id="rId634"/>
+    <hyperlink ref="A636" r:id="rId635"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -18420,7 +18525,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18451,114 +18556,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>1564</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>1565</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46139.33263888889</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1566</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46137.52569444444</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1567</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>820</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46139.35625</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1568</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1569</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46137.56736111111</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>1570</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>1571</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46139.601388888885</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A6" r:id="rId5"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-04-30 13:15
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3187" uniqueCount="1572">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3192" uniqueCount="1574">
   <si>
     <t>link</t>
   </si>
@@ -4734,6 +4734,12 @@
   </si>
   <si>
     <t>120 €</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/saldus-and-reg/novadnieku-pag/cgleep.html</t>
+  </si>
+  <si>
+    <t>84720030176</t>
   </si>
 </sst>
 </file>
@@ -18525,7 +18531,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18556,7 +18562,30 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>1572</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>1573</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46141.76736111111</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-05-01 12:49
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3192" uniqueCount="1574">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3197" uniqueCount="1576">
   <si>
     <t>link</t>
   </si>
@@ -4740,6 +4740,12 @@
   </si>
   <si>
     <t>84720030176</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/makonkalna-pag/fimin.html</t>
+  </si>
+  <si>
+    <t>3.50 ha.</t>
   </si>
 </sst>
 </file>
@@ -5152,7 +5158,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F636"/>
+  <dimension ref="A1:F637"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17881,6 +17887,26 @@
       </c>
       <c r="F636" s="2">
         <v>46139.601388888885</v>
+      </c>
+    </row>
+    <row r="637" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A637" s="3" t="s">
+        <v>1572</v>
+      </c>
+      <c r="B637" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C637" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="D637" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="E637" s="4" t="s">
+        <v>1573</v>
+      </c>
+      <c r="F637" s="2">
+        <v>46141.76736111111</v>
       </c>
     </row>
   </sheetData>
@@ -18520,6 +18546,7 @@
     <hyperlink ref="A634" r:id="rId633"/>
     <hyperlink ref="A635" r:id="rId634"/>
     <hyperlink ref="A636" r:id="rId635"/>
+    <hyperlink ref="A637" r:id="rId636"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -18564,22 +18591,22 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1572</v>
+        <v>1574</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>131</v>
+        <v>707</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>346</v>
+        <v>294</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>212</v>
+        <v>1575</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1573</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46141.76736111111</v>
+        <v>46143.04652777778</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-05-04 13:17
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3197" uniqueCount="1576">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3217" uniqueCount="1585">
   <si>
     <t>link</t>
   </si>
@@ -4746,6 +4746,33 @@
   </si>
   <si>
     <t>3.50 ha.</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/demenes-pag/obhkd.html</t>
+  </si>
+  <si>
+    <t>44500040390</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/praulienas-pag/cfepm.html</t>
+  </si>
+  <si>
+    <t>7.90 ha.</t>
+  </si>
+  <si>
+    <t>70860110092</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/sakstagala-pag/hnxeg.html</t>
+  </si>
+  <si>
+    <t>78860060501</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/tukums-and-reg/irlavas-pag/bbhbc.html</t>
+  </si>
+  <si>
+    <t>90540030059</t>
   </si>
 </sst>
 </file>
@@ -5158,7 +5185,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F637"/>
+  <dimension ref="A1:F638"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17907,6 +17934,26 @@
       </c>
       <c r="F637" s="2">
         <v>46141.76736111111</v>
+      </c>
+    </row>
+    <row r="638" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A638" s="3" t="s">
+        <v>1574</v>
+      </c>
+      <c r="B638" s="4" t="s">
+        <v>707</v>
+      </c>
+      <c r="C638" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D638" s="4" t="s">
+        <v>1575</v>
+      </c>
+      <c r="E638" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F638" s="2">
+        <v>46143.04652777778</v>
       </c>
     </row>
   </sheetData>
@@ -18547,6 +18594,7 @@
     <hyperlink ref="A635" r:id="rId634"/>
     <hyperlink ref="A636" r:id="rId635"/>
     <hyperlink ref="A637" r:id="rId636"/>
+    <hyperlink ref="A638" r:id="rId637"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -18558,7 +18606,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18591,27 +18639,90 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1574</v>
+        <v>1576</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>707</v>
+        <v>501</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>1577</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46143.81875</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1578</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>1579</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1580</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46145.57916666666</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1581</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>294</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>1575</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46143.04652777778</v>
+      <c r="D4" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1582</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46146.59722222222</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1583</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1584</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46144.40277777778</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-05-05 13:04
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -5185,7 +5185,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F638"/>
+  <dimension ref="A1:F642"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -17954,6 +17954,86 @@
       </c>
       <c r="F638" s="2">
         <v>46143.04652777778</v>
+      </c>
+    </row>
+    <row r="639" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A639" s="3" t="s">
+        <v>1576</v>
+      </c>
+      <c r="B639" s="4" t="s">
+        <v>501</v>
+      </c>
+      <c r="C639" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D639" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E639" s="4" t="s">
+        <v>1577</v>
+      </c>
+      <c r="F639" s="2">
+        <v>46143.81875</v>
+      </c>
+    </row>
+    <row r="640" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A640" s="3" t="s">
+        <v>1578</v>
+      </c>
+      <c r="B640" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="C640" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D640" s="4" t="s">
+        <v>1579</v>
+      </c>
+      <c r="E640" s="4" t="s">
+        <v>1580</v>
+      </c>
+      <c r="F640" s="2">
+        <v>46145.57916666666</v>
+      </c>
+    </row>
+    <row r="641" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A641" s="3" t="s">
+        <v>1581</v>
+      </c>
+      <c r="B641" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="C641" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D641" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E641" s="4" t="s">
+        <v>1582</v>
+      </c>
+      <c r="F641" s="2">
+        <v>46146.59722222222</v>
+      </c>
+    </row>
+    <row r="642" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A642" s="3" t="s">
+        <v>1583</v>
+      </c>
+      <c r="B642" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C642" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D642" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E642" s="4" t="s">
+        <v>1584</v>
+      </c>
+      <c r="F642" s="2">
+        <v>46144.40277777778</v>
       </c>
     </row>
   </sheetData>
@@ -18595,6 +18675,10 @@
     <hyperlink ref="A636" r:id="rId635"/>
     <hyperlink ref="A637" r:id="rId636"/>
     <hyperlink ref="A638" r:id="rId637"/>
+    <hyperlink ref="A639" r:id="rId638"/>
+    <hyperlink ref="A640" r:id="rId639"/>
+    <hyperlink ref="A641" r:id="rId640"/>
+    <hyperlink ref="A642" r:id="rId641"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -18606,7 +18690,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18637,93 +18721,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>1576</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>501</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>1577</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46143.81875</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1578</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>1579</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1580</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46145.57916666666</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1581</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>576</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1582</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46146.59722222222</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1583</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>376</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1584</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46144.40277777778</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-05-06 13:24
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3217" uniqueCount="1585">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3222" uniqueCount="1587">
   <si>
     <t>link</t>
   </si>
@@ -4773,6 +4773,12 @@
   </si>
   <si>
     <t>90540030059</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aizkraukle-and-reg/sunakstes-pag/iehgk.html</t>
+  </si>
+  <si>
+    <t>32850080014</t>
   </si>
 </sst>
 </file>
@@ -18690,7 +18696,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18721,7 +18727,30 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>1585</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>1586</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46147.9875</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-05-07 13:26
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3222" uniqueCount="1587">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3257" uniqueCount="1599">
   <si>
     <t>link</t>
   </si>
@@ -4779,6 +4779,42 @@
   </si>
   <si>
     <t>32850080014</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aizkraukle-and-reg/klintaines-pag/ibnkx.html</t>
+  </si>
+  <si>
+    <t>32580060031</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/aluksne/cxobxp.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/jaunaluksnes-pag/njkdi.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/ziguru-pag/jhfig.html</t>
+  </si>
+  <si>
+    <t>38980040118</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/balvi/fblgk.html</t>
+  </si>
+  <si>
+    <t>38980040049</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/berzpils-pag/oegpj.html</t>
+  </si>
+  <si>
+    <t>4.85 ha.</t>
+  </si>
+  <si>
+    <t>38500070087</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valka-and-reg/other/ebmil.html</t>
   </si>
 </sst>
 </file>
@@ -5191,7 +5227,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F642"/>
+  <dimension ref="A1:F643"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18040,6 +18076,26 @@
       </c>
       <c r="F642" s="2">
         <v>46144.40277777778</v>
+      </c>
+    </row>
+    <row r="643" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A643" s="3" t="s">
+        <v>1585</v>
+      </c>
+      <c r="B643" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="C643" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D643" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E643" s="4" t="s">
+        <v>1586</v>
+      </c>
+      <c r="F643" s="2">
+        <v>46147.9875</v>
       </c>
     </row>
   </sheetData>
@@ -18685,6 +18741,7 @@
     <hyperlink ref="A640" r:id="rId639"/>
     <hyperlink ref="A641" r:id="rId640"/>
     <hyperlink ref="A642" r:id="rId641"/>
+    <hyperlink ref="A643" r:id="rId642"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -18696,7 +18753,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18729,27 +18786,153 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1585</v>
+        <v>1587</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>211</v>
+        <v>106</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>85</v>
+        <v>13</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1586</v>
+        <v>1588</v>
       </c>
       <c r="F2" s="2">
-        <v>46147.9875</v>
+        <v>46149.50208333333</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1589</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46148.79513888889</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1590</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46148.74652777778</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1591</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1592</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46149.32291666667</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>1593</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>1594</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46149.320138888885</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>1595</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>1596</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>1597</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46149.31458333333</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>1598</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" s="2">
+        <v>46149.42361111111</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+    <hyperlink ref="A6" r:id="rId5"/>
+    <hyperlink ref="A7" r:id="rId6"/>
+    <hyperlink ref="A8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-05-08 13:06
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3257" uniqueCount="1599">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3277" uniqueCount="1607">
   <si>
     <t>link</t>
   </si>
@@ -4815,6 +4815,30 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/valka-and-reg/other/ebmil.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/aluksne/ghfcg.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/bauska-and-reg/skaistkalnes-pag/ddclf.html</t>
+  </si>
+  <si>
+    <t>32 400 €</t>
+  </si>
+  <si>
+    <t>40800010099</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/gulbene-and-reg/daukstu-pag/jdbkl.html</t>
+  </si>
+  <si>
+    <t>7.10 ha.</t>
+  </si>
+  <si>
+    <t>50480030108</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valka-and-reg/smiltenes-pag/bdhhic.html</t>
   </si>
 </sst>
 </file>
@@ -5227,7 +5251,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F643"/>
+  <dimension ref="A1:F650"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18096,6 +18120,146 @@
       </c>
       <c r="F643" s="2">
         <v>46147.9875</v>
+      </c>
+    </row>
+    <row r="644" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A644" s="3" t="s">
+        <v>1587</v>
+      </c>
+      <c r="B644" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C644" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D644" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E644" s="4" t="s">
+        <v>1588</v>
+      </c>
+      <c r="F644" s="2">
+        <v>46149.50208333333</v>
+      </c>
+    </row>
+    <row r="645" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A645" s="3" t="s">
+        <v>1589</v>
+      </c>
+      <c r="B645" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C645" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D645" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E645" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F645" s="2">
+        <v>46148.79513888889</v>
+      </c>
+    </row>
+    <row r="646" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A646" s="3" t="s">
+        <v>1590</v>
+      </c>
+      <c r="B646" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C646" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D646" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E646" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F646" s="2">
+        <v>46148.74652777778</v>
+      </c>
+    </row>
+    <row r="647" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A647" s="3" t="s">
+        <v>1591</v>
+      </c>
+      <c r="B647" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="C647" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D647" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E647" s="4" t="s">
+        <v>1592</v>
+      </c>
+      <c r="F647" s="2">
+        <v>46149.32291666667</v>
+      </c>
+    </row>
+    <row r="648" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A648" s="3" t="s">
+        <v>1593</v>
+      </c>
+      <c r="B648" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="C648" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D648" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E648" s="4" t="s">
+        <v>1594</v>
+      </c>
+      <c r="F648" s="2">
+        <v>46149.320138888885</v>
+      </c>
+    </row>
+    <row r="649" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A649" s="3" t="s">
+        <v>1595</v>
+      </c>
+      <c r="B649" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="C649" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D649" s="4" t="s">
+        <v>1596</v>
+      </c>
+      <c r="E649" s="4" t="s">
+        <v>1597</v>
+      </c>
+      <c r="F649" s="2">
+        <v>46149.31458333333</v>
+      </c>
+    </row>
+    <row r="650" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A650" s="3" t="s">
+        <v>1598</v>
+      </c>
+      <c r="B650" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C650" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="D650" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E650" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F650" s="2">
+        <v>46149.42361111111</v>
       </c>
     </row>
   </sheetData>
@@ -18742,6 +18906,13 @@
     <hyperlink ref="A641" r:id="rId640"/>
     <hyperlink ref="A642" r:id="rId641"/>
     <hyperlink ref="A643" r:id="rId642"/>
+    <hyperlink ref="A644" r:id="rId643"/>
+    <hyperlink ref="A645" r:id="rId644"/>
+    <hyperlink ref="A646" r:id="rId645"/>
+    <hyperlink ref="A647" r:id="rId646"/>
+    <hyperlink ref="A648" r:id="rId647"/>
+    <hyperlink ref="A649" r:id="rId648"/>
+    <hyperlink ref="A650" r:id="rId649"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -18753,7 +18924,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18786,142 +18957,82 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1587</v>
+        <v>1599</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>106</v>
+        <v>25</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>8</v>
+        <v>435</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1588</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46149.50208333333</v>
+        <v>46150.228472222225</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1589</v>
+        <v>1600</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>25</v>
+        <v>1601</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>435</v>
+        <v>48</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>25</v>
+        <v>1602</v>
       </c>
       <c r="F3" s="2">
-        <v>46148.79513888889</v>
+        <v>46150.367361111115</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>1590</v>
+        <v>1603</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>435</v>
+        <v>124</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>25</v>
+        <v>1604</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>25</v>
+        <v>1605</v>
       </c>
       <c r="F4" s="2">
-        <v>46148.74652777778</v>
+        <v>46150.481944444444</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>1591</v>
+        <v>1606</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>274</v>
+        <v>25</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>28</v>
+        <v>392</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>135</v>
+        <v>25</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>1592</v>
+        <v>25</v>
       </c>
       <c r="F5" s="2">
-        <v>46149.32291666667</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>1593</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>1594</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46149.320138888885</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>1595</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>1596</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>1597</v>
-      </c>
-      <c r="F7" s="2">
-        <v>46149.31458333333</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>1598</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>392</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F8" s="2">
-        <v>46149.42361111111</v>
+        <v>46150.231944444444</v>
       </c>
     </row>
   </sheetData>
@@ -18930,9 +19041,6 @@
     <hyperlink ref="A3" r:id="rId2"/>
     <hyperlink ref="A4" r:id="rId3"/>
     <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A6" r:id="rId5"/>
-    <hyperlink ref="A7" r:id="rId6"/>
-    <hyperlink ref="A8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-05-11 19:01
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3277" uniqueCount="1607">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3297" uniqueCount="1614">
   <si>
     <t>link</t>
   </si>
@@ -4839,6 +4839,27 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/valka-and-reg/smiltenes-pag/bdhhic.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/jaunannas-pag/bboken.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/aluksne/dkpfd.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/limbadzi-and-reg/aloja/odlbl.html</t>
+  </si>
+  <si>
+    <t>87 000 €</t>
+  </si>
+  <si>
+    <t>66270040395</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/dzelzavas-pag/oddlb.html</t>
+  </si>
+  <si>
+    <t>70500080034</t>
   </si>
 </sst>
 </file>
@@ -5251,7 +5272,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F650"/>
+  <dimension ref="A1:F654"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18260,6 +18281,86 @@
       </c>
       <c r="F650" s="2">
         <v>46149.42361111111</v>
+      </c>
+    </row>
+    <row r="651" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A651" s="3" t="s">
+        <v>1599</v>
+      </c>
+      <c r="B651" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C651" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D651" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E651" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F651" s="2">
+        <v>46150.228472222225</v>
+      </c>
+    </row>
+    <row r="652" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A652" s="3" t="s">
+        <v>1600</v>
+      </c>
+      <c r="B652" s="4" t="s">
+        <v>1601</v>
+      </c>
+      <c r="C652" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D652" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E652" s="4" t="s">
+        <v>1602</v>
+      </c>
+      <c r="F652" s="2">
+        <v>46150.367361111115</v>
+      </c>
+    </row>
+    <row r="653" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A653" s="3" t="s">
+        <v>1603</v>
+      </c>
+      <c r="B653" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C653" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D653" s="4" t="s">
+        <v>1604</v>
+      </c>
+      <c r="E653" s="4" t="s">
+        <v>1605</v>
+      </c>
+      <c r="F653" s="2">
+        <v>46150.481944444444</v>
+      </c>
+    </row>
+    <row r="654" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A654" s="3" t="s">
+        <v>1606</v>
+      </c>
+      <c r="B654" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C654" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="D654" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E654" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F654" s="2">
+        <v>46150.231944444444</v>
       </c>
     </row>
   </sheetData>
@@ -18913,6 +19014,10 @@
     <hyperlink ref="A648" r:id="rId647"/>
     <hyperlink ref="A649" r:id="rId648"/>
     <hyperlink ref="A650" r:id="rId649"/>
+    <hyperlink ref="A651" r:id="rId650"/>
+    <hyperlink ref="A652" r:id="rId651"/>
+    <hyperlink ref="A653" r:id="rId652"/>
+    <hyperlink ref="A654" r:id="rId653"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -18957,7 +19062,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1599</v>
+        <v>1607</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>25</v>
@@ -18972,67 +19077,67 @@
         <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46150.228472222225</v>
+        <v>46153.65</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1600</v>
+        <v>1608</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>1601</v>
+        <v>25</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>48</v>
+        <v>435</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1602</v>
+        <v>25</v>
       </c>
       <c r="F3" s="2">
-        <v>46150.367361111115</v>
+        <v>46153.388194444444</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>1603</v>
+        <v>1609</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>91</v>
+        <v>1610</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>124</v>
+        <v>208</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>1604</v>
+        <v>67</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>1605</v>
+        <v>1611</v>
       </c>
       <c r="F4" s="2">
-        <v>46150.481944444444</v>
+        <v>46150.76944444445</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>1606</v>
+        <v>1612</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>25</v>
+        <v>116</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>392</v>
+        <v>256</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>25</v>
+        <v>272</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>25</v>
+        <v>1613</v>
       </c>
       <c r="F5" s="2">
-        <v>46150.231944444444</v>
+        <v>46150.875</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-05-12 13:34
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3297" uniqueCount="1614">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3307" uniqueCount="1616">
   <si>
     <t>link</t>
   </si>
@@ -4860,6 +4860,12 @@
   </si>
   <si>
     <t>70500080034</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/other/bfmmp.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/markalnes-pag/bcdcfb.html</t>
   </si>
 </sst>
 </file>
@@ -5272,7 +5278,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F654"/>
+  <dimension ref="A1:F658"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18361,6 +18367,86 @@
       </c>
       <c r="F654" s="2">
         <v>46150.231944444444</v>
+      </c>
+    </row>
+    <row r="655" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A655" s="3" t="s">
+        <v>1607</v>
+      </c>
+      <c r="B655" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C655" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D655" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E655" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F655" s="2">
+        <v>46153.65</v>
+      </c>
+    </row>
+    <row r="656" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A656" s="3" t="s">
+        <v>1608</v>
+      </c>
+      <c r="B656" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C656" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D656" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E656" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F656" s="2">
+        <v>46153.388194444444</v>
+      </c>
+    </row>
+    <row r="657" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A657" s="3" t="s">
+        <v>1609</v>
+      </c>
+      <c r="B657" s="4" t="s">
+        <v>1610</v>
+      </c>
+      <c r="C657" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D657" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E657" s="4" t="s">
+        <v>1611</v>
+      </c>
+      <c r="F657" s="2">
+        <v>46150.76944444445</v>
+      </c>
+    </row>
+    <row r="658" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A658" s="3" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B658" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C658" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D658" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E658" s="4" t="s">
+        <v>1613</v>
+      </c>
+      <c r="F658" s="2">
+        <v>46150.875</v>
       </c>
     </row>
   </sheetData>
@@ -19018,6 +19104,10 @@
     <hyperlink ref="A652" r:id="rId651"/>
     <hyperlink ref="A653" r:id="rId652"/>
     <hyperlink ref="A654" r:id="rId653"/>
+    <hyperlink ref="A655" r:id="rId654"/>
+    <hyperlink ref="A656" r:id="rId655"/>
+    <hyperlink ref="A657" r:id="rId656"/>
+    <hyperlink ref="A658" r:id="rId657"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -19029,7 +19119,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19062,7 +19152,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1607</v>
+        <v>1614</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>25</v>
@@ -19077,12 +19167,12 @@
         <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46153.65</v>
+        <v>46154.603472222225</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1608</v>
+        <v>1615</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>25</v>
@@ -19097,55 +19187,13 @@
         <v>25</v>
       </c>
       <c r="F3" s="2">
-        <v>46153.388194444444</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1609</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>1610</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1611</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46150.76944444445</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1612</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1613</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46150.875</v>
+        <v>46154.39791666667</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-05-13 14:00
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3307" uniqueCount="1616">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3322" uniqueCount="1621">
   <si>
     <t>link</t>
   </si>
@@ -4866,6 +4866,21 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/markalnes-pag/bcdcfb.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/dobele-and-reg/annenieku-pag/dlfpn.html</t>
+  </si>
+  <si>
+    <t>46420040012</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/krustpils-pag/ocjxm.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kuldiga-and-reg/skrunda/lfino.html</t>
+  </si>
+  <si>
+    <t>62820070018</t>
   </si>
 </sst>
 </file>
@@ -5278,7 +5293,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F658"/>
+  <dimension ref="A1:F660"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18447,6 +18462,46 @@
       </c>
       <c r="F658" s="2">
         <v>46150.875</v>
+      </c>
+    </row>
+    <row r="659" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A659" s="3" t="s">
+        <v>1614</v>
+      </c>
+      <c r="B659" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C659" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D659" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E659" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F659" s="2">
+        <v>46154.603472222225</v>
+      </c>
+    </row>
+    <row r="660" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A660" s="3" t="s">
+        <v>1615</v>
+      </c>
+      <c r="B660" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C660" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D660" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E660" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F660" s="2">
+        <v>46154.39791666667</v>
       </c>
     </row>
   </sheetData>
@@ -19108,6 +19163,8 @@
     <hyperlink ref="A656" r:id="rId655"/>
     <hyperlink ref="A657" r:id="rId656"/>
     <hyperlink ref="A658" r:id="rId657"/>
+    <hyperlink ref="A659" r:id="rId658"/>
+    <hyperlink ref="A660" r:id="rId659"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -19119,7 +19176,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19152,48 +19209,69 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1614</v>
+        <v>1616</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>25</v>
+        <v>793</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>435</v>
+        <v>117</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>25</v>
+        <v>1575</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>25</v>
+        <v>1617</v>
       </c>
       <c r="F2" s="2">
-        <v>46154.603472222225</v>
+        <v>46154.83263888889</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1615</v>
+        <v>1618</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>25</v>
+        <v>271</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>435</v>
+        <v>127</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>25</v>
+        <v>186</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>25</v>
       </c>
       <c r="F3" s="2">
-        <v>46154.39791666667</v>
+        <v>46155.629166666666</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1619</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1620</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46155.54652777778</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-05-14 13:25
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -5293,7 +5293,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F660"/>
+  <dimension ref="A1:F663"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18502,6 +18502,66 @@
       </c>
       <c r="F660" s="2">
         <v>46154.39791666667</v>
+      </c>
+    </row>
+    <row r="661" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A661" s="3" t="s">
+        <v>1616</v>
+      </c>
+      <c r="B661" s="4" t="s">
+        <v>793</v>
+      </c>
+      <c r="C661" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D661" s="4" t="s">
+        <v>1575</v>
+      </c>
+      <c r="E661" s="4" t="s">
+        <v>1617</v>
+      </c>
+      <c r="F661" s="2">
+        <v>46154.83263888889</v>
+      </c>
+    </row>
+    <row r="662" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A662" s="3" t="s">
+        <v>1618</v>
+      </c>
+      <c r="B662" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="C662" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D662" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E662" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F662" s="2">
+        <v>46155.629166666666</v>
+      </c>
+    </row>
+    <row r="663" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A663" s="3" t="s">
+        <v>1619</v>
+      </c>
+      <c r="B663" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C663" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="D663" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="E663" s="4" t="s">
+        <v>1620</v>
+      </c>
+      <c r="F663" s="2">
+        <v>46155.54652777778</v>
       </c>
     </row>
   </sheetData>
@@ -19165,6 +19225,9 @@
     <hyperlink ref="A658" r:id="rId657"/>
     <hyperlink ref="A659" r:id="rId658"/>
     <hyperlink ref="A660" r:id="rId659"/>
+    <hyperlink ref="A661" r:id="rId660"/>
+    <hyperlink ref="A662" r:id="rId661"/>
+    <hyperlink ref="A663" r:id="rId662"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -19176,7 +19239,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19207,72 +19270,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>1616</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>793</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>1575</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>1617</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46154.83263888889</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1618</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46155.629166666666</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1619</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>424</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1620</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46155.54652777778</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-05-15 13:25
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3322" uniqueCount="1621">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3342" uniqueCount="1629">
   <si>
     <t>link</t>
   </si>
@@ -4881,6 +4881,30 @@
   </si>
   <si>
     <t>62820070018</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/liepnas-pag/bjejde.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/aluksne/glhpx.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/salienas-pag/jdxbj.html</t>
+  </si>
+  <si>
+    <t>Cits</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/laudonas-pag/bcnjo.html</t>
+  </si>
+  <si>
+    <t>49 980 €</t>
+  </si>
+  <si>
+    <t>14.28 ha.</t>
+  </si>
+  <si>
+    <t>70700080094</t>
   </si>
 </sst>
 </file>
@@ -19239,7 +19263,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19270,7 +19294,93 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>1621</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46157.39097222222</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1622</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46156.68680555555</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1623</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1624</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46157.52638888889</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1625</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>1626</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>1627</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1628</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46157.49722222222</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-05-18 14:50
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3342" uniqueCount="1629">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3347" uniqueCount="1630">
   <si>
     <t>link</t>
   </si>
@@ -4905,6 +4905,9 @@
   </si>
   <si>
     <t>70700080094</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/trapenes-pag/cclkbg.html</t>
   </si>
 </sst>
 </file>
@@ -5317,7 +5320,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F663"/>
+  <dimension ref="A1:F667"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18586,6 +18589,86 @@
       </c>
       <c r="F663" s="2">
         <v>46155.54652777778</v>
+      </c>
+    </row>
+    <row r="664" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A664" s="3" t="s">
+        <v>1621</v>
+      </c>
+      <c r="B664" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C664" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D664" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E664" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F664" s="2">
+        <v>46157.39097222222</v>
+      </c>
+    </row>
+    <row r="665" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A665" s="3" t="s">
+        <v>1622</v>
+      </c>
+      <c r="B665" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C665" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D665" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E665" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F665" s="2">
+        <v>46156.68680555555</v>
+      </c>
+    </row>
+    <row r="666" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A666" s="3" t="s">
+        <v>1623</v>
+      </c>
+      <c r="B666" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="C666" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D666" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E666" s="4" t="s">
+        <v>1624</v>
+      </c>
+      <c r="F666" s="2">
+        <v>46157.52638888889</v>
+      </c>
+    </row>
+    <row r="667" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A667" s="3" t="s">
+        <v>1625</v>
+      </c>
+      <c r="B667" s="4" t="s">
+        <v>1626</v>
+      </c>
+      <c r="C667" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D667" s="4" t="s">
+        <v>1627</v>
+      </c>
+      <c r="E667" s="4" t="s">
+        <v>1628</v>
+      </c>
+      <c r="F667" s="2">
+        <v>46157.49722222222</v>
       </c>
     </row>
   </sheetData>
@@ -19252,6 +19335,10 @@
     <hyperlink ref="A661" r:id="rId660"/>
     <hyperlink ref="A662" r:id="rId661"/>
     <hyperlink ref="A663" r:id="rId662"/>
+    <hyperlink ref="A664" r:id="rId663"/>
+    <hyperlink ref="A665" r:id="rId664"/>
+    <hyperlink ref="A666" r:id="rId665"/>
+    <hyperlink ref="A667" r:id="rId666"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -19263,7 +19350,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19296,7 +19383,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1621</v>
+        <v>1629</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>25</v>
@@ -19311,75 +19398,12 @@
         <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46157.39097222222</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1622</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46156.68680555555</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1623</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>274</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1624</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46157.52638888889</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1625</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>1626</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>1627</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1628</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46157.49722222222</v>
+        <v>46160.64583333333</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-05-19 14:31
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3347" uniqueCount="1630">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3362" uniqueCount="1634">
   <si>
     <t>link</t>
   </si>
@@ -4908,6 +4908,18 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/trapenes-pag/cclkbg.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/malienas-pag/bbllho.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/other/adelg.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ogre-and-reg/suntazu-pag/fjcmg.html</t>
+  </si>
+  <si>
+    <t>74880020159</t>
   </si>
 </sst>
 </file>
@@ -5320,7 +5332,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F667"/>
+  <dimension ref="A1:F668"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18669,6 +18681,26 @@
       </c>
       <c r="F667" s="2">
         <v>46157.49722222222</v>
+      </c>
+    </row>
+    <row r="668" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A668" s="3" t="s">
+        <v>1629</v>
+      </c>
+      <c r="B668" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C668" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D668" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E668" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F668" s="2">
+        <v>46160.64583333333</v>
       </c>
     </row>
   </sheetData>
@@ -19339,6 +19371,7 @@
     <hyperlink ref="A665" r:id="rId664"/>
     <hyperlink ref="A666" r:id="rId665"/>
     <hyperlink ref="A667" r:id="rId666"/>
+    <hyperlink ref="A668" r:id="rId667"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -19350,7 +19383,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19383,7 +19416,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1629</v>
+        <v>1630</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>25</v>
@@ -19398,12 +19431,54 @@
         <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46160.64583333333</v>
+        <v>46161.48472222222</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1631</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46160.76875</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1632</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>1192</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1633</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46161.55208333333</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-05-20 14:30
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3362" uniqueCount="1634">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3397" uniqueCount="1646">
   <si>
     <t>link</t>
   </si>
@@ -4920,6 +4920,42 @@
   </si>
   <si>
     <t>74880020159</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/aluksne/cxnopm.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/raiskuma-pag/jepgk.html</t>
+  </si>
+  <si>
+    <t>42740060117</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/zosenu-pag/npieh.html</t>
+  </si>
+  <si>
+    <t>42980030161</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jelgava-and-reg/svetes-pag/hxgbp.html</t>
+  </si>
+  <si>
+    <t>54820030168</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ludza-and-reg/pildas-pag/cgljdh.html</t>
+  </si>
+  <si>
+    <t>68860040128</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ogre-and-reg/mengeles-pag/lilee.html</t>
+  </si>
+  <si>
+    <t>44 800 €</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/tukums-and-reg/irlavas-pag/dpmlb.html</t>
   </si>
 </sst>
 </file>
@@ -5332,7 +5368,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F668"/>
+  <dimension ref="A1:F671"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18701,6 +18737,66 @@
       </c>
       <c r="F668" s="2">
         <v>46160.64583333333</v>
+      </c>
+    </row>
+    <row r="669" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A669" s="3" t="s">
+        <v>1630</v>
+      </c>
+      <c r="B669" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C669" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D669" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E669" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F669" s="2">
+        <v>46161.48472222222</v>
+      </c>
+    </row>
+    <row r="670" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A670" s="3" t="s">
+        <v>1631</v>
+      </c>
+      <c r="B670" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C670" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D670" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E670" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F670" s="2">
+        <v>46160.76875</v>
+      </c>
+    </row>
+    <row r="671" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A671" s="3" t="s">
+        <v>1632</v>
+      </c>
+      <c r="B671" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C671" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="D671" s="4" t="s">
+        <v>1192</v>
+      </c>
+      <c r="E671" s="4" t="s">
+        <v>1633</v>
+      </c>
+      <c r="F671" s="2">
+        <v>46161.55208333333</v>
       </c>
     </row>
   </sheetData>
@@ -19372,6 +19468,9 @@
     <hyperlink ref="A666" r:id="rId665"/>
     <hyperlink ref="A667" r:id="rId666"/>
     <hyperlink ref="A668" r:id="rId667"/>
+    <hyperlink ref="A669" r:id="rId668"/>
+    <hyperlink ref="A670" r:id="rId669"/>
+    <hyperlink ref="A671" r:id="rId670"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -19383,7 +19482,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19416,7 +19515,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1630</v>
+        <v>1634</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>25</v>
@@ -19431,47 +19530,127 @@
         <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46161.48472222222</v>
+        <v>46161.77847222222</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1631</v>
+        <v>1635</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>25</v>
+        <v>106</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>435</v>
+        <v>63</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>25</v>
+        <v>1636</v>
       </c>
       <c r="F3" s="2">
-        <v>46160.76875</v>
+        <v>46162.523611111115</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>1632</v>
+        <v>1637</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>27</v>
+        <v>355</v>
       </c>
       <c r="C4" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1638</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46162.52222222222</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1639</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>745</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1640</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46162.40833333333</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>1641</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>1642</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46161.745833333334</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>1643</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>1644</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>1192</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1633</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46161.55208333333</v>
+      <c r="D7" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>1226</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46161.836805555555</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>1645</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>1584</v>
+      </c>
+      <c r="F8" s="2">
+        <v>46162.39583333333</v>
       </c>
     </row>
   </sheetData>
@@ -19479,6 +19658,10 @@
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
     <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+    <hyperlink ref="A6" r:id="rId5"/>
+    <hyperlink ref="A7" r:id="rId6"/>
+    <hyperlink ref="A8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-05-21 14:35
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3397" uniqueCount="1646">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3432" uniqueCount="1658">
   <si>
     <t>link</t>
   </si>
@@ -4956,6 +4956,42 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/tukums-and-reg/irlavas-pag/dpmlb.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/veclaicenes-pag/bliehn.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/dobele-and-reg/iles-pag/pdloi.html</t>
+  </si>
+  <si>
+    <t>46640030071</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/atasienes-pag/jfgxo.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/kombulu-pag/bhehle.html</t>
+  </si>
+  <si>
+    <t>60740040045</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kuldiga-and-reg/padures-pag/kcoeg.html</t>
+  </si>
+  <si>
+    <t>9.20 ha.</t>
+  </si>
+  <si>
+    <t>62720050126</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/limbadzi-and-reg/salacgrivas-l-t/jllpl.html</t>
+  </si>
+  <si>
+    <t>66720030023</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/luznavas-pag/gfcjn.html</t>
   </si>
 </sst>
 </file>
@@ -5368,7 +5404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F671"/>
+  <dimension ref="A1:F678"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18797,6 +18833,146 @@
       </c>
       <c r="F671" s="2">
         <v>46161.55208333333</v>
+      </c>
+    </row>
+    <row r="672" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A672" s="3" t="s">
+        <v>1634</v>
+      </c>
+      <c r="B672" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C672" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D672" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E672" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F672" s="2">
+        <v>46161.77847222222</v>
+      </c>
+    </row>
+    <row r="673" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A673" s="3" t="s">
+        <v>1635</v>
+      </c>
+      <c r="B673" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C673" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D673" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E673" s="4" t="s">
+        <v>1636</v>
+      </c>
+      <c r="F673" s="2">
+        <v>46162.523611111115</v>
+      </c>
+    </row>
+    <row r="674" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A674" s="3" t="s">
+        <v>1637</v>
+      </c>
+      <c r="B674" s="4" t="s">
+        <v>355</v>
+      </c>
+      <c r="C674" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D674" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E674" s="4" t="s">
+        <v>1638</v>
+      </c>
+      <c r="F674" s="2">
+        <v>46162.52222222222</v>
+      </c>
+    </row>
+    <row r="675" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A675" s="3" t="s">
+        <v>1639</v>
+      </c>
+      <c r="B675" s="4" t="s">
+        <v>745</v>
+      </c>
+      <c r="C675" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="D675" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E675" s="4" t="s">
+        <v>1640</v>
+      </c>
+      <c r="F675" s="2">
+        <v>46162.40833333333</v>
+      </c>
+    </row>
+    <row r="676" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A676" s="3" t="s">
+        <v>1641</v>
+      </c>
+      <c r="B676" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C676" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D676" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E676" s="4" t="s">
+        <v>1642</v>
+      </c>
+      <c r="F676" s="2">
+        <v>46161.745833333334</v>
+      </c>
+    </row>
+    <row r="677" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A677" s="3" t="s">
+        <v>1643</v>
+      </c>
+      <c r="B677" s="4" t="s">
+        <v>1644</v>
+      </c>
+      <c r="C677" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="D677" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="E677" s="4" t="s">
+        <v>1226</v>
+      </c>
+      <c r="F677" s="2">
+        <v>46161.836805555555</v>
+      </c>
+    </row>
+    <row r="678" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A678" s="3" t="s">
+        <v>1645</v>
+      </c>
+      <c r="B678" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C678" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D678" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E678" s="4" t="s">
+        <v>1584</v>
+      </c>
+      <c r="F678" s="2">
+        <v>46162.39583333333</v>
       </c>
     </row>
   </sheetData>
@@ -19471,6 +19647,13 @@
     <hyperlink ref="A669" r:id="rId668"/>
     <hyperlink ref="A670" r:id="rId669"/>
     <hyperlink ref="A671" r:id="rId670"/>
+    <hyperlink ref="A672" r:id="rId671"/>
+    <hyperlink ref="A673" r:id="rId672"/>
+    <hyperlink ref="A674" r:id="rId673"/>
+    <hyperlink ref="A675" r:id="rId674"/>
+    <hyperlink ref="A676" r:id="rId675"/>
+    <hyperlink ref="A677" r:id="rId676"/>
+    <hyperlink ref="A678" r:id="rId677"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -19515,7 +19698,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1634</v>
+        <v>1646</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>25</v>
@@ -19530,127 +19713,127 @@
         <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46161.77847222222</v>
+        <v>46162.884722222225</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1635</v>
+        <v>1647</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>106</v>
+        <v>131</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>63</v>
+        <v>117</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>17</v>
+        <v>272</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1636</v>
+        <v>1648</v>
       </c>
       <c r="F3" s="2">
-        <v>46162.523611111115</v>
+        <v>46163.680555555555</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>1637</v>
+        <v>1649</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>355</v>
+        <v>760</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>63</v>
+        <v>127</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>13</v>
+        <v>186</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>1638</v>
+        <v>1389</v>
       </c>
       <c r="F4" s="2">
-        <v>46162.52222222222</v>
+        <v>46163.45625</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>1639</v>
+        <v>1650</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>745</v>
+        <v>268</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>518</v>
+        <v>146</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>75</v>
+        <v>162</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>1640</v>
+        <v>1651</v>
       </c>
       <c r="F5" s="2">
-        <v>46162.40833333333</v>
+        <v>46163.509722222225</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>1641</v>
+        <v>1652</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>39</v>
+        <v>106</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>234</v>
+        <v>424</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>82</v>
+        <v>1653</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>1642</v>
+        <v>1654</v>
       </c>
       <c r="F6" s="2">
-        <v>46161.745833333334</v>
+        <v>46163.396527777775</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>1643</v>
+        <v>1655</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>1644</v>
+        <v>39</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>275</v>
+        <v>208</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>194</v>
+        <v>1011</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>1226</v>
+        <v>1656</v>
       </c>
       <c r="F7" s="2">
-        <v>46161.836805555555</v>
+        <v>46163.430555555555</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>1645</v>
+        <v>1657</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>52</v>
+        <v>707</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>376</v>
+        <v>294</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>272</v>
+        <v>36</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>1584</v>
+        <v>25</v>
       </c>
       <c r="F8" s="2">
-        <v>46162.39583333333</v>
+        <v>46163.410416666666</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-05-22 14:10
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3432" uniqueCount="1658">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3442" uniqueCount="1662">
   <si>
     <t>link</t>
   </si>
@@ -4992,6 +4992,18 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/luznavas-pag/gfcjn.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/gulbene-and-reg/belavas-pag/beihoh.html</t>
+  </si>
+  <si>
+    <t>50440030032</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/andrupenes-pag/ohije.html</t>
+  </si>
+  <si>
+    <t>60420110092</t>
   </si>
 </sst>
 </file>
@@ -5404,7 +5416,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F678"/>
+  <dimension ref="A1:F685"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -18973,6 +18985,146 @@
       </c>
       <c r="F678" s="2">
         <v>46162.39583333333</v>
+      </c>
+    </row>
+    <row r="679" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A679" s="3" t="s">
+        <v>1646</v>
+      </c>
+      <c r="B679" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C679" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D679" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E679" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F679" s="2">
+        <v>46162.884722222225</v>
+      </c>
+    </row>
+    <row r="680" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A680" s="3" t="s">
+        <v>1647</v>
+      </c>
+      <c r="B680" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C680" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D680" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E680" s="4" t="s">
+        <v>1648</v>
+      </c>
+      <c r="F680" s="2">
+        <v>46163.680555555555</v>
+      </c>
+    </row>
+    <row r="681" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A681" s="3" t="s">
+        <v>1649</v>
+      </c>
+      <c r="B681" s="4" t="s">
+        <v>760</v>
+      </c>
+      <c r="C681" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D681" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E681" s="4" t="s">
+        <v>1389</v>
+      </c>
+      <c r="F681" s="2">
+        <v>46163.45625</v>
+      </c>
+    </row>
+    <row r="682" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A682" s="3" t="s">
+        <v>1650</v>
+      </c>
+      <c r="B682" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="C682" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D682" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="E682" s="4" t="s">
+        <v>1651</v>
+      </c>
+      <c r="F682" s="2">
+        <v>46163.509722222225</v>
+      </c>
+    </row>
+    <row r="683" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A683" s="3" t="s">
+        <v>1652</v>
+      </c>
+      <c r="B683" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C683" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="D683" s="4" t="s">
+        <v>1653</v>
+      </c>
+      <c r="E683" s="4" t="s">
+        <v>1654</v>
+      </c>
+      <c r="F683" s="2">
+        <v>46163.396527777775</v>
+      </c>
+    </row>
+    <row r="684" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A684" s="3" t="s">
+        <v>1655</v>
+      </c>
+      <c r="B684" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C684" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D684" s="4" t="s">
+        <v>1011</v>
+      </c>
+      <c r="E684" s="4" t="s">
+        <v>1656</v>
+      </c>
+      <c r="F684" s="2">
+        <v>46163.430555555555</v>
+      </c>
+    </row>
+    <row r="685" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A685" s="3" t="s">
+        <v>1657</v>
+      </c>
+      <c r="B685" s="4" t="s">
+        <v>707</v>
+      </c>
+      <c r="C685" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D685" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E685" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F685" s="2">
+        <v>46163.410416666666</v>
       </c>
     </row>
   </sheetData>
@@ -19654,6 +19806,13 @@
     <hyperlink ref="A676" r:id="rId675"/>
     <hyperlink ref="A677" r:id="rId676"/>
     <hyperlink ref="A678" r:id="rId677"/>
+    <hyperlink ref="A679" r:id="rId678"/>
+    <hyperlink ref="A680" r:id="rId679"/>
+    <hyperlink ref="A681" r:id="rId680"/>
+    <hyperlink ref="A682" r:id="rId681"/>
+    <hyperlink ref="A683" r:id="rId682"/>
+    <hyperlink ref="A684" r:id="rId683"/>
+    <hyperlink ref="A685" r:id="rId684"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -19665,7 +19824,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19698,153 +19857,48 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1646</v>
+        <v>1658</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>25</v>
+        <v>106</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>435</v>
+        <v>124</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>25</v>
+        <v>959</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>25</v>
+        <v>1659</v>
       </c>
       <c r="F2" s="2">
-        <v>46162.884722222225</v>
+        <v>46163.75069444445</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1647</v>
+        <v>1660</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>131</v>
+        <v>576</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>117</v>
+        <v>146</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>272</v>
+        <v>186</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1648</v>
+        <v>1661</v>
       </c>
       <c r="F3" s="2">
-        <v>46163.680555555555</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1649</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>760</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1389</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46163.45625</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1650</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>268</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1651</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46163.509722222225</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>1652</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>424</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>1653</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>1654</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46163.396527777775</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>1655</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>1011</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>1656</v>
-      </c>
-      <c r="F7" s="2">
-        <v>46163.430555555555</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>1657</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>707</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F8" s="2">
-        <v>46163.410416666666</v>
+        <v>46164.652083333334</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A6" r:id="rId5"/>
-    <hyperlink ref="A7" r:id="rId6"/>
-    <hyperlink ref="A8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-05-25 14:29
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3442" uniqueCount="1662">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3467" uniqueCount="1670">
   <si>
     <t>link</t>
   </si>
@@ -5004,6 +5004,30 @@
   </si>
   <si>
     <t>60420110092</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/alsviku-pag/bdbfho.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/jekabpils/mfiph.html</t>
+  </si>
+  <si>
+    <t>56700060231</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/andrupenes-pag/fnfdx.html</t>
+  </si>
+  <si>
+    <t>60420050064</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ogre-and-reg/jumpravas-pag/hlnfm.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/talsi-and-reg/other/excgd.html</t>
+  </si>
+  <si>
+    <t>88940050350</t>
   </si>
 </sst>
 </file>
@@ -5416,7 +5440,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F685"/>
+  <dimension ref="A1:F687"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19125,6 +19149,46 @@
       </c>
       <c r="F685" s="2">
         <v>46163.410416666666</v>
+      </c>
+    </row>
+    <row r="686" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A686" s="3" t="s">
+        <v>1658</v>
+      </c>
+      <c r="B686" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C686" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D686" s="4" t="s">
+        <v>959</v>
+      </c>
+      <c r="E686" s="4" t="s">
+        <v>1659</v>
+      </c>
+      <c r="F686" s="2">
+        <v>46163.75069444445</v>
+      </c>
+    </row>
+    <row r="687" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A687" s="3" t="s">
+        <v>1660</v>
+      </c>
+      <c r="B687" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="C687" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D687" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E687" s="4" t="s">
+        <v>1661</v>
+      </c>
+      <c r="F687" s="2">
+        <v>46164.652083333334</v>
       </c>
     </row>
   </sheetData>
@@ -19813,6 +19877,8 @@
     <hyperlink ref="A683" r:id="rId682"/>
     <hyperlink ref="A684" r:id="rId683"/>
     <hyperlink ref="A685" r:id="rId684"/>
+    <hyperlink ref="A686" r:id="rId685"/>
+    <hyperlink ref="A687" r:id="rId686"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -19824,7 +19890,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19857,48 +19923,111 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1658</v>
+        <v>1662</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>106</v>
+        <v>25</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>124</v>
+        <v>435</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>959</v>
+        <v>25</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1659</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46163.75069444445</v>
+        <v>46166.36875</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1660</v>
+        <v>1663</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1664</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46166.8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1665</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1666</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46167.39375</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1667</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>1417</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46166.38680555555</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>1668</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>576</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1661</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46164.652083333334</v>
+      <c r="C6" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>1076</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>1669</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46167.37013888889</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+    <hyperlink ref="A6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-05-26 14:32
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3467" uniqueCount="1670">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3477" uniqueCount="1677">
   <si>
     <t>link</t>
   </si>
@@ -5028,6 +5028,27 @@
   </si>
   <si>
     <t>88940050350</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/viksnas-pag/ledpl.html</t>
+  </si>
+  <si>
+    <t>64 000 €</t>
+  </si>
+  <si>
+    <t>14.90 ha.</t>
+  </si>
+  <si>
+    <t>38580080142</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/sventes-pag/bcciie.html</t>
+  </si>
+  <si>
+    <t>15 €</t>
+  </si>
+  <si>
+    <t>44880010114</t>
   </si>
 </sst>
 </file>
@@ -5440,7 +5461,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F687"/>
+  <dimension ref="A1:F692"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19189,6 +19210,106 @@
       </c>
       <c r="F687" s="2">
         <v>46164.652083333334</v>
+      </c>
+    </row>
+    <row r="688" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A688" s="3" t="s">
+        <v>1662</v>
+      </c>
+      <c r="B688" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C688" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D688" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E688" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F688" s="2">
+        <v>46166.36875</v>
+      </c>
+    </row>
+    <row r="689" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A689" s="3" t="s">
+        <v>1663</v>
+      </c>
+      <c r="B689" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C689" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D689" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E689" s="4" t="s">
+        <v>1664</v>
+      </c>
+      <c r="F689" s="2">
+        <v>46166.8</v>
+      </c>
+    </row>
+    <row r="690" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A690" s="3" t="s">
+        <v>1665</v>
+      </c>
+      <c r="B690" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="C690" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D690" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E690" s="4" t="s">
+        <v>1666</v>
+      </c>
+      <c r="F690" s="2">
+        <v>46167.39375</v>
+      </c>
+    </row>
+    <row r="691" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A691" s="3" t="s">
+        <v>1667</v>
+      </c>
+      <c r="B691" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C691" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="D691" s="4" t="s">
+        <v>1417</v>
+      </c>
+      <c r="E691" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F691" s="2">
+        <v>46166.38680555555</v>
+      </c>
+    </row>
+    <row r="692" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A692" s="3" t="s">
+        <v>1668</v>
+      </c>
+      <c r="B692" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="C692" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="D692" s="4" t="s">
+        <v>1076</v>
+      </c>
+      <c r="E692" s="4" t="s">
+        <v>1669</v>
+      </c>
+      <c r="F692" s="2">
+        <v>46167.37013888889</v>
       </c>
     </row>
   </sheetData>
@@ -19879,6 +20000,11 @@
     <hyperlink ref="A685" r:id="rId684"/>
     <hyperlink ref="A686" r:id="rId685"/>
     <hyperlink ref="A687" r:id="rId686"/>
+    <hyperlink ref="A688" r:id="rId687"/>
+    <hyperlink ref="A689" r:id="rId688"/>
+    <hyperlink ref="A690" r:id="rId689"/>
+    <hyperlink ref="A691" r:id="rId690"/>
+    <hyperlink ref="A692" r:id="rId691"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -19890,7 +20016,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19923,111 +20049,48 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1662</v>
+        <v>1670</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>25</v>
+        <v>1671</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>435</v>
+        <v>28</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>25</v>
+        <v>1672</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>25</v>
+        <v>1673</v>
       </c>
       <c r="F2" s="2">
-        <v>46166.36875</v>
+        <v>46168.71041666667</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1663</v>
+        <v>1674</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>23</v>
+        <v>1675</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>127</v>
+        <v>74</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>85</v>
+        <v>36</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1664</v>
+        <v>1676</v>
       </c>
       <c r="F3" s="2">
-        <v>46166.8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1665</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>274</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1666</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46167.39375</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1667</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>275</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>1417</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46166.38680555555</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>1668</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>576</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>356</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>1076</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>1669</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46167.37013888889</v>
+        <v>46167.90069444444</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-05-27 14:51
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -5461,7 +5461,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F692"/>
+  <dimension ref="A1:F694"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19310,6 +19310,46 @@
       </c>
       <c r="F692" s="2">
         <v>46167.37013888889</v>
+      </c>
+    </row>
+    <row r="693" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A693" s="3" t="s">
+        <v>1670</v>
+      </c>
+      <c r="B693" s="4" t="s">
+        <v>1671</v>
+      </c>
+      <c r="C693" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D693" s="4" t="s">
+        <v>1672</v>
+      </c>
+      <c r="E693" s="4" t="s">
+        <v>1673</v>
+      </c>
+      <c r="F693" s="2">
+        <v>46168.71041666667</v>
+      </c>
+    </row>
+    <row r="694" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A694" s="3" t="s">
+        <v>1674</v>
+      </c>
+      <c r="B694" s="4" t="s">
+        <v>1675</v>
+      </c>
+      <c r="C694" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D694" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E694" s="4" t="s">
+        <v>1676</v>
+      </c>
+      <c r="F694" s="2">
+        <v>46167.90069444444</v>
       </c>
     </row>
   </sheetData>
@@ -20005,6 +20045,8 @@
     <hyperlink ref="A690" r:id="rId689"/>
     <hyperlink ref="A691" r:id="rId690"/>
     <hyperlink ref="A692" r:id="rId691"/>
+    <hyperlink ref="A693" r:id="rId692"/>
+    <hyperlink ref="A694" r:id="rId693"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -20016,7 +20058,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -20047,51 +20089,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>1670</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>1671</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>1672</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>1673</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46168.71041666667</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1674</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>1675</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1676</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46167.90069444444</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-05-28 15:00
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3477" uniqueCount="1677">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3487" uniqueCount="1682">
   <si>
     <t>link</t>
   </si>
@@ -5049,6 +5049,21 @@
   </si>
   <si>
     <t>44880010114</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/stalbes-pag/hhllx.html</t>
+  </si>
+  <si>
+    <t>42800050175</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/sokolku-pag/mkecl.html</t>
+  </si>
+  <si>
+    <t>5.90 ha.</t>
+  </si>
+  <si>
+    <t>78900030029</t>
   </si>
 </sst>
 </file>
@@ -20058,7 +20073,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -20089,7 +20104,51 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>1677</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>1014</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>1678</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46170.48611111111</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1679</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>1680</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1681</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46170.52638888889</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-05-29 14:34
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3487" uniqueCount="1682">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3497" uniqueCount="1684">
   <si>
     <t>link</t>
   </si>
@@ -5064,6 +5064,12 @@
   </si>
   <si>
     <t>78900030029</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/jaunlaicenes-pag/bdilcj.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/jaunaluksnes-pag/blimkd.html</t>
   </si>
 </sst>
 </file>
@@ -5476,7 +5482,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F694"/>
+  <dimension ref="A1:F696"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19365,6 +19371,46 @@
       </c>
       <c r="F694" s="2">
         <v>46167.90069444444</v>
+      </c>
+    </row>
+    <row r="695" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A695" s="3" t="s">
+        <v>1677</v>
+      </c>
+      <c r="B695" s="4" t="s">
+        <v>1014</v>
+      </c>
+      <c r="C695" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D695" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E695" s="4" t="s">
+        <v>1678</v>
+      </c>
+      <c r="F695" s="2">
+        <v>46170.48611111111</v>
+      </c>
+    </row>
+    <row r="696" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A696" s="3" t="s">
+        <v>1679</v>
+      </c>
+      <c r="B696" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C696" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D696" s="4" t="s">
+        <v>1680</v>
+      </c>
+      <c r="E696" s="4" t="s">
+        <v>1681</v>
+      </c>
+      <c r="F696" s="2">
+        <v>46170.52638888889</v>
       </c>
     </row>
   </sheetData>
@@ -20062,6 +20108,8 @@
     <hyperlink ref="A692" r:id="rId691"/>
     <hyperlink ref="A693" r:id="rId692"/>
     <hyperlink ref="A694" r:id="rId693"/>
+    <hyperlink ref="A695" r:id="rId694"/>
+    <hyperlink ref="A696" r:id="rId695"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -20106,42 +20154,42 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1677</v>
+        <v>1682</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1014</v>
+        <v>25</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>63</v>
+        <v>435</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>103</v>
+        <v>25</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1678</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46170.48611111111</v>
+        <v>46171.356944444444</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1679</v>
+        <v>1683</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>88</v>
+        <v>25</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>294</v>
+        <v>435</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>1680</v>
+        <v>25</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1681</v>
+        <v>25</v>
       </c>
       <c r="F3" s="2">
-        <v>46170.52638888889</v>
+        <v>46171.17291666666</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-06-01 17:14
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3497" uniqueCount="1684">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3537" uniqueCount="1695">
   <si>
     <t>link</t>
   </si>
@@ -5070,6 +5070,39 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/jaunaluksnes-pag/blimkd.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/ziemera-pag/bhofjb.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/gaujienas-pag/bbokek.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/aluksne/mgokl.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/liepnas-pag/bbokfb.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/aluksne/moxfk.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/gulbene-and-reg/lejasciema-pag/bxkihm.html</t>
+  </si>
+  <si>
+    <t>1.26 ha.</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valmiera-and-reg/vaidavas-pag/dkljg.html</t>
+  </si>
+  <si>
+    <t>96880020142</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valmiera-and-reg/lodes-pag/hpidh.html</t>
+  </si>
+  <si>
+    <t>96680020029</t>
   </si>
 </sst>
 </file>
@@ -5482,7 +5515,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F696"/>
+  <dimension ref="A1:F698"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19411,6 +19444,46 @@
       </c>
       <c r="F696" s="2">
         <v>46170.52638888889</v>
+      </c>
+    </row>
+    <row r="697" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A697" s="3" t="s">
+        <v>1682</v>
+      </c>
+      <c r="B697" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C697" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D697" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E697" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F697" s="2">
+        <v>46171.356944444444</v>
+      </c>
+    </row>
+    <row r="698" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A698" s="3" t="s">
+        <v>1683</v>
+      </c>
+      <c r="B698" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C698" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D698" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E698" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F698" s="2">
+        <v>46171.17291666666</v>
       </c>
     </row>
   </sheetData>
@@ -20110,6 +20183,8 @@
     <hyperlink ref="A694" r:id="rId693"/>
     <hyperlink ref="A695" r:id="rId694"/>
     <hyperlink ref="A696" r:id="rId695"/>
+    <hyperlink ref="A697" r:id="rId696"/>
+    <hyperlink ref="A698" r:id="rId697"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -20121,7 +20196,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -20154,7 +20229,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1682</v>
+        <v>1684</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>25</v>
@@ -20169,12 +20244,12 @@
         <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46171.356944444444</v>
+        <v>46174.42847222222</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1683</v>
+        <v>1685</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>25</v>
@@ -20183,19 +20258,145 @@
         <v>435</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>25</v>
+        <v>272</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>25</v>
       </c>
       <c r="F3" s="2">
-        <v>46171.17291666666</v>
+        <v>46174.41666666667</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1686</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46174.39166666666</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1687</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46173.89097222222</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>1688</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46172.80625</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>1689</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>1690</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46172.44930555555</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>1691</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>816</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>1692</v>
+      </c>
+      <c r="F8" s="2">
+        <v>46174.52847222222</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>1693</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>1694</v>
+      </c>
+      <c r="F9" s="2">
+        <v>46174.325</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+    <hyperlink ref="A6" r:id="rId5"/>
+    <hyperlink ref="A7" r:id="rId6"/>
+    <hyperlink ref="A8" r:id="rId7"/>
+    <hyperlink ref="A9" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-06-02 15:54
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3537" uniqueCount="1695">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3547" uniqueCount="1699">
   <si>
     <t>link</t>
   </si>
@@ -5103,6 +5103,18 @@
   </si>
   <si>
     <t>96680020029</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/other/bfoin.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kuldiga-and-reg/nikraces-pag/elnmj.html</t>
+  </si>
+  <si>
+    <t>32 395 €</t>
+  </si>
+  <si>
+    <t>62680060060</t>
   </si>
 </sst>
 </file>
@@ -5515,7 +5527,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F698"/>
+  <dimension ref="A1:F706"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19484,6 +19496,166 @@
       </c>
       <c r="F698" s="2">
         <v>46171.17291666666</v>
+      </c>
+    </row>
+    <row r="699" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A699" s="3" t="s">
+        <v>1684</v>
+      </c>
+      <c r="B699" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C699" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D699" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E699" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F699" s="2">
+        <v>46174.42847222222</v>
+      </c>
+    </row>
+    <row r="700" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A700" s="3" t="s">
+        <v>1685</v>
+      </c>
+      <c r="B700" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C700" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D700" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E700" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F700" s="2">
+        <v>46174.41666666667</v>
+      </c>
+    </row>
+    <row r="701" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A701" s="3" t="s">
+        <v>1686</v>
+      </c>
+      <c r="B701" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C701" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D701" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E701" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F701" s="2">
+        <v>46174.39166666666</v>
+      </c>
+    </row>
+    <row r="702" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A702" s="3" t="s">
+        <v>1687</v>
+      </c>
+      <c r="B702" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C702" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D702" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E702" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F702" s="2">
+        <v>46173.89097222222</v>
+      </c>
+    </row>
+    <row r="703" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A703" s="3" t="s">
+        <v>1688</v>
+      </c>
+      <c r="B703" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C703" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D703" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E703" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F703" s="2">
+        <v>46172.80625</v>
+      </c>
+    </row>
+    <row r="704" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A704" s="3" t="s">
+        <v>1689</v>
+      </c>
+      <c r="B704" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C704" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D704" s="4" t="s">
+        <v>1690</v>
+      </c>
+      <c r="E704" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F704" s="2">
+        <v>46172.44930555555</v>
+      </c>
+    </row>
+    <row r="705" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A705" s="3" t="s">
+        <v>1691</v>
+      </c>
+      <c r="B705" s="4" t="s">
+        <v>816</v>
+      </c>
+      <c r="C705" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D705" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E705" s="4" t="s">
+        <v>1692</v>
+      </c>
+      <c r="F705" s="2">
+        <v>46174.52847222222</v>
+      </c>
+    </row>
+    <row r="706" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A706" s="3" t="s">
+        <v>1693</v>
+      </c>
+      <c r="B706" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C706" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D706" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E706" s="4" t="s">
+        <v>1694</v>
+      </c>
+      <c r="F706" s="2">
+        <v>46174.325</v>
       </c>
     </row>
   </sheetData>
@@ -20185,6 +20357,14 @@
     <hyperlink ref="A696" r:id="rId695"/>
     <hyperlink ref="A697" r:id="rId696"/>
     <hyperlink ref="A698" r:id="rId697"/>
+    <hyperlink ref="A699" r:id="rId698"/>
+    <hyperlink ref="A700" r:id="rId699"/>
+    <hyperlink ref="A701" r:id="rId700"/>
+    <hyperlink ref="A702" r:id="rId701"/>
+    <hyperlink ref="A703" r:id="rId702"/>
+    <hyperlink ref="A704" r:id="rId703"/>
+    <hyperlink ref="A705" r:id="rId704"/>
+    <hyperlink ref="A706" r:id="rId705"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -20196,7 +20376,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -20229,7 +20409,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1684</v>
+        <v>1695</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>25</v>
@@ -20238,165 +20418,39 @@
         <v>435</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>25</v>
+        <v>162</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46174.42847222222</v>
+        <v>46175.71319444444</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1685</v>
+        <v>1696</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>25</v>
+        <v>1697</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>435</v>
+        <v>424</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>272</v>
+        <v>205</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>25</v>
+        <v>1698</v>
       </c>
       <c r="F3" s="2">
-        <v>46174.41666666667</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1686</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46174.39166666666</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1687</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46173.89097222222</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>1688</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46172.80625</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>1689</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>1690</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F7" s="2">
-        <v>46172.44930555555</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>1691</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>816</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>1692</v>
-      </c>
-      <c r="F8" s="2">
-        <v>46174.52847222222</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>1693</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>1694</v>
-      </c>
-      <c r="F9" s="2">
-        <v>46174.325</v>
+        <v>46175.441666666666</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A6" r:id="rId5"/>
-    <hyperlink ref="A7" r:id="rId6"/>
-    <hyperlink ref="A8" r:id="rId7"/>
-    <hyperlink ref="A9" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-06-03 16:12
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3547" uniqueCount="1699">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3557" uniqueCount="1702">
   <si>
     <t>link</t>
   </si>
@@ -5115,6 +5115,15 @@
   </si>
   <si>
     <t>62680060060</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/aluksne/cxngoc.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valmiera-and-reg/ramatas-pag/fxkkn.html</t>
+  </si>
+  <si>
+    <t>96760040158</t>
   </si>
 </sst>
 </file>
@@ -5527,7 +5536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F706"/>
+  <dimension ref="A1:F708"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19656,6 +19665,46 @@
       </c>
       <c r="F706" s="2">
         <v>46174.325</v>
+      </c>
+    </row>
+    <row r="707" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A707" s="3" t="s">
+        <v>1695</v>
+      </c>
+      <c r="B707" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C707" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D707" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="E707" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F707" s="2">
+        <v>46175.71319444444</v>
+      </c>
+    </row>
+    <row r="708" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A708" s="3" t="s">
+        <v>1696</v>
+      </c>
+      <c r="B708" s="4" t="s">
+        <v>1697</v>
+      </c>
+      <c r="C708" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="D708" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="E708" s="4" t="s">
+        <v>1698</v>
+      </c>
+      <c r="F708" s="2">
+        <v>46175.441666666666</v>
       </c>
     </row>
   </sheetData>
@@ -20365,6 +20414,8 @@
     <hyperlink ref="A704" r:id="rId703"/>
     <hyperlink ref="A705" r:id="rId704"/>
     <hyperlink ref="A706" r:id="rId705"/>
+    <hyperlink ref="A707" r:id="rId706"/>
+    <hyperlink ref="A708" r:id="rId707"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -20409,7 +20460,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1695</v>
+        <v>1699</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>25</v>
@@ -20418,33 +20469,33 @@
         <v>435</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>162</v>
+        <v>25</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46175.71319444444</v>
+        <v>46175.81319444445</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1696</v>
+        <v>1700</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>1697</v>
+        <v>91</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>424</v>
+        <v>396</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>205</v>
+        <v>514</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1698</v>
+        <v>1701</v>
       </c>
       <c r="F3" s="2">
-        <v>46175.441666666666</v>
+        <v>46176.65416666667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-06-04 14:28
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3557" uniqueCount="1702">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3562" uniqueCount="1705">
   <si>
     <t>link</t>
   </si>
@@ -5124,6 +5124,15 @@
   </si>
   <si>
     <t>96760040158</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/stolerovas-pag/nghhi.html</t>
+  </si>
+  <si>
+    <t>4.82 ha.</t>
+  </si>
+  <si>
+    <t>78920030195</t>
   </si>
 </sst>
 </file>
@@ -5536,7 +5545,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F708"/>
+  <dimension ref="A1:F710"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19705,6 +19714,46 @@
       </c>
       <c r="F708" s="2">
         <v>46175.441666666666</v>
+      </c>
+    </row>
+    <row r="709" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A709" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="B709" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C709" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D709" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E709" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F709" s="2">
+        <v>46175.81319444445</v>
+      </c>
+    </row>
+    <row r="710" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A710" s="3" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B710" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C710" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D710" s="4" t="s">
+        <v>514</v>
+      </c>
+      <c r="E710" s="4" t="s">
+        <v>1701</v>
+      </c>
+      <c r="F710" s="2">
+        <v>46176.65416666667</v>
       </c>
     </row>
   </sheetData>
@@ -20416,6 +20465,8 @@
     <hyperlink ref="A706" r:id="rId705"/>
     <hyperlink ref="A707" r:id="rId706"/>
     <hyperlink ref="A708" r:id="rId707"/>
+    <hyperlink ref="A709" r:id="rId708"/>
+    <hyperlink ref="A710" r:id="rId709"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -20427,7 +20478,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -20460,48 +20511,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1699</v>
+        <v>1702</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>435</v>
+        <v>294</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>25</v>
+        <v>1703</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>25</v>
+        <v>1704</v>
       </c>
       <c r="F2" s="2">
-        <v>46175.81319444445</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1700</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>514</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1701</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46176.65416666667</v>
+        <v>46177.7125</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-06-05 14:19
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3562" uniqueCount="1705">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3572" uniqueCount="1708">
   <si>
     <t>link</t>
   </si>
@@ -5133,6 +5133,15 @@
   </si>
   <si>
     <t>78920030195</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/gaujienas-pag/bihxex.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/gulbene-and-reg/belavas-pag/befldp.html</t>
+  </si>
+  <si>
+    <t>50440060039</t>
   </si>
 </sst>
 </file>
@@ -5545,7 +5554,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F710"/>
+  <dimension ref="A1:F711"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19754,6 +19763,26 @@
       </c>
       <c r="F710" s="2">
         <v>46176.65416666667</v>
+      </c>
+    </row>
+    <row r="711" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A711" s="3" t="s">
+        <v>1702</v>
+      </c>
+      <c r="B711" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C711" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D711" s="4" t="s">
+        <v>1703</v>
+      </c>
+      <c r="E711" s="4" t="s">
+        <v>1704</v>
+      </c>
+      <c r="F711" s="2">
+        <v>46177.7125</v>
       </c>
     </row>
   </sheetData>
@@ -20467,6 +20496,7 @@
     <hyperlink ref="A708" r:id="rId707"/>
     <hyperlink ref="A709" r:id="rId708"/>
     <hyperlink ref="A710" r:id="rId709"/>
+    <hyperlink ref="A711" r:id="rId710"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -20478,7 +20508,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -20511,27 +20541,48 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1702</v>
+        <v>1705</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>294</v>
+        <v>435</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>1703</v>
+        <v>25</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1704</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46177.7125</v>
+        <v>46178.21527777778</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1706</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>781</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1707</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46177.93194444444</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-06-08 15:23
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3572" uniqueCount="1708">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3597" uniqueCount="1722">
   <si>
     <t>link</t>
   </si>
@@ -5142,6 +5142,48 @@
   </si>
   <si>
     <t>50440060039</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/apes-l-t/jcojl.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/liepas-pag/mhixj.html</t>
+  </si>
+  <si>
+    <t>88 000 €</t>
+  </si>
+  <si>
+    <t>42600010133</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/vestienas-pag/deckf.html</t>
+  </si>
+  <si>
+    <t>16.90 ha.</t>
+  </si>
+  <si>
+    <t>70960090113</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/cornajas-pag/kcbef.html</t>
+  </si>
+  <si>
+    <t>9 750 €</t>
+  </si>
+  <si>
+    <t>1.24 ha.</t>
+  </si>
+  <si>
+    <t>78460040381</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/talsi-and-reg/virbu-pag/bhoppi.html</t>
+  </si>
+  <si>
+    <t>113 500 €</t>
+  </si>
+  <si>
+    <t>88960010042</t>
   </si>
 </sst>
 </file>
@@ -5554,7 +5596,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F711"/>
+  <dimension ref="A1:F713"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19783,6 +19825,46 @@
       </c>
       <c r="F711" s="2">
         <v>46177.7125</v>
+      </c>
+    </row>
+    <row r="712" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A712" s="3" t="s">
+        <v>1705</v>
+      </c>
+      <c r="B712" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C712" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D712" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E712" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F712" s="2">
+        <v>46178.21527777778</v>
+      </c>
+    </row>
+    <row r="713" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A713" s="3" t="s">
+        <v>1706</v>
+      </c>
+      <c r="B713" s="4" t="s">
+        <v>781</v>
+      </c>
+      <c r="C713" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D713" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="E713" s="4" t="s">
+        <v>1707</v>
+      </c>
+      <c r="F713" s="2">
+        <v>46177.93194444444</v>
       </c>
     </row>
   </sheetData>
@@ -20497,6 +20579,8 @@
     <hyperlink ref="A709" r:id="rId708"/>
     <hyperlink ref="A710" r:id="rId709"/>
     <hyperlink ref="A711" r:id="rId710"/>
+    <hyperlink ref="A712" r:id="rId711"/>
+    <hyperlink ref="A713" r:id="rId712"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -20508,7 +20592,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -20541,7 +20625,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1705</v>
+        <v>1708</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>25</v>
@@ -20556,33 +20640,96 @@
         <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46178.21527777778</v>
+        <v>46181.49166666667</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1706</v>
+        <v>1709</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>781</v>
+        <v>1710</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>124</v>
+        <v>63</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>154</v>
+        <v>75</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1707</v>
+        <v>1711</v>
       </c>
       <c r="F3" s="2">
-        <v>46177.93194444444</v>
+        <v>46179.93958333333</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1712</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>1713</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1714</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46181.41458333333</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1715</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>1716</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>1717</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1718</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46181.45625</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>1719</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>1720</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>903</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>1721</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46178.75</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+    <hyperlink ref="A6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-06-09 14:15
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3597" uniqueCount="1722">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3602" uniqueCount="1724">
   <si>
     <t>link</t>
   </si>
@@ -5184,6 +5184,12 @@
   </si>
   <si>
     <t>88960010042</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/gaujienas-pag/lhchl.html</t>
+  </si>
+  <si>
+    <t>55 200 €</t>
   </si>
 </sst>
 </file>
@@ -5596,7 +5602,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F713"/>
+  <dimension ref="A1:F718"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19865,6 +19871,106 @@
       </c>
       <c r="F713" s="2">
         <v>46177.93194444444</v>
+      </c>
+    </row>
+    <row r="714" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A714" s="3" t="s">
+        <v>1708</v>
+      </c>
+      <c r="B714" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C714" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D714" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E714" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F714" s="2">
+        <v>46181.49166666667</v>
+      </c>
+    </row>
+    <row r="715" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A715" s="3" t="s">
+        <v>1709</v>
+      </c>
+      <c r="B715" s="4" t="s">
+        <v>1710</v>
+      </c>
+      <c r="C715" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D715" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E715" s="4" t="s">
+        <v>1711</v>
+      </c>
+      <c r="F715" s="2">
+        <v>46179.93958333333</v>
+      </c>
+    </row>
+    <row r="716" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A716" s="3" t="s">
+        <v>1712</v>
+      </c>
+      <c r="B716" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C716" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D716" s="4" t="s">
+        <v>1713</v>
+      </c>
+      <c r="E716" s="4" t="s">
+        <v>1714</v>
+      </c>
+      <c r="F716" s="2">
+        <v>46181.41458333333</v>
+      </c>
+    </row>
+    <row r="717" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A717" s="3" t="s">
+        <v>1715</v>
+      </c>
+      <c r="B717" s="4" t="s">
+        <v>1716</v>
+      </c>
+      <c r="C717" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D717" s="4" t="s">
+        <v>1717</v>
+      </c>
+      <c r="E717" s="4" t="s">
+        <v>1718</v>
+      </c>
+      <c r="F717" s="2">
+        <v>46181.45625</v>
+      </c>
+    </row>
+    <row r="718" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A718" s="3" t="s">
+        <v>1719</v>
+      </c>
+      <c r="B718" s="4" t="s">
+        <v>1720</v>
+      </c>
+      <c r="C718" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="D718" s="4" t="s">
+        <v>903</v>
+      </c>
+      <c r="E718" s="4" t="s">
+        <v>1721</v>
+      </c>
+      <c r="F718" s="2">
+        <v>46178.75</v>
       </c>
     </row>
   </sheetData>
@@ -20581,6 +20687,11 @@
     <hyperlink ref="A711" r:id="rId710"/>
     <hyperlink ref="A712" r:id="rId711"/>
     <hyperlink ref="A713" r:id="rId712"/>
+    <hyperlink ref="A714" r:id="rId713"/>
+    <hyperlink ref="A715" r:id="rId714"/>
+    <hyperlink ref="A716" r:id="rId715"/>
+    <hyperlink ref="A717" r:id="rId716"/>
+    <hyperlink ref="A718" r:id="rId717"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -20592,7 +20703,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -20625,111 +20736,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1708</v>
+        <v>1722</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>25</v>
+        <v>1723</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>435</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46181.49166666667</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1709</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>1710</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1711</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46179.93958333333</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1712</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>1713</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1714</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46181.41458333333</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1715</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>1716</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>1717</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1718</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46181.45625</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>1719</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>1720</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>356</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>903</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>1721</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46178.75</v>
+        <v>46181.902083333334</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-06-10 14:46
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3602" uniqueCount="1724">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3612" uniqueCount="1727">
   <si>
     <t>link</t>
   </si>
@@ -5190,6 +5190,15 @@
   </si>
   <si>
     <t>55 200 €</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/visku-pag/depeo.html</t>
+  </si>
+  <si>
+    <t>44980010373</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valka-and-reg/blomes-pag/bxpdni.html</t>
   </si>
 </sst>
 </file>
@@ -5602,7 +5611,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F718"/>
+  <dimension ref="A1:F719"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -19971,6 +19980,26 @@
       </c>
       <c r="F718" s="2">
         <v>46178.75</v>
+      </c>
+    </row>
+    <row r="719" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A719" s="3" t="s">
+        <v>1722</v>
+      </c>
+      <c r="B719" s="4" t="s">
+        <v>1723</v>
+      </c>
+      <c r="C719" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D719" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E719" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F719" s="2">
+        <v>46181.902083333334</v>
       </c>
     </row>
   </sheetData>
@@ -20692,6 +20721,7 @@
     <hyperlink ref="A716" r:id="rId715"/>
     <hyperlink ref="A717" r:id="rId716"/>
     <hyperlink ref="A718" r:id="rId717"/>
+    <hyperlink ref="A719" r:id="rId718"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -20703,7 +20733,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -20736,27 +20766,48 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1722</v>
+        <v>1724</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1723</v>
+        <v>637</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>435</v>
+        <v>74</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>24</v>
+        <v>162</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>25</v>
+        <v>1725</v>
       </c>
       <c r="F2" s="2">
-        <v>46181.902083333334</v>
+        <v>46183.461111111115</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1726</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>563</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46183.38958333334</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-06-11 15:29
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3612" uniqueCount="1727">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3827" uniqueCount="1840">
   <si>
     <t>link</t>
   </si>
@@ -5199,6 +5199,345 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/valka-and-reg/blomes-pag/bxpdni.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/alsviku-pag/mejkn.html</t>
+  </si>
+  <si>
+    <t>36420060113</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/lazdukalna-pag/egcfd.html</t>
+  </si>
+  <si>
+    <t>2.80 ha.</t>
+  </si>
+  <si>
+    <t>38640070053</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/krisjanu-pag/ingpc.html</t>
+  </si>
+  <si>
+    <t>38560020207</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/krisjanu-pag/fxhfx.html</t>
+  </si>
+  <si>
+    <t>54 000 €</t>
+  </si>
+  <si>
+    <t>15.40 ha.</t>
+  </si>
+  <si>
+    <t>38560020203</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/naujenes-pag/pbdpn.html</t>
+  </si>
+  <si>
+    <t>1.84 ha.</t>
+  </si>
+  <si>
+    <t>44740080189</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/visku-pag/bxfmce.html</t>
+  </si>
+  <si>
+    <t>3.34 ha.</t>
+  </si>
+  <si>
+    <t>44980030318</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/pilskalnes-pag/ljndg.html</t>
+  </si>
+  <si>
+    <t>44800050009</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/elksnu-pag/cncif.html</t>
+  </si>
+  <si>
+    <t>81 000 €</t>
+  </si>
+  <si>
+    <t>22.90 ha.</t>
+  </si>
+  <si>
+    <t>56580080044</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/viesites-l-t/gjkpd.html</t>
+  </si>
+  <si>
+    <t>24.70 ha.</t>
+  </si>
+  <si>
+    <t>56350140047</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/dignajas-pag/jhjfx.html</t>
+  </si>
+  <si>
+    <t>56520060039</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/kalna-pag/jpfkm.html</t>
+  </si>
+  <si>
+    <t>56660010163</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/kuku-pag/ieimi.html</t>
+  </si>
+  <si>
+    <t>56700080012</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/kastulinas-pag/hnggg.html</t>
+  </si>
+  <si>
+    <t>17.90 ha.</t>
+  </si>
+  <si>
+    <t>60720010154</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/asunes-pag/oemee.html</t>
+  </si>
+  <si>
+    <t>60460020037</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/indras-pag/fbgdb.html</t>
+  </si>
+  <si>
+    <t>5.10 ha.</t>
+  </si>
+  <si>
+    <t>60640010233</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/skeltovas-pag/exhei.html</t>
+  </si>
+  <si>
+    <t>1.50 ha.</t>
+  </si>
+  <si>
+    <t>60940050045</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/ezernieku-pag/eibfp.html</t>
+  </si>
+  <si>
+    <t>16.50 ha.</t>
+  </si>
+  <si>
+    <t>60560050026</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/skaistas-pag/liecf.html</t>
+  </si>
+  <si>
+    <t>15.02 ha.</t>
+  </si>
+  <si>
+    <t>60880040190</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/skeltovas-pag/mkmho.html</t>
+  </si>
+  <si>
+    <t>4.20 ha.</t>
+  </si>
+  <si>
+    <t>60940060218</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kuldiga-and-reg/rumbas-pag/dpnfx.html</t>
+  </si>
+  <si>
+    <t>32.85 ha.</t>
+  </si>
+  <si>
+    <t>62840100190</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/limbadzi-and-reg/staiceles-l-t/ildld.html</t>
+  </si>
+  <si>
+    <t>66370010260</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/limbadzi-and-reg/salacgrivas-l-t/dmexb.html</t>
+  </si>
+  <si>
+    <t>1.30 ha.</t>
+  </si>
+  <si>
+    <t>66720100405</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/limbadzi-and-reg/braslavas-pag/kfble.html</t>
+  </si>
+  <si>
+    <t>66440030103</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/limbadzi-and-reg/vilkenes-pag/gihxx.html</t>
+  </si>
+  <si>
+    <t>6.57 ha.</t>
+  </si>
+  <si>
+    <t>66880060366</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/limbadzi-and-reg/skultes-pag/efpxk.html</t>
+  </si>
+  <si>
+    <t>66760160088</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ludza-and-reg/merdzenes-pag/dpxip.html</t>
+  </si>
+  <si>
+    <t>68720050211</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ludza-and-reg/nirzas-pag/ipcox.html</t>
+  </si>
+  <si>
+    <t>10.50 ha.</t>
+  </si>
+  <si>
+    <t>68780070085</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ludza-and-reg/pildas-pag/cgmxkh.html</t>
+  </si>
+  <si>
+    <t>68860010454</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ludza-and-reg/nirzas-pag/ikfof.html</t>
+  </si>
+  <si>
+    <t>29.30 ha.</t>
+  </si>
+  <si>
+    <t>68780020159</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/aglonas-pag/hcnob.html</t>
+  </si>
+  <si>
+    <t>10.10 ha.</t>
+  </si>
+  <si>
+    <t>76420010366</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/rusonas-pag/fohnn.html</t>
+  </si>
+  <si>
+    <t>76700050091</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/saunas-pag/jixpm.html</t>
+  </si>
+  <si>
+    <t>5.41 ha.</t>
+  </si>
+  <si>
+    <t>76740020297</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/varkavas-pag/fnxep.html</t>
+  </si>
+  <si>
+    <t>76940020311</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/aglonas-pag/ckcjj.html</t>
+  </si>
+  <si>
+    <t>1.40 ha.</t>
+  </si>
+  <si>
+    <t>76420040112</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/makonkalna-pag/coikf.html</t>
+  </si>
+  <si>
+    <t>25.20 ha.</t>
+  </si>
+  <si>
+    <t>78720100164</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/gaigalavas-pag/jjkmk.html</t>
+  </si>
+  <si>
+    <t>10.51 ha.</t>
+  </si>
+  <si>
+    <t>78540040049</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/feimanu-pag/aidpe.html</t>
+  </si>
+  <si>
+    <t>9.10 ha.</t>
+  </si>
+  <si>
+    <t>78520070044</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/sakstagala-pag/epohp.html</t>
+  </si>
+  <si>
+    <t>78860030607</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/talsi-and-reg/virbu-pag/bhgkgx.html</t>
+  </si>
+  <si>
+    <t>88960010020</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/tukums-and-reg/zentenes-pag/mjxlf.html</t>
+  </si>
+  <si>
+    <t>13.42 ha.</t>
+  </si>
+  <si>
+    <t>90960040281</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/tukums-and-reg/vanes-pag/gipbp.html</t>
+  </si>
+  <si>
+    <t>90880070025</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valka-and-reg/karku-pag/pnkok.html</t>
+  </si>
+  <si>
+    <t>52 000 €</t>
+  </si>
+  <si>
+    <t>14.68 ha.</t>
+  </si>
+  <si>
+    <t>94660090189</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valmiera-and-reg/jeru-pag/bhhccd.html</t>
   </si>
 </sst>
 </file>
@@ -5611,7 +5950,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F719"/>
+  <dimension ref="A1:F721"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -20000,6 +20339,46 @@
       </c>
       <c r="F719" s="2">
         <v>46181.902083333334</v>
+      </c>
+    </row>
+    <row r="720" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A720" s="3" t="s">
+        <v>1724</v>
+      </c>
+      <c r="B720" s="4" t="s">
+        <v>637</v>
+      </c>
+      <c r="C720" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D720" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="E720" s="4" t="s">
+        <v>1725</v>
+      </c>
+      <c r="F720" s="2">
+        <v>46183.461111111115</v>
+      </c>
+    </row>
+    <row r="721" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A721" s="3" t="s">
+        <v>1726</v>
+      </c>
+      <c r="B721" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C721" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="D721" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E721" s="4" t="s">
+        <v>563</v>
+      </c>
+      <c r="F721" s="2">
+        <v>46183.38958333334</v>
       </c>
     </row>
   </sheetData>
@@ -20722,6 +21101,8 @@
     <hyperlink ref="A717" r:id="rId716"/>
     <hyperlink ref="A718" r:id="rId717"/>
     <hyperlink ref="A719" r:id="rId718"/>
+    <hyperlink ref="A720" r:id="rId719"/>
+    <hyperlink ref="A721" r:id="rId720"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -20733,7 +21114,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -20766,48 +21147,909 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1724</v>
+        <v>1727</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>637</v>
+        <v>185</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>74</v>
+        <v>435</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>162</v>
+        <v>49</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1725</v>
+        <v>1728</v>
       </c>
       <c r="F2" s="2">
-        <v>46183.461111111115</v>
+        <v>46184.44930555555</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1726</v>
+        <v>1729</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>1730</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1731</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46184.45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1732</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1733</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46184.45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1734</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>1735</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>1736</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1737</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46184.45</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>1738</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>505</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>1739</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>1740</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46184.45277777778</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>1741</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>1742</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>1743</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46184.45208333334</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>1744</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>505</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>737</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>1745</v>
+      </c>
+      <c r="F8" s="2">
+        <v>46184.447222222225</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>1746</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>1747</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>1748</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>1749</v>
+      </c>
+      <c r="F9" s="2">
+        <v>46184.45208333334</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>1750</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>1751</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>1752</v>
+      </c>
+      <c r="F10" s="2">
+        <v>46184.45138888889</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>1753</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>1754</v>
+      </c>
+      <c r="F11" s="2">
+        <v>46184.450694444444</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>1755</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>1505</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>1756</v>
+      </c>
+      <c r="F12" s="2">
+        <v>46184.450694444444</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>1757</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>536</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>659</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>1758</v>
+      </c>
+      <c r="F13" s="2">
+        <v>46184.45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>1759</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>854</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>1760</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>1761</v>
+      </c>
+      <c r="F14" s="2">
+        <v>46184.45277777778</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>1762</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>707</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>1763</v>
+      </c>
+      <c r="F15" s="2">
+        <v>46184.450694444444</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>1764</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>1765</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>1766</v>
+      </c>
+      <c r="F16" s="2">
+        <v>46184.450694444444</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>1767</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>1768</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>1769</v>
+      </c>
+      <c r="F17" s="2">
+        <v>46184.45</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>1770</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>1771</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>1772</v>
+      </c>
+      <c r="F18" s="2">
+        <v>46184.44930555555</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>1773</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>1774</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>1775</v>
+      </c>
+      <c r="F19" s="2">
+        <v>46184.44930555555</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>1776</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>1777</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>1778</v>
+      </c>
+      <c r="F20" s="2">
+        <v>46184.447222222225</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>1779</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>673</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>1780</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>1781</v>
+      </c>
+      <c r="F21" s="2">
+        <v>46184.44861111111</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>1782</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>1783</v>
+      </c>
+      <c r="F22" s="2">
+        <v>46184.71875</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>1784</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>1785</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>1786</v>
+      </c>
+      <c r="F23" s="2">
+        <v>46184.45208333334</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>1787</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>1788</v>
+      </c>
+      <c r="F24" s="2">
+        <v>46184.45208333334</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>1789</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>1790</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>1791</v>
+      </c>
+      <c r="F25" s="2">
+        <v>46184.45208333334</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>1792</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>1575</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>1793</v>
+      </c>
+      <c r="F26" s="2">
+        <v>46184.450694444444</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>1794</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>1795</v>
+      </c>
+      <c r="F27" s="2">
+        <v>46184.450694444444</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>1796</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>1797</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>1798</v>
+      </c>
+      <c r="F28" s="2">
+        <v>46184.450694444444</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>1799</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>793</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>1800</v>
+      </c>
+      <c r="F29" s="2">
+        <v>46184.44930555555</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>1801</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>1313</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>1802</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>1803</v>
+      </c>
+      <c r="F30" s="2">
+        <v>46184.447222222225</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>1804</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>1805</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>1806</v>
+      </c>
+      <c r="F31" s="2">
+        <v>46184.45208333334</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>1807</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>716</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>1808</v>
+      </c>
+      <c r="F32" s="2">
+        <v>46184.45208333334</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>1809</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>1810</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>1811</v>
+      </c>
+      <c r="F33" s="2">
+        <v>46184.44930555555</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
+        <v>1812</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>1259</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>1813</v>
+      </c>
+      <c r="F34" s="2">
+        <v>46184.447222222225</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>1814</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>1815</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>1816</v>
+      </c>
+      <c r="F35" s="2">
+        <v>46184.447222222225</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>1817</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>1313</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>1818</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>1819</v>
+      </c>
+      <c r="F36" s="2">
+        <v>46184.45138888889</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>1822</v>
+      </c>
+      <c r="F37" s="2">
+        <v>46184.45138888889</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
+        <v>1823</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>1824</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>1825</v>
+      </c>
+      <c r="F38" s="2">
+        <v>46184.450694444444</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>1826</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>334</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>1827</v>
+      </c>
+      <c r="F39" s="2">
+        <v>46184.44861111111</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
+        <v>1828</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>816</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>1829</v>
+      </c>
+      <c r="F40" s="2">
+        <v>46184.45138888889</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>1830</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>906</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>1831</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>1832</v>
+      </c>
+      <c r="F41" s="2">
+        <v>46184.71875</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
+        <v>1833</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>871</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>1834</v>
+      </c>
+      <c r="F42" s="2">
+        <v>46184.45208333334</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
+        <v>1835</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>1836</v>
+      </c>
+      <c r="C43" s="4" t="s">
         <v>392</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>563</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46183.38958333334</v>
+      <c r="D43" s="4" t="s">
+        <v>1837</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>1838</v>
+      </c>
+      <c r="F43" s="2">
+        <v>46184.44930555555</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
+        <v>1839</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>988</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>1064</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>1065</v>
+      </c>
+      <c r="F44" s="2">
+        <v>46184.45208333334</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+    <hyperlink ref="A6" r:id="rId5"/>
+    <hyperlink ref="A7" r:id="rId6"/>
+    <hyperlink ref="A8" r:id="rId7"/>
+    <hyperlink ref="A9" r:id="rId8"/>
+    <hyperlink ref="A10" r:id="rId9"/>
+    <hyperlink ref="A11" r:id="rId10"/>
+    <hyperlink ref="A12" r:id="rId11"/>
+    <hyperlink ref="A13" r:id="rId12"/>
+    <hyperlink ref="A14" r:id="rId13"/>
+    <hyperlink ref="A15" r:id="rId14"/>
+    <hyperlink ref="A16" r:id="rId15"/>
+    <hyperlink ref="A17" r:id="rId16"/>
+    <hyperlink ref="A18" r:id="rId17"/>
+    <hyperlink ref="A19" r:id="rId18"/>
+    <hyperlink ref="A20" r:id="rId19"/>
+    <hyperlink ref="A21" r:id="rId20"/>
+    <hyperlink ref="A22" r:id="rId21"/>
+    <hyperlink ref="A23" r:id="rId22"/>
+    <hyperlink ref="A24" r:id="rId23"/>
+    <hyperlink ref="A25" r:id="rId24"/>
+    <hyperlink ref="A26" r:id="rId25"/>
+    <hyperlink ref="A27" r:id="rId26"/>
+    <hyperlink ref="A28" r:id="rId27"/>
+    <hyperlink ref="A29" r:id="rId28"/>
+    <hyperlink ref="A30" r:id="rId29"/>
+    <hyperlink ref="A31" r:id="rId30"/>
+    <hyperlink ref="A32" r:id="rId31"/>
+    <hyperlink ref="A33" r:id="rId32"/>
+    <hyperlink ref="A34" r:id="rId33"/>
+    <hyperlink ref="A35" r:id="rId34"/>
+    <hyperlink ref="A36" r:id="rId35"/>
+    <hyperlink ref="A37" r:id="rId36"/>
+    <hyperlink ref="A38" r:id="rId37"/>
+    <hyperlink ref="A39" r:id="rId38"/>
+    <hyperlink ref="A40" r:id="rId39"/>
+    <hyperlink ref="A41" r:id="rId40"/>
+    <hyperlink ref="A42" r:id="rId41"/>
+    <hyperlink ref="A43" r:id="rId42"/>
+    <hyperlink ref="A44" r:id="rId43"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-06-12 14:27
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3827" uniqueCount="1840">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3837" uniqueCount="1845">
   <si>
     <t>link</t>
   </si>
@@ -5538,6 +5538,21 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/valmiera-and-reg/jeru-pag/bhhccd.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/ligatnes-pag/kkonj.html</t>
+  </si>
+  <si>
+    <t>5.70 ha.</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/saldus-and-reg/zirnu-pag/nikmd.html</t>
+  </si>
+  <si>
+    <t>77 000 €</t>
+  </si>
+  <si>
+    <t>84960070140</t>
   </si>
 </sst>
 </file>
@@ -5950,7 +5965,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F721"/>
+  <dimension ref="A1:F764"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -20379,6 +20394,866 @@
       </c>
       <c r="F721" s="2">
         <v>46183.38958333334</v>
+      </c>
+    </row>
+    <row r="722" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A722" s="3" t="s">
+        <v>1727</v>
+      </c>
+      <c r="B722" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C722" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D722" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E722" s="4" t="s">
+        <v>1728</v>
+      </c>
+      <c r="F722" s="2">
+        <v>46184.44930555555</v>
+      </c>
+    </row>
+    <row r="723" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A723" s="3" t="s">
+        <v>1729</v>
+      </c>
+      <c r="B723" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C723" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D723" s="4" t="s">
+        <v>1730</v>
+      </c>
+      <c r="E723" s="4" t="s">
+        <v>1731</v>
+      </c>
+      <c r="F723" s="2">
+        <v>46184.45</v>
+      </c>
+    </row>
+    <row r="724" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A724" s="3" t="s">
+        <v>1732</v>
+      </c>
+      <c r="B724" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C724" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D724" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="E724" s="4" t="s">
+        <v>1733</v>
+      </c>
+      <c r="F724" s="2">
+        <v>46184.45</v>
+      </c>
+    </row>
+    <row r="725" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A725" s="3" t="s">
+        <v>1734</v>
+      </c>
+      <c r="B725" s="4" t="s">
+        <v>1735</v>
+      </c>
+      <c r="C725" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D725" s="4" t="s">
+        <v>1736</v>
+      </c>
+      <c r="E725" s="4" t="s">
+        <v>1737</v>
+      </c>
+      <c r="F725" s="2">
+        <v>46184.45</v>
+      </c>
+    </row>
+    <row r="726" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A726" s="3" t="s">
+        <v>1738</v>
+      </c>
+      <c r="B726" s="4" t="s">
+        <v>505</v>
+      </c>
+      <c r="C726" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D726" s="4" t="s">
+        <v>1739</v>
+      </c>
+      <c r="E726" s="4" t="s">
+        <v>1740</v>
+      </c>
+      <c r="F726" s="2">
+        <v>46184.45277777778</v>
+      </c>
+    </row>
+    <row r="727" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A727" s="3" t="s">
+        <v>1741</v>
+      </c>
+      <c r="B727" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C727" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D727" s="4" t="s">
+        <v>1742</v>
+      </c>
+      <c r="E727" s="4" t="s">
+        <v>1743</v>
+      </c>
+      <c r="F727" s="2">
+        <v>46184.45208333334</v>
+      </c>
+    </row>
+    <row r="728" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A728" s="3" t="s">
+        <v>1744</v>
+      </c>
+      <c r="B728" s="4" t="s">
+        <v>505</v>
+      </c>
+      <c r="C728" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D728" s="4" t="s">
+        <v>737</v>
+      </c>
+      <c r="E728" s="4" t="s">
+        <v>1745</v>
+      </c>
+      <c r="F728" s="2">
+        <v>46184.447222222225</v>
+      </c>
+    </row>
+    <row r="729" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A729" s="3" t="s">
+        <v>1746</v>
+      </c>
+      <c r="B729" s="4" t="s">
+        <v>1747</v>
+      </c>
+      <c r="C729" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D729" s="4" t="s">
+        <v>1748</v>
+      </c>
+      <c r="E729" s="4" t="s">
+        <v>1749</v>
+      </c>
+      <c r="F729" s="2">
+        <v>46184.45208333334</v>
+      </c>
+    </row>
+    <row r="730" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A730" s="3" t="s">
+        <v>1750</v>
+      </c>
+      <c r="B730" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="C730" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D730" s="4" t="s">
+        <v>1751</v>
+      </c>
+      <c r="E730" s="4" t="s">
+        <v>1752</v>
+      </c>
+      <c r="F730" s="2">
+        <v>46184.45138888889</v>
+      </c>
+    </row>
+    <row r="731" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A731" s="3" t="s">
+        <v>1753</v>
+      </c>
+      <c r="B731" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C731" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D731" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="E731" s="4" t="s">
+        <v>1754</v>
+      </c>
+      <c r="F731" s="2">
+        <v>46184.450694444444</v>
+      </c>
+    </row>
+    <row r="732" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A732" s="3" t="s">
+        <v>1755</v>
+      </c>
+      <c r="B732" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C732" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D732" s="4" t="s">
+        <v>1505</v>
+      </c>
+      <c r="E732" s="4" t="s">
+        <v>1756</v>
+      </c>
+      <c r="F732" s="2">
+        <v>46184.450694444444</v>
+      </c>
+    </row>
+    <row r="733" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A733" s="3" t="s">
+        <v>1757</v>
+      </c>
+      <c r="B733" s="4" t="s">
+        <v>536</v>
+      </c>
+      <c r="C733" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D733" s="4" t="s">
+        <v>659</v>
+      </c>
+      <c r="E733" s="4" t="s">
+        <v>1758</v>
+      </c>
+      <c r="F733" s="2">
+        <v>46184.45</v>
+      </c>
+    </row>
+    <row r="734" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A734" s="3" t="s">
+        <v>1759</v>
+      </c>
+      <c r="B734" s="4" t="s">
+        <v>854</v>
+      </c>
+      <c r="C734" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D734" s="4" t="s">
+        <v>1760</v>
+      </c>
+      <c r="E734" s="4" t="s">
+        <v>1761</v>
+      </c>
+      <c r="F734" s="2">
+        <v>46184.45277777778</v>
+      </c>
+    </row>
+    <row r="735" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A735" s="3" t="s">
+        <v>1762</v>
+      </c>
+      <c r="B735" s="4" t="s">
+        <v>707</v>
+      </c>
+      <c r="C735" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D735" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="E735" s="4" t="s">
+        <v>1763</v>
+      </c>
+      <c r="F735" s="2">
+        <v>46184.450694444444</v>
+      </c>
+    </row>
+    <row r="736" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A736" s="3" t="s">
+        <v>1764</v>
+      </c>
+      <c r="B736" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C736" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D736" s="4" t="s">
+        <v>1765</v>
+      </c>
+      <c r="E736" s="4" t="s">
+        <v>1766</v>
+      </c>
+      <c r="F736" s="2">
+        <v>46184.450694444444</v>
+      </c>
+    </row>
+    <row r="737" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A737" s="3" t="s">
+        <v>1767</v>
+      </c>
+      <c r="B737" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="C737" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D737" s="4" t="s">
+        <v>1768</v>
+      </c>
+      <c r="E737" s="4" t="s">
+        <v>1769</v>
+      </c>
+      <c r="F737" s="2">
+        <v>46184.45</v>
+      </c>
+    </row>
+    <row r="738" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A738" s="3" t="s">
+        <v>1770</v>
+      </c>
+      <c r="B738" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="C738" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D738" s="4" t="s">
+        <v>1771</v>
+      </c>
+      <c r="E738" s="4" t="s">
+        <v>1772</v>
+      </c>
+      <c r="F738" s="2">
+        <v>46184.44930555555</v>
+      </c>
+    </row>
+    <row r="739" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A739" s="3" t="s">
+        <v>1773</v>
+      </c>
+      <c r="B739" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="C739" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D739" s="4" t="s">
+        <v>1774</v>
+      </c>
+      <c r="E739" s="4" t="s">
+        <v>1775</v>
+      </c>
+      <c r="F739" s="2">
+        <v>46184.44930555555</v>
+      </c>
+    </row>
+    <row r="740" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A740" s="3" t="s">
+        <v>1776</v>
+      </c>
+      <c r="B740" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="C740" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D740" s="4" t="s">
+        <v>1777</v>
+      </c>
+      <c r="E740" s="4" t="s">
+        <v>1778</v>
+      </c>
+      <c r="F740" s="2">
+        <v>46184.447222222225</v>
+      </c>
+    </row>
+    <row r="741" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A741" s="3" t="s">
+        <v>1779</v>
+      </c>
+      <c r="B741" s="4" t="s">
+        <v>673</v>
+      </c>
+      <c r="C741" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="D741" s="4" t="s">
+        <v>1780</v>
+      </c>
+      <c r="E741" s="4" t="s">
+        <v>1781</v>
+      </c>
+      <c r="F741" s="2">
+        <v>46184.44861111111</v>
+      </c>
+    </row>
+    <row r="742" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A742" s="3" t="s">
+        <v>1782</v>
+      </c>
+      <c r="B742" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C742" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D742" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E742" s="4" t="s">
+        <v>1783</v>
+      </c>
+      <c r="F742" s="2">
+        <v>46184.71875</v>
+      </c>
+    </row>
+    <row r="743" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A743" s="3" t="s">
+        <v>1784</v>
+      </c>
+      <c r="B743" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="C743" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D743" s="4" t="s">
+        <v>1785</v>
+      </c>
+      <c r="E743" s="4" t="s">
+        <v>1786</v>
+      </c>
+      <c r="F743" s="2">
+        <v>46184.45208333334</v>
+      </c>
+    </row>
+    <row r="744" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A744" s="3" t="s">
+        <v>1787</v>
+      </c>
+      <c r="B744" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C744" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D744" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="E744" s="4" t="s">
+        <v>1788</v>
+      </c>
+      <c r="F744" s="2">
+        <v>46184.45208333334</v>
+      </c>
+    </row>
+    <row r="745" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A745" s="3" t="s">
+        <v>1789</v>
+      </c>
+      <c r="B745" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C745" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D745" s="4" t="s">
+        <v>1790</v>
+      </c>
+      <c r="E745" s="4" t="s">
+        <v>1791</v>
+      </c>
+      <c r="F745" s="2">
+        <v>46184.45208333334</v>
+      </c>
+    </row>
+    <row r="746" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A746" s="3" t="s">
+        <v>1792</v>
+      </c>
+      <c r="B746" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C746" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D746" s="4" t="s">
+        <v>1575</v>
+      </c>
+      <c r="E746" s="4" t="s">
+        <v>1793</v>
+      </c>
+      <c r="F746" s="2">
+        <v>46184.450694444444</v>
+      </c>
+    </row>
+    <row r="747" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A747" s="3" t="s">
+        <v>1794</v>
+      </c>
+      <c r="B747" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C747" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D747" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="E747" s="4" t="s">
+        <v>1795</v>
+      </c>
+      <c r="F747" s="2">
+        <v>46184.450694444444</v>
+      </c>
+    </row>
+    <row r="748" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A748" s="3" t="s">
+        <v>1796</v>
+      </c>
+      <c r="B748" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C748" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D748" s="4" t="s">
+        <v>1797</v>
+      </c>
+      <c r="E748" s="4" t="s">
+        <v>1798</v>
+      </c>
+      <c r="F748" s="2">
+        <v>46184.450694444444</v>
+      </c>
+    </row>
+    <row r="749" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A749" s="3" t="s">
+        <v>1799</v>
+      </c>
+      <c r="B749" s="4" t="s">
+        <v>793</v>
+      </c>
+      <c r="C749" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D749" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="E749" s="4" t="s">
+        <v>1800</v>
+      </c>
+      <c r="F749" s="2">
+        <v>46184.44930555555</v>
+      </c>
+    </row>
+    <row r="750" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A750" s="3" t="s">
+        <v>1801</v>
+      </c>
+      <c r="B750" s="4" t="s">
+        <v>1313</v>
+      </c>
+      <c r="C750" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D750" s="4" t="s">
+        <v>1802</v>
+      </c>
+      <c r="E750" s="4" t="s">
+        <v>1803</v>
+      </c>
+      <c r="F750" s="2">
+        <v>46184.447222222225</v>
+      </c>
+    </row>
+    <row r="751" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A751" s="3" t="s">
+        <v>1804</v>
+      </c>
+      <c r="B751" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C751" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D751" s="4" t="s">
+        <v>1805</v>
+      </c>
+      <c r="E751" s="4" t="s">
+        <v>1806</v>
+      </c>
+      <c r="F751" s="2">
+        <v>46184.45208333334</v>
+      </c>
+    </row>
+    <row r="752" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A752" s="3" t="s">
+        <v>1807</v>
+      </c>
+      <c r="B752" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C752" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D752" s="4" t="s">
+        <v>716</v>
+      </c>
+      <c r="E752" s="4" t="s">
+        <v>1808</v>
+      </c>
+      <c r="F752" s="2">
+        <v>46184.45208333334</v>
+      </c>
+    </row>
+    <row r="753" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A753" s="3" t="s">
+        <v>1809</v>
+      </c>
+      <c r="B753" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C753" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D753" s="4" t="s">
+        <v>1810</v>
+      </c>
+      <c r="E753" s="4" t="s">
+        <v>1811</v>
+      </c>
+      <c r="F753" s="2">
+        <v>46184.44930555555</v>
+      </c>
+    </row>
+    <row r="754" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A754" s="3" t="s">
+        <v>1812</v>
+      </c>
+      <c r="B754" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="C754" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D754" s="4" t="s">
+        <v>1259</v>
+      </c>
+      <c r="E754" s="4" t="s">
+        <v>1813</v>
+      </c>
+      <c r="F754" s="2">
+        <v>46184.447222222225</v>
+      </c>
+    </row>
+    <row r="755" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A755" s="3" t="s">
+        <v>1814</v>
+      </c>
+      <c r="B755" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="C755" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D755" s="4" t="s">
+        <v>1815</v>
+      </c>
+      <c r="E755" s="4" t="s">
+        <v>1816</v>
+      </c>
+      <c r="F755" s="2">
+        <v>46184.447222222225</v>
+      </c>
+    </row>
+    <row r="756" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A756" s="3" t="s">
+        <v>1817</v>
+      </c>
+      <c r="B756" s="4" t="s">
+        <v>1313</v>
+      </c>
+      <c r="C756" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D756" s="4" t="s">
+        <v>1818</v>
+      </c>
+      <c r="E756" s="4" t="s">
+        <v>1819</v>
+      </c>
+      <c r="F756" s="2">
+        <v>46184.45138888889</v>
+      </c>
+    </row>
+    <row r="757" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A757" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="B757" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C757" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D757" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="E757" s="4" t="s">
+        <v>1822</v>
+      </c>
+      <c r="F757" s="2">
+        <v>46184.45138888889</v>
+      </c>
+    </row>
+    <row r="758" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A758" s="3" t="s">
+        <v>1823</v>
+      </c>
+      <c r="B758" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C758" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D758" s="4" t="s">
+        <v>1824</v>
+      </c>
+      <c r="E758" s="4" t="s">
+        <v>1825</v>
+      </c>
+      <c r="F758" s="2">
+        <v>46184.450694444444</v>
+      </c>
+    </row>
+    <row r="759" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A759" s="3" t="s">
+        <v>1826</v>
+      </c>
+      <c r="B759" s="4" t="s">
+        <v>334</v>
+      </c>
+      <c r="C759" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D759" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="E759" s="4" t="s">
+        <v>1827</v>
+      </c>
+      <c r="F759" s="2">
+        <v>46184.44861111111</v>
+      </c>
+    </row>
+    <row r="760" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A760" s="3" t="s">
+        <v>1828</v>
+      </c>
+      <c r="B760" s="4" t="s">
+        <v>816</v>
+      </c>
+      <c r="C760" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="D760" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="E760" s="4" t="s">
+        <v>1829</v>
+      </c>
+      <c r="F760" s="2">
+        <v>46184.45138888889</v>
+      </c>
+    </row>
+    <row r="761" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A761" s="3" t="s">
+        <v>1830</v>
+      </c>
+      <c r="B761" s="4" t="s">
+        <v>906</v>
+      </c>
+      <c r="C761" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D761" s="4" t="s">
+        <v>1831</v>
+      </c>
+      <c r="E761" s="4" t="s">
+        <v>1832</v>
+      </c>
+      <c r="F761" s="2">
+        <v>46184.71875</v>
+      </c>
+    </row>
+    <row r="762" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A762" s="3" t="s">
+        <v>1833</v>
+      </c>
+      <c r="B762" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="C762" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D762" s="4" t="s">
+        <v>871</v>
+      </c>
+      <c r="E762" s="4" t="s">
+        <v>1834</v>
+      </c>
+      <c r="F762" s="2">
+        <v>46184.45208333334</v>
+      </c>
+    </row>
+    <row r="763" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A763" s="3" t="s">
+        <v>1835</v>
+      </c>
+      <c r="B763" s="4" t="s">
+        <v>1836</v>
+      </c>
+      <c r="C763" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="D763" s="4" t="s">
+        <v>1837</v>
+      </c>
+      <c r="E763" s="4" t="s">
+        <v>1838</v>
+      </c>
+      <c r="F763" s="2">
+        <v>46184.44930555555</v>
+      </c>
+    </row>
+    <row r="764" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A764" s="3" t="s">
+        <v>1839</v>
+      </c>
+      <c r="B764" s="4" t="s">
+        <v>988</v>
+      </c>
+      <c r="C764" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D764" s="4" t="s">
+        <v>1064</v>
+      </c>
+      <c r="E764" s="4" t="s">
+        <v>1065</v>
+      </c>
+      <c r="F764" s="2">
+        <v>46184.45208333334</v>
       </c>
     </row>
   </sheetData>
@@ -21103,6 +21978,49 @@
     <hyperlink ref="A719" r:id="rId718"/>
     <hyperlink ref="A720" r:id="rId719"/>
     <hyperlink ref="A721" r:id="rId720"/>
+    <hyperlink ref="A722" r:id="rId721"/>
+    <hyperlink ref="A723" r:id="rId722"/>
+    <hyperlink ref="A724" r:id="rId723"/>
+    <hyperlink ref="A725" r:id="rId724"/>
+    <hyperlink ref="A726" r:id="rId725"/>
+    <hyperlink ref="A727" r:id="rId726"/>
+    <hyperlink ref="A728" r:id="rId727"/>
+    <hyperlink ref="A729" r:id="rId728"/>
+    <hyperlink ref="A730" r:id="rId729"/>
+    <hyperlink ref="A731" r:id="rId730"/>
+    <hyperlink ref="A732" r:id="rId731"/>
+    <hyperlink ref="A733" r:id="rId732"/>
+    <hyperlink ref="A734" r:id="rId733"/>
+    <hyperlink ref="A735" r:id="rId734"/>
+    <hyperlink ref="A736" r:id="rId735"/>
+    <hyperlink ref="A737" r:id="rId736"/>
+    <hyperlink ref="A738" r:id="rId737"/>
+    <hyperlink ref="A739" r:id="rId738"/>
+    <hyperlink ref="A740" r:id="rId739"/>
+    <hyperlink ref="A741" r:id="rId740"/>
+    <hyperlink ref="A742" r:id="rId741"/>
+    <hyperlink ref="A743" r:id="rId742"/>
+    <hyperlink ref="A744" r:id="rId743"/>
+    <hyperlink ref="A745" r:id="rId744"/>
+    <hyperlink ref="A746" r:id="rId745"/>
+    <hyperlink ref="A747" r:id="rId746"/>
+    <hyperlink ref="A748" r:id="rId747"/>
+    <hyperlink ref="A749" r:id="rId748"/>
+    <hyperlink ref="A750" r:id="rId749"/>
+    <hyperlink ref="A751" r:id="rId750"/>
+    <hyperlink ref="A752" r:id="rId751"/>
+    <hyperlink ref="A753" r:id="rId752"/>
+    <hyperlink ref="A754" r:id="rId753"/>
+    <hyperlink ref="A755" r:id="rId754"/>
+    <hyperlink ref="A756" r:id="rId755"/>
+    <hyperlink ref="A757" r:id="rId756"/>
+    <hyperlink ref="A758" r:id="rId757"/>
+    <hyperlink ref="A759" r:id="rId758"/>
+    <hyperlink ref="A760" r:id="rId759"/>
+    <hyperlink ref="A761" r:id="rId760"/>
+    <hyperlink ref="A762" r:id="rId761"/>
+    <hyperlink ref="A763" r:id="rId762"/>
+    <hyperlink ref="A764" r:id="rId763"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -21114,7 +22032,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -21147,909 +22065,48 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1727</v>
+        <v>1840</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>185</v>
+        <v>549</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>435</v>
+        <v>63</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>49</v>
+        <v>1841</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1728</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46184.44930555555</v>
+        <v>46184.80208333333</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1729</v>
+        <v>1842</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>116</v>
+        <v>1843</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>28</v>
+        <v>346</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>1730</v>
+        <v>32</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1731</v>
+        <v>1844</v>
       </c>
       <c r="F3" s="2">
-        <v>46184.45</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1732</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>401</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1733</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46184.45</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1734</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>1735</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>1736</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1737</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46184.45</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>1738</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>505</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>1739</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>1740</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46184.45277777778</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>1741</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>1742</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>1743</v>
-      </c>
-      <c r="F7" s="2">
-        <v>46184.45208333334</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>1744</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>505</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>737</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>1745</v>
-      </c>
-      <c r="F8" s="2">
-        <v>46184.447222222225</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>1746</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>1747</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>1748</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>1749</v>
-      </c>
-      <c r="F9" s="2">
-        <v>46184.45208333334</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>1750</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>533</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>1751</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>1752</v>
-      </c>
-      <c r="F10" s="2">
-        <v>46184.45138888889</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>1753</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>329</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>1754</v>
-      </c>
-      <c r="F11" s="2">
-        <v>46184.450694444444</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>1755</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>1505</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>1756</v>
-      </c>
-      <c r="F12" s="2">
-        <v>46184.450694444444</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>1757</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>536</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>659</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>1758</v>
-      </c>
-      <c r="F13" s="2">
-        <v>46184.45</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>1759</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>854</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>1760</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>1761</v>
-      </c>
-      <c r="F14" s="2">
-        <v>46184.45277777778</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>1762</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>707</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>405</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>1763</v>
-      </c>
-      <c r="F15" s="2">
-        <v>46184.450694444444</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
-        <v>1764</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>1765</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>1766</v>
-      </c>
-      <c r="F16" s="2">
-        <v>46184.450694444444</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
-        <v>1767</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>576</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>1768</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>1769</v>
-      </c>
-      <c r="F17" s="2">
-        <v>46184.45</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
-        <v>1770</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>596</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>1771</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>1772</v>
-      </c>
-      <c r="F18" s="2">
-        <v>46184.44930555555</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>1773</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>1774</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>1775</v>
-      </c>
-      <c r="F19" s="2">
-        <v>46184.44930555555</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
-        <v>1776</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>360</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>1777</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>1778</v>
-      </c>
-      <c r="F20" s="2">
-        <v>46184.447222222225</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>1779</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>673</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>424</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>1780</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>1781</v>
-      </c>
-      <c r="F21" s="2">
-        <v>46184.44861111111</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>1782</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>1783</v>
-      </c>
-      <c r="F22" s="2">
-        <v>46184.71875</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
-        <v>1784</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>467</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>1785</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>1786</v>
-      </c>
-      <c r="F23" s="2">
-        <v>46184.45208333334</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
-        <v>1787</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>329</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>1788</v>
-      </c>
-      <c r="F24" s="2">
-        <v>46184.45208333334</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
-        <v>1789</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>1790</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>1791</v>
-      </c>
-      <c r="F25" s="2">
-        <v>46184.45208333334</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>1792</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>1575</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>1793</v>
-      </c>
-      <c r="F26" s="2">
-        <v>46184.450694444444</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
-        <v>1794</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>695</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>1795</v>
-      </c>
-      <c r="F27" s="2">
-        <v>46184.450694444444</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>1796</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>1797</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>1798</v>
-      </c>
-      <c r="F28" s="2">
-        <v>46184.450694444444</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
-        <v>1799</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>793</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>371</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>1800</v>
-      </c>
-      <c r="F29" s="2">
-        <v>46184.44930555555</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
-        <v>1801</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>1313</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>1802</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>1803</v>
-      </c>
-      <c r="F30" s="2">
-        <v>46184.447222222225</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
-        <v>1804</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>1805</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>1806</v>
-      </c>
-      <c r="F31" s="2">
-        <v>46184.45208333334</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
-        <v>1807</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>716</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>1808</v>
-      </c>
-      <c r="F32" s="2">
-        <v>46184.45208333334</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
-        <v>1809</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>1810</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>1811</v>
-      </c>
-      <c r="F33" s="2">
-        <v>46184.44930555555</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
-        <v>1812</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>1259</v>
-      </c>
-      <c r="E34" s="4" t="s">
-        <v>1813</v>
-      </c>
-      <c r="F34" s="2">
-        <v>46184.447222222225</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="3" t="s">
-        <v>1814</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>467</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>1815</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>1816</v>
-      </c>
-      <c r="F35" s="2">
-        <v>46184.447222222225</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
-        <v>1817</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>1313</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="D36" s="4" t="s">
-        <v>1818</v>
-      </c>
-      <c r="E36" s="4" t="s">
-        <v>1819</v>
-      </c>
-      <c r="F36" s="2">
-        <v>46184.45138888889</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
-        <v>1820</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>1821</v>
-      </c>
-      <c r="E37" s="4" t="s">
-        <v>1822</v>
-      </c>
-      <c r="F37" s="2">
-        <v>46184.45138888889</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
-        <v>1823</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="D38" s="4" t="s">
-        <v>1824</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>1825</v>
-      </c>
-      <c r="F38" s="2">
-        <v>46184.450694444444</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="3" t="s">
-        <v>1826</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>334</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="E39" s="4" t="s">
-        <v>1827</v>
-      </c>
-      <c r="F39" s="2">
-        <v>46184.44861111111</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="3" t="s">
-        <v>1828</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>816</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>356</v>
-      </c>
-      <c r="D40" s="4" t="s">
-        <v>401</v>
-      </c>
-      <c r="E40" s="4" t="s">
-        <v>1829</v>
-      </c>
-      <c r="F40" s="2">
-        <v>46184.45138888889</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="3" t="s">
-        <v>1830</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>906</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>376</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>1831</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>1832</v>
-      </c>
-      <c r="F41" s="2">
-        <v>46184.71875</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" s="3" t="s">
-        <v>1833</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>274</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>376</v>
-      </c>
-      <c r="D42" s="4" t="s">
-        <v>871</v>
-      </c>
-      <c r="E42" s="4" t="s">
-        <v>1834</v>
-      </c>
-      <c r="F42" s="2">
-        <v>46184.45208333334</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" s="3" t="s">
-        <v>1835</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>1836</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>392</v>
-      </c>
-      <c r="D43" s="4" t="s">
-        <v>1837</v>
-      </c>
-      <c r="E43" s="4" t="s">
-        <v>1838</v>
-      </c>
-      <c r="F43" s="2">
-        <v>46184.44930555555</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="3" t="s">
-        <v>1839</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>988</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="D44" s="4" t="s">
-        <v>1064</v>
-      </c>
-      <c r="E44" s="4" t="s">
-        <v>1065</v>
-      </c>
-      <c r="F44" s="2">
-        <v>46184.45208333334</v>
+        <v>46185.3</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A6" r:id="rId5"/>
-    <hyperlink ref="A7" r:id="rId6"/>
-    <hyperlink ref="A8" r:id="rId7"/>
-    <hyperlink ref="A9" r:id="rId8"/>
-    <hyperlink ref="A10" r:id="rId9"/>
-    <hyperlink ref="A11" r:id="rId10"/>
-    <hyperlink ref="A12" r:id="rId11"/>
-    <hyperlink ref="A13" r:id="rId12"/>
-    <hyperlink ref="A14" r:id="rId13"/>
-    <hyperlink ref="A15" r:id="rId14"/>
-    <hyperlink ref="A16" r:id="rId15"/>
-    <hyperlink ref="A17" r:id="rId16"/>
-    <hyperlink ref="A18" r:id="rId17"/>
-    <hyperlink ref="A19" r:id="rId18"/>
-    <hyperlink ref="A20" r:id="rId19"/>
-    <hyperlink ref="A21" r:id="rId20"/>
-    <hyperlink ref="A22" r:id="rId21"/>
-    <hyperlink ref="A23" r:id="rId22"/>
-    <hyperlink ref="A24" r:id="rId23"/>
-    <hyperlink ref="A25" r:id="rId24"/>
-    <hyperlink ref="A26" r:id="rId25"/>
-    <hyperlink ref="A27" r:id="rId26"/>
-    <hyperlink ref="A28" r:id="rId27"/>
-    <hyperlink ref="A29" r:id="rId28"/>
-    <hyperlink ref="A30" r:id="rId29"/>
-    <hyperlink ref="A31" r:id="rId30"/>
-    <hyperlink ref="A32" r:id="rId31"/>
-    <hyperlink ref="A33" r:id="rId32"/>
-    <hyperlink ref="A34" r:id="rId33"/>
-    <hyperlink ref="A35" r:id="rId34"/>
-    <hyperlink ref="A36" r:id="rId35"/>
-    <hyperlink ref="A37" r:id="rId36"/>
-    <hyperlink ref="A38" r:id="rId37"/>
-    <hyperlink ref="A39" r:id="rId38"/>
-    <hyperlink ref="A40" r:id="rId39"/>
-    <hyperlink ref="A41" r:id="rId40"/>
-    <hyperlink ref="A42" r:id="rId41"/>
-    <hyperlink ref="A43" r:id="rId42"/>
-    <hyperlink ref="A44" r:id="rId43"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-06-15 16:49
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3837" uniqueCount="1845">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3857" uniqueCount="1853">
   <si>
     <t>link</t>
   </si>
@@ -5553,6 +5553,30 @@
   </si>
   <si>
     <t>84960070140</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/ilzenes-pag/coilm.html</t>
+  </si>
+  <si>
+    <t>20.50 ha.</t>
+  </si>
+  <si>
+    <t>36520050104</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/aulejas-pag/hjddo.html</t>
+  </si>
+  <si>
+    <t>60480040017</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/ezernieku-pag/hiffg.html</t>
+  </si>
+  <si>
+    <t>60560070179</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/indranu-pag/obhbd.html</t>
   </si>
 </sst>
 </file>
@@ -5965,7 +5989,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F764"/>
+  <dimension ref="A1:F766"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -21254,6 +21278,46 @@
       </c>
       <c r="F764" s="2">
         <v>46184.45208333334</v>
+      </c>
+    </row>
+    <row r="765" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A765" s="3" t="s">
+        <v>1840</v>
+      </c>
+      <c r="B765" s="4" t="s">
+        <v>549</v>
+      </c>
+      <c r="C765" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D765" s="4" t="s">
+        <v>1841</v>
+      </c>
+      <c r="E765" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F765" s="2">
+        <v>46184.80208333333</v>
+      </c>
+    </row>
+    <row r="766" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A766" s="3" t="s">
+        <v>1842</v>
+      </c>
+      <c r="B766" s="4" t="s">
+        <v>1843</v>
+      </c>
+      <c r="C766" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="D766" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E766" s="4" t="s">
+        <v>1844</v>
+      </c>
+      <c r="F766" s="2">
+        <v>46185.3</v>
       </c>
     </row>
   </sheetData>
@@ -22021,6 +22085,8 @@
     <hyperlink ref="A762" r:id="rId761"/>
     <hyperlink ref="A763" r:id="rId762"/>
     <hyperlink ref="A764" r:id="rId763"/>
+    <hyperlink ref="A765" r:id="rId764"/>
+    <hyperlink ref="A766" r:id="rId765"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -22032,7 +22098,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22065,48 +22131,90 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1840</v>
+        <v>1845</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>549</v>
+        <v>27</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>63</v>
+        <v>435</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>1841</v>
+        <v>1846</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>25</v>
+        <v>1847</v>
       </c>
       <c r="F2" s="2">
-        <v>46184.80208333333</v>
+        <v>46187.28680555556</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1842</v>
+        <v>1848</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>1843</v>
+        <v>417</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>346</v>
+        <v>146</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>32</v>
+        <v>272</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1844</v>
+        <v>1849</v>
       </c>
       <c r="F3" s="2">
-        <v>46185.3</v>
+        <v>46188.481944444444</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1850</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>737</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1851</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46186.87847222222</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1852</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>956</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>730</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46185.88680555555</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-06-16 16:18
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3857" uniqueCount="1853">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3867" uniqueCount="1856">
   <si>
     <t>link</t>
   </si>
@@ -5577,6 +5577,15 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/indranu-pag/obhbd.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/raiskuma-pag/higjh.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/limbadzi-and-reg/limbazu-pag/aieep.html</t>
+  </si>
+  <si>
+    <t>66800060114</t>
   </si>
 </sst>
 </file>
@@ -5989,7 +5998,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F766"/>
+  <dimension ref="A1:F770"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -21318,6 +21327,86 @@
       </c>
       <c r="F766" s="2">
         <v>46185.3</v>
+      </c>
+    </row>
+    <row r="767" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A767" s="3" t="s">
+        <v>1845</v>
+      </c>
+      <c r="B767" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C767" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D767" s="4" t="s">
+        <v>1846</v>
+      </c>
+      <c r="E767" s="4" t="s">
+        <v>1847</v>
+      </c>
+      <c r="F767" s="2">
+        <v>46187.28680555556</v>
+      </c>
+    </row>
+    <row r="768" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A768" s="3" t="s">
+        <v>1848</v>
+      </c>
+      <c r="B768" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="C768" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D768" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E768" s="4" t="s">
+        <v>1849</v>
+      </c>
+      <c r="F768" s="2">
+        <v>46188.481944444444</v>
+      </c>
+    </row>
+    <row r="769" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A769" s="3" t="s">
+        <v>1850</v>
+      </c>
+      <c r="B769" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="C769" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D769" s="4" t="s">
+        <v>737</v>
+      </c>
+      <c r="E769" s="4" t="s">
+        <v>1851</v>
+      </c>
+      <c r="F769" s="2">
+        <v>46186.87847222222</v>
+      </c>
+    </row>
+    <row r="770" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A770" s="3" t="s">
+        <v>1852</v>
+      </c>
+      <c r="B770" s="4" t="s">
+        <v>956</v>
+      </c>
+      <c r="C770" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D770" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E770" s="4" t="s">
+        <v>730</v>
+      </c>
+      <c r="F770" s="2">
+        <v>46185.88680555555</v>
       </c>
     </row>
   </sheetData>
@@ -22087,6 +22176,10 @@
     <hyperlink ref="A764" r:id="rId763"/>
     <hyperlink ref="A765" r:id="rId764"/>
     <hyperlink ref="A766" r:id="rId765"/>
+    <hyperlink ref="A767" r:id="rId766"/>
+    <hyperlink ref="A768" r:id="rId767"/>
+    <hyperlink ref="A769" r:id="rId768"/>
+    <hyperlink ref="A770" r:id="rId769"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -22098,7 +22191,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22131,90 +22224,48 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1845</v>
+        <v>1853</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>27</v>
+        <v>106</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>435</v>
+        <v>63</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>1846</v>
+        <v>24</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1847</v>
+        <v>1636</v>
       </c>
       <c r="F2" s="2">
-        <v>46187.28680555556</v>
+        <v>46189.61458333333</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1848</v>
+        <v>1854</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>417</v>
+        <v>271</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>146</v>
+        <v>208</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>272</v>
+        <v>930</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1849</v>
+        <v>1855</v>
       </c>
       <c r="F3" s="2">
-        <v>46188.481944444444</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1850</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>576</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>737</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1851</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46186.87847222222</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1852</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>956</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>730</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46185.88680555555</v>
+        <v>46188.90486111111</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-06-17 14:45
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3867" uniqueCount="1856">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3872" uniqueCount="1858">
   <si>
     <t>link</t>
   </si>
@@ -5586,6 +5586,12 @@
   </si>
   <si>
     <t>66800060114</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/liksnas-pag/jiojj.html</t>
+  </si>
+  <si>
+    <t>44680060585</t>
   </si>
 </sst>
 </file>
@@ -5998,7 +6004,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F770"/>
+  <dimension ref="A1:F772"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -21407,6 +21413,46 @@
       </c>
       <c r="F770" s="2">
         <v>46185.88680555555</v>
+      </c>
+    </row>
+    <row r="771" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A771" s="3" t="s">
+        <v>1853</v>
+      </c>
+      <c r="B771" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C771" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D771" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E771" s="4" t="s">
+        <v>1636</v>
+      </c>
+      <c r="F771" s="2">
+        <v>46189.61458333333</v>
+      </c>
+    </row>
+    <row r="772" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A772" s="3" t="s">
+        <v>1854</v>
+      </c>
+      <c r="B772" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="C772" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D772" s="4" t="s">
+        <v>930</v>
+      </c>
+      <c r="E772" s="4" t="s">
+        <v>1855</v>
+      </c>
+      <c r="F772" s="2">
+        <v>46188.90486111111</v>
       </c>
     </row>
   </sheetData>
@@ -22180,6 +22226,8 @@
     <hyperlink ref="A768" r:id="rId767"/>
     <hyperlink ref="A769" r:id="rId768"/>
     <hyperlink ref="A770" r:id="rId769"/>
+    <hyperlink ref="A771" r:id="rId770"/>
+    <hyperlink ref="A772" r:id="rId771"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -22191,7 +22239,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22224,48 +22272,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1853</v>
+        <v>1856</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>106</v>
+        <v>969</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>24</v>
+        <v>186</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1636</v>
+        <v>1857</v>
       </c>
       <c r="F2" s="2">
-        <v>46189.61458333333</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1854</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>930</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1855</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46188.90486111111</v>
+        <v>46190.72708333333</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-06-18 14:39
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -6004,7 +6004,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F772"/>
+  <dimension ref="A1:F773"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -21453,6 +21453,26 @@
       </c>
       <c r="F772" s="2">
         <v>46188.90486111111</v>
+      </c>
+    </row>
+    <row r="773" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A773" s="3" t="s">
+        <v>1856</v>
+      </c>
+      <c r="B773" s="4" t="s">
+        <v>969</v>
+      </c>
+      <c r="C773" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D773" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E773" s="4" t="s">
+        <v>1857</v>
+      </c>
+      <c r="F773" s="2">
+        <v>46190.72708333333</v>
       </c>
     </row>
   </sheetData>
@@ -22228,6 +22248,7 @@
     <hyperlink ref="A770" r:id="rId769"/>
     <hyperlink ref="A771" r:id="rId770"/>
     <hyperlink ref="A772" r:id="rId771"/>
+    <hyperlink ref="A773" r:id="rId772"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -22239,7 +22260,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22270,30 +22291,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>1856</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>969</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>1857</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46190.72708333333</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-06-19 14:36
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3872" uniqueCount="1858">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3877" uniqueCount="1861">
   <si>
     <t>link</t>
   </si>
@@ -5592,6 +5592,15 @@
   </si>
   <si>
     <t>44680060585</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/indranu-pag/bmijol.html</t>
+  </si>
+  <si>
+    <t>15.20 ha.</t>
+  </si>
+  <si>
+    <t>70580010025</t>
   </si>
 </sst>
 </file>
@@ -22260,7 +22269,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22291,7 +22300,30 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>1858</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>1859</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>1860</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46192.3875</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-06-22 16:22
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -6013,7 +6013,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F773"/>
+  <dimension ref="A1:F774"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -21482,6 +21482,26 @@
       </c>
       <c r="F773" s="2">
         <v>46190.72708333333</v>
+      </c>
+    </row>
+    <row r="774" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A774" s="3" t="s">
+        <v>1858</v>
+      </c>
+      <c r="B774" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="C774" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D774" s="4" t="s">
+        <v>1859</v>
+      </c>
+      <c r="E774" s="4" t="s">
+        <v>1860</v>
+      </c>
+      <c r="F774" s="2">
+        <v>46192.3875</v>
       </c>
     </row>
   </sheetData>
@@ -22258,6 +22278,7 @@
     <hyperlink ref="A771" r:id="rId770"/>
     <hyperlink ref="A772" r:id="rId771"/>
     <hyperlink ref="A773" r:id="rId772"/>
+    <hyperlink ref="A774" r:id="rId773"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -22269,7 +22290,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22300,30 +22321,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>1858</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>1859</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>1860</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46192.3875</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-06-23 14:14
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3877" uniqueCount="1861">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3882" uniqueCount="1862">
   <si>
     <t>link</t>
   </si>
@@ -5601,6 +5601,9 @@
   </si>
   <si>
     <t>70580010025</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/talsi-and-reg/rojas-pag/bpglx.html</t>
   </si>
 </sst>
 </file>
@@ -22290,7 +22293,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22321,7 +22324,30 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>1861</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46196.674305555556</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-06-24 14:00
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -6016,7 +6016,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F774"/>
+  <dimension ref="A1:F775"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -21505,6 +21505,26 @@
       </c>
       <c r="F774" s="2">
         <v>46192.3875</v>
+      </c>
+    </row>
+    <row r="775" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A775" s="3" t="s">
+        <v>1861</v>
+      </c>
+      <c r="B775" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C775" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="D775" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E775" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F775" s="2">
+        <v>46196.674305555556</v>
       </c>
     </row>
   </sheetData>
@@ -22282,6 +22302,7 @@
     <hyperlink ref="A772" r:id="rId771"/>
     <hyperlink ref="A773" r:id="rId772"/>
     <hyperlink ref="A774" r:id="rId773"/>
+    <hyperlink ref="A775" r:id="rId774"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -22293,7 +22314,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22324,30 +22345,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>1861</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>356</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46196.674305555556</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-06-25 13:57
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3882" uniqueCount="1862">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3887" uniqueCount="1865">
   <si>
     <t>link</t>
   </si>
@@ -5604,6 +5604,15 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/talsi-and-reg/rojas-pag/bpglx.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/marcienas-pag/fkkoh.html</t>
+  </si>
+  <si>
+    <t>200 000 €</t>
+  </si>
+  <si>
+    <t>70740040013</t>
   </si>
 </sst>
 </file>
@@ -22314,7 +22323,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22345,7 +22354,30 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>1862</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>1863</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>1864</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46198.024305555555</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-06-26 13:55
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -6025,7 +6025,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F775"/>
+  <dimension ref="A1:F776"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -21534,6 +21534,26 @@
       </c>
       <c r="F775" s="2">
         <v>46196.674305555556</v>
+      </c>
+    </row>
+    <row r="776" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A776" s="3" t="s">
+        <v>1862</v>
+      </c>
+      <c r="B776" s="4" t="s">
+        <v>1863</v>
+      </c>
+      <c r="C776" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D776" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E776" s="4" t="s">
+        <v>1864</v>
+      </c>
+      <c r="F776" s="2">
+        <v>46198.024305555555</v>
       </c>
     </row>
   </sheetData>
@@ -22312,6 +22332,7 @@
     <hyperlink ref="A773" r:id="rId772"/>
     <hyperlink ref="A774" r:id="rId773"/>
     <hyperlink ref="A775" r:id="rId774"/>
+    <hyperlink ref="A776" r:id="rId775"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -22323,7 +22344,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22354,30 +22375,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>1862</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>1863</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>1864</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46198.024305555555</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-06-29 15:24
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3887" uniqueCount="1865">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3912" uniqueCount="1876">
   <si>
     <t>link</t>
   </si>
@@ -5613,6 +5613,39 @@
   </si>
   <si>
     <t>70740040013</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/dubnas-pag/iphlh.html</t>
+  </si>
+  <si>
+    <t>44520010078</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/daugavpils/dcmog.html</t>
+  </si>
+  <si>
+    <t>44700010122</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/limbadzi-and-reg/limbazi/fgxep.html</t>
+  </si>
+  <si>
+    <t>55 €</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/ilzeskalna-pag/bdngeb.html</t>
+  </si>
+  <si>
+    <t>1.11 ha.</t>
+  </si>
+  <si>
+    <t>78580050435</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ventspils-and-reg/targales-pag/pgcgn.html</t>
+  </si>
+  <si>
+    <t>98660220032</t>
   </si>
 </sst>
 </file>
@@ -22344,7 +22377,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22375,7 +22408,114 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>1865</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>1866</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46202.513194444444</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1867</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1868</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46201.41666666667</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1869</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>1870</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46202.43958333333</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>1872</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1873</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46201.04375</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>1874</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>1875</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46202.606944444444</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+    <hyperlink ref="A6" r:id="rId5"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-06-30 13:49
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3912" uniqueCount="1876">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3917" uniqueCount="1878">
   <si>
     <t>link</t>
   </si>
@@ -5646,6 +5646,12 @@
   </si>
   <si>
     <t>98660220032</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/bauska-and-reg/other/pknog.html</t>
+  </si>
+  <si>
+    <t>32620040077</t>
   </si>
 </sst>
 </file>
@@ -6058,7 +6064,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F776"/>
+  <dimension ref="A1:F781"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -21587,6 +21593,106 @@
       </c>
       <c r="F776" s="2">
         <v>46198.024305555555</v>
+      </c>
+    </row>
+    <row r="777" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A777" s="3" t="s">
+        <v>1865</v>
+      </c>
+      <c r="B777" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C777" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D777" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E777" s="4" t="s">
+        <v>1866</v>
+      </c>
+      <c r="F777" s="2">
+        <v>46202.513194444444</v>
+      </c>
+    </row>
+    <row r="778" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A778" s="3" t="s">
+        <v>1867</v>
+      </c>
+      <c r="B778" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="C778" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D778" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E778" s="4" t="s">
+        <v>1868</v>
+      </c>
+      <c r="F778" s="2">
+        <v>46201.41666666667</v>
+      </c>
+    </row>
+    <row r="779" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A779" s="3" t="s">
+        <v>1869</v>
+      </c>
+      <c r="B779" s="4" t="s">
+        <v>1870</v>
+      </c>
+      <c r="C779" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D779" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="E779" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F779" s="2">
+        <v>46202.43958333333</v>
+      </c>
+    </row>
+    <row r="780" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A780" s="3" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B780" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="C780" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D780" s="4" t="s">
+        <v>1872</v>
+      </c>
+      <c r="E780" s="4" t="s">
+        <v>1873</v>
+      </c>
+      <c r="F780" s="2">
+        <v>46201.04375</v>
+      </c>
+    </row>
+    <row r="781" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A781" s="3" t="s">
+        <v>1874</v>
+      </c>
+      <c r="B781" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C781" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D781" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E781" s="4" t="s">
+        <v>1875</v>
+      </c>
+      <c r="F781" s="2">
+        <v>46202.606944444444</v>
       </c>
     </row>
   </sheetData>
@@ -22366,6 +22472,11 @@
     <hyperlink ref="A774" r:id="rId773"/>
     <hyperlink ref="A775" r:id="rId774"/>
     <hyperlink ref="A776" r:id="rId775"/>
+    <hyperlink ref="A777" r:id="rId776"/>
+    <hyperlink ref="A778" r:id="rId777"/>
+    <hyperlink ref="A779" r:id="rId778"/>
+    <hyperlink ref="A780" r:id="rId779"/>
+    <hyperlink ref="A781" r:id="rId780"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -22377,7 +22488,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22410,111 +22521,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1865</v>
+        <v>1876</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>52</v>
+        <v>745</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>82</v>
+        <v>135</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1866</v>
+        <v>1877</v>
       </c>
       <c r="F2" s="2">
-        <v>46202.513194444444</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1867</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>274</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1868</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46201.41666666667</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1869</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>1870</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46202.43958333333</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1871</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>576</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>1872</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1873</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46201.04375</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>1874</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>404</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>1875</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46202.606944444444</v>
+        <v>46203.59375</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-07-01 14:00
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3917" uniqueCount="1878">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3922" uniqueCount="1880">
   <si>
     <t>link</t>
   </si>
@@ -5652,6 +5652,12 @@
   </si>
   <si>
     <t>32620040077</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/varkavas-pag/kmxgx.html</t>
+  </si>
+  <si>
+    <t>76940010474</t>
   </si>
 </sst>
 </file>
@@ -6064,7 +6070,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F781"/>
+  <dimension ref="A1:F782"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -21693,6 +21699,26 @@
       </c>
       <c r="F781" s="2">
         <v>46202.606944444444</v>
+      </c>
+    </row>
+    <row r="782" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A782" s="3" t="s">
+        <v>1876</v>
+      </c>
+      <c r="B782" s="4" t="s">
+        <v>745</v>
+      </c>
+      <c r="C782" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D782" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E782" s="4" t="s">
+        <v>1877</v>
+      </c>
+      <c r="F782" s="2">
+        <v>46203.59375</v>
       </c>
     </row>
   </sheetData>
@@ -22477,6 +22503,7 @@
     <hyperlink ref="A779" r:id="rId778"/>
     <hyperlink ref="A780" r:id="rId779"/>
     <hyperlink ref="A781" r:id="rId780"/>
+    <hyperlink ref="A782" r:id="rId781"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -22521,22 +22548,22 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1876</v>
+        <v>1878</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>745</v>
+        <v>793</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>48</v>
+        <v>284</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>135</v>
+        <v>82</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1877</v>
+        <v>1879</v>
       </c>
       <c r="F2" s="2">
-        <v>46203.59375</v>
+        <v>46204.40416666667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-07-02 13:25
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3922" uniqueCount="1880">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3942" uniqueCount="1888">
   <si>
     <t>link</t>
   </si>
@@ -5658,6 +5658,30 @@
   </si>
   <si>
     <t>76940010474</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aizkraukle-and-reg/bebru-pag/dlfjb.html</t>
+  </si>
+  <si>
+    <t>32460010024</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/kombulu-pag/bhbdeh.html</t>
+  </si>
+  <si>
+    <t>60740040147</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/talsi-and-reg/dundagas-pag/apbim.html</t>
+  </si>
+  <si>
+    <t>88500110029</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ventspils-and-reg/ances-pag/anoij.html</t>
+  </si>
+  <si>
+    <t>98440080005</t>
   </si>
 </sst>
 </file>
@@ -6070,7 +6094,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F782"/>
+  <dimension ref="A1:F783"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -21719,6 +21743,26 @@
       </c>
       <c r="F782" s="2">
         <v>46203.59375</v>
+      </c>
+    </row>
+    <row r="783" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A783" s="3" t="s">
+        <v>1878</v>
+      </c>
+      <c r="B783" s="4" t="s">
+        <v>793</v>
+      </c>
+      <c r="C783" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D783" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E783" s="4" t="s">
+        <v>1879</v>
+      </c>
+      <c r="F783" s="2">
+        <v>46204.40416666667</v>
       </c>
     </row>
   </sheetData>
@@ -22504,6 +22548,7 @@
     <hyperlink ref="A780" r:id="rId779"/>
     <hyperlink ref="A781" r:id="rId780"/>
     <hyperlink ref="A782" r:id="rId781"/>
+    <hyperlink ref="A783" r:id="rId782"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -22515,7 +22560,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22548,27 +22593,90 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1878</v>
+        <v>1880</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>793</v>
+        <v>88</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>284</v>
+        <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>82</v>
+        <v>1841</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1879</v>
+        <v>1881</v>
       </c>
       <c r="F2" s="2">
-        <v>46204.40416666667</v>
+        <v>46205.28125</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1882</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>1557</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>670</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1883</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46205.57083333333</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1884</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1885</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46205.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1886</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>876</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1887</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46205.51458333334</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-07-03 13:28
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -6094,7 +6094,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F783"/>
+  <dimension ref="A1:F787"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -21763,6 +21763,86 @@
       </c>
       <c r="F783" s="2">
         <v>46204.40416666667</v>
+      </c>
+    </row>
+    <row r="784" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A784" s="3" t="s">
+        <v>1880</v>
+      </c>
+      <c r="B784" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C784" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D784" s="4" t="s">
+        <v>1841</v>
+      </c>
+      <c r="E784" s="4" t="s">
+        <v>1881</v>
+      </c>
+      <c r="F784" s="2">
+        <v>46205.28125</v>
+      </c>
+    </row>
+    <row r="785" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A785" s="3" t="s">
+        <v>1882</v>
+      </c>
+      <c r="B785" s="4" t="s">
+        <v>1557</v>
+      </c>
+      <c r="C785" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D785" s="4" t="s">
+        <v>670</v>
+      </c>
+      <c r="E785" s="4" t="s">
+        <v>1883</v>
+      </c>
+      <c r="F785" s="2">
+        <v>46205.57083333333</v>
+      </c>
+    </row>
+    <row r="786" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A786" s="3" t="s">
+        <v>1884</v>
+      </c>
+      <c r="B786" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="C786" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="D786" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E786" s="4" t="s">
+        <v>1885</v>
+      </c>
+      <c r="F786" s="2">
+        <v>46205.5</v>
+      </c>
+    </row>
+    <row r="787" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A787" s="3" t="s">
+        <v>1886</v>
+      </c>
+      <c r="B787" s="4" t="s">
+        <v>876</v>
+      </c>
+      <c r="C787" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D787" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E787" s="4" t="s">
+        <v>1887</v>
+      </c>
+      <c r="F787" s="2">
+        <v>46205.51458333334</v>
       </c>
     </row>
   </sheetData>
@@ -22549,6 +22629,10 @@
     <hyperlink ref="A781" r:id="rId780"/>
     <hyperlink ref="A782" r:id="rId781"/>
     <hyperlink ref="A783" r:id="rId782"/>
+    <hyperlink ref="A784" r:id="rId783"/>
+    <hyperlink ref="A785" r:id="rId784"/>
+    <hyperlink ref="A786" r:id="rId785"/>
+    <hyperlink ref="A787" r:id="rId786"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -22560,7 +22644,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22591,93 +22675,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>1880</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>1841</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>1881</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46205.28125</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1882</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>1557</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>670</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1883</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46205.57083333333</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1884</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>356</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1885</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46205.5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1886</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>876</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>404</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1887</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46205.51458333334</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-07-06 14:51
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3942" uniqueCount="1888">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3962" uniqueCount="1896">
   <si>
     <t>link</t>
   </si>
@@ -5682,6 +5682,30 @@
   </si>
   <si>
     <t>98440080005</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/ezernieku-pag/mhdim.html</t>
+  </si>
+  <si>
+    <t>60560040044</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/kastulinas-pag/fhkxp.html</t>
+  </si>
+  <si>
+    <t>60720070059</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/aglonas-pag/anjko.html</t>
+  </si>
+  <si>
+    <t>76420040221</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/kaunatas-pag/lenoe.html</t>
+  </si>
+  <si>
+    <t>78620110036</t>
   </si>
 </sst>
 </file>
@@ -22644,7 +22668,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22675,7 +22699,93 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>1888</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>793</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>1889</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46209.53472222222</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1890</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1891</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46207.975694444445</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1892</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1893</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46207.773611111115</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1894</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>562</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1895</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46208.625</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-07-07 14:00
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3962" uniqueCount="1896">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3967" uniqueCount="1898">
   <si>
     <t>link</t>
   </si>
@@ -5706,6 +5706,12 @@
   </si>
   <si>
     <t>78620110036</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/tukums-and-reg/viesatu-pag/micnb.html</t>
+  </si>
+  <si>
+    <t>90900020168</t>
   </si>
 </sst>
 </file>
@@ -6118,7 +6124,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F787"/>
+  <dimension ref="A1:F791"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -21867,6 +21873,86 @@
       </c>
       <c r="F787" s="2">
         <v>46205.51458333334</v>
+      </c>
+    </row>
+    <row r="788" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A788" s="3" t="s">
+        <v>1888</v>
+      </c>
+      <c r="B788" s="4" t="s">
+        <v>793</v>
+      </c>
+      <c r="C788" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D788" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E788" s="4" t="s">
+        <v>1889</v>
+      </c>
+      <c r="F788" s="2">
+        <v>46209.53472222222</v>
+      </c>
+    </row>
+    <row r="789" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A789" s="3" t="s">
+        <v>1890</v>
+      </c>
+      <c r="B789" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C789" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D789" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E789" s="4" t="s">
+        <v>1891</v>
+      </c>
+      <c r="F789" s="2">
+        <v>46207.975694444445</v>
+      </c>
+    </row>
+    <row r="790" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A790" s="3" t="s">
+        <v>1892</v>
+      </c>
+      <c r="B790" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C790" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D790" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E790" s="4" t="s">
+        <v>1893</v>
+      </c>
+      <c r="F790" s="2">
+        <v>46207.773611111115</v>
+      </c>
+    </row>
+    <row r="791" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A791" s="3" t="s">
+        <v>1894</v>
+      </c>
+      <c r="B791" s="4" t="s">
+        <v>562</v>
+      </c>
+      <c r="C791" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D791" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E791" s="4" t="s">
+        <v>1895</v>
+      </c>
+      <c r="F791" s="2">
+        <v>46208.625</v>
       </c>
     </row>
   </sheetData>
@@ -22657,6 +22743,10 @@
     <hyperlink ref="A785" r:id="rId784"/>
     <hyperlink ref="A786" r:id="rId785"/>
     <hyperlink ref="A787" r:id="rId786"/>
+    <hyperlink ref="A788" r:id="rId787"/>
+    <hyperlink ref="A789" r:id="rId788"/>
+    <hyperlink ref="A790" r:id="rId789"/>
+    <hyperlink ref="A791" r:id="rId790"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -22668,7 +22758,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22701,90 +22791,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1888</v>
+        <v>1896</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>793</v>
+        <v>23</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>146</v>
+        <v>376</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>272</v>
+        <v>918</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1889</v>
+        <v>1897</v>
       </c>
       <c r="F2" s="2">
-        <v>46209.53472222222</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1890</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1891</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46207.975694444445</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1892</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1893</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46207.773611111115</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1894</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>562</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1895</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46208.625</v>
+        <v>46210.43402777778</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-07-08 13:23
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3967" uniqueCount="1898">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3977" uniqueCount="1904">
   <si>
     <t>link</t>
   </si>
@@ -5712,6 +5712,24 @@
   </si>
   <si>
     <t>90900020168</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/mezares-pag/bbmbjo.html</t>
+  </si>
+  <si>
+    <t>1.34 ha.</t>
+  </si>
+  <si>
+    <t>56760060018</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valmiera-and-reg/ramatas-pag/akxjd.html</t>
+  </si>
+  <si>
+    <t>8.80 ha.</t>
+  </si>
+  <si>
+    <t>96760060032</t>
   </si>
 </sst>
 </file>
@@ -6124,7 +6142,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F791"/>
+  <dimension ref="A1:F792"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -21953,6 +21971,26 @@
       </c>
       <c r="F791" s="2">
         <v>46208.625</v>
+      </c>
+    </row>
+    <row r="792" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A792" s="3" t="s">
+        <v>1896</v>
+      </c>
+      <c r="B792" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C792" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D792" s="4" t="s">
+        <v>918</v>
+      </c>
+      <c r="E792" s="4" t="s">
+        <v>1897</v>
+      </c>
+      <c r="F792" s="2">
+        <v>46210.43402777778</v>
       </c>
     </row>
   </sheetData>
@@ -22747,6 +22785,7 @@
     <hyperlink ref="A789" r:id="rId788"/>
     <hyperlink ref="A790" r:id="rId789"/>
     <hyperlink ref="A791" r:id="rId790"/>
+    <hyperlink ref="A792" r:id="rId791"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -22758,7 +22797,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22791,27 +22830,48 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1896</v>
+        <v>1898</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>23</v>
+        <v>131</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>376</v>
+        <v>127</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>918</v>
+        <v>1899</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1897</v>
+        <v>1900</v>
       </c>
       <c r="F2" s="2">
-        <v>46210.43402777778</v>
+        <v>46211.50138888889</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1901</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>1902</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1903</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46211.40972222222</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-07-09 14:24
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3977" uniqueCount="1904">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3982" uniqueCount="1905">
   <si>
     <t>link</t>
   </si>
@@ -5730,6 +5730,9 @@
   </si>
   <si>
     <t>96760060032</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/madona/llbef.html</t>
   </si>
 </sst>
 </file>
@@ -6142,7 +6145,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F792"/>
+  <dimension ref="A1:F794"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -21991,6 +21994,46 @@
       </c>
       <c r="F792" s="2">
         <v>46210.43402777778</v>
+      </c>
+    </row>
+    <row r="793" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A793" s="3" t="s">
+        <v>1898</v>
+      </c>
+      <c r="B793" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C793" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D793" s="4" t="s">
+        <v>1899</v>
+      </c>
+      <c r="E793" s="4" t="s">
+        <v>1900</v>
+      </c>
+      <c r="F793" s="2">
+        <v>46211.50138888889</v>
+      </c>
+    </row>
+    <row r="794" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A794" s="3" t="s">
+        <v>1901</v>
+      </c>
+      <c r="B794" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C794" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D794" s="4" t="s">
+        <v>1902</v>
+      </c>
+      <c r="E794" s="4" t="s">
+        <v>1903</v>
+      </c>
+      <c r="F794" s="2">
+        <v>46211.40972222222</v>
       </c>
     </row>
   </sheetData>
@@ -22786,6 +22829,8 @@
     <hyperlink ref="A790" r:id="rId789"/>
     <hyperlink ref="A791" r:id="rId790"/>
     <hyperlink ref="A792" r:id="rId791"/>
+    <hyperlink ref="A793" r:id="rId792"/>
+    <hyperlink ref="A794" r:id="rId793"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -22797,7 +22842,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22830,48 +22875,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1898</v>
+        <v>1904</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>131</v>
+        <v>268</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>127</v>
+        <v>256</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>1899</v>
+        <v>154</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1900</v>
+        <v>654</v>
       </c>
       <c r="F2" s="2">
-        <v>46211.50138888889</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1901</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>1902</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1903</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46211.40972222222</v>
+        <v>46212.40694444445</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-07-10 13:50
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3982" uniqueCount="1905">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3997" uniqueCount="1913">
   <si>
     <t>link</t>
   </si>
@@ -5733,6 +5733,30 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/madona/llbef.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kuldiga-and-reg/edoles-pag/bgkgcb.html</t>
+  </si>
+  <si>
+    <t>5.13 ha.</t>
+  </si>
+  <si>
+    <t>62460090076</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/ozolaines-pag/gjdbn.html</t>
+  </si>
+  <si>
+    <t>78760060439/0438</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/saldus-and-reg/jaunlutrinu-pag/jkjfe.html</t>
+  </si>
+  <si>
+    <t>22 300 €</t>
+  </si>
+  <si>
+    <t>845880020006</t>
   </si>
 </sst>
 </file>
@@ -6145,7 +6169,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F794"/>
+  <dimension ref="A1:F795"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22034,6 +22058,26 @@
       </c>
       <c r="F794" s="2">
         <v>46211.40972222222</v>
+      </c>
+    </row>
+    <row r="795" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A795" s="3" t="s">
+        <v>1904</v>
+      </c>
+      <c r="B795" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="C795" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D795" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="E795" s="4" t="s">
+        <v>654</v>
+      </c>
+      <c r="F795" s="2">
+        <v>46212.40694444445</v>
       </c>
     </row>
   </sheetData>
@@ -22831,6 +22875,7 @@
     <hyperlink ref="A792" r:id="rId791"/>
     <hyperlink ref="A793" r:id="rId792"/>
     <hyperlink ref="A794" r:id="rId793"/>
+    <hyperlink ref="A795" r:id="rId794"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -22842,7 +22887,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22875,27 +22920,69 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1904</v>
+        <v>1905</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>268</v>
+        <v>161</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>256</v>
+        <v>424</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>154</v>
+        <v>1906</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>654</v>
+        <v>1907</v>
       </c>
       <c r="F2" s="2">
-        <v>46212.40694444445</v>
+        <v>46212.72916666667</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1908</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>497</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>1575</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1909</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46213.69305555556</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1910</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>1911</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1912</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46212.73611111111</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-07-13 13:56
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3997" uniqueCount="1913">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4027" uniqueCount="1929">
   <si>
     <t>link</t>
   </si>
@@ -5757,6 +5757,54 @@
   </si>
   <si>
     <t>845880020006</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/berzpils-pag/nhfcb.html</t>
+  </si>
+  <si>
+    <t>9.30 ha.</t>
+  </si>
+  <si>
+    <t>38500040151</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/skujenes-pag/gffcg.html</t>
+  </si>
+  <si>
+    <t>60 ha.</t>
+  </si>
+  <si>
+    <t>427800080044</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/kalsnavas-pag/plhdk.html</t>
+  </si>
+  <si>
+    <t>14 500 €</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/dricanu-pag/jlnde.html</t>
+  </si>
+  <si>
+    <t>16 450 €</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valka-and-reg/trikatas-pag/nildb.html</t>
+  </si>
+  <si>
+    <t>8.90 ha.</t>
+  </si>
+  <si>
+    <t>94840020044</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valka-and-reg/trikatas-pag/jlkcx.html</t>
+  </si>
+  <si>
+    <t>27 500 €</t>
+  </si>
+  <si>
+    <t>94840020042</t>
   </si>
 </sst>
 </file>
@@ -6169,7 +6217,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F795"/>
+  <dimension ref="A1:F798"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22078,6 +22126,66 @@
       </c>
       <c r="F795" s="2">
         <v>46212.40694444445</v>
+      </c>
+    </row>
+    <row r="796" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A796" s="3" t="s">
+        <v>1905</v>
+      </c>
+      <c r="B796" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C796" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="D796" s="4" t="s">
+        <v>1906</v>
+      </c>
+      <c r="E796" s="4" t="s">
+        <v>1907</v>
+      </c>
+      <c r="F796" s="2">
+        <v>46212.72916666667</v>
+      </c>
+    </row>
+    <row r="797" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A797" s="3" t="s">
+        <v>1908</v>
+      </c>
+      <c r="B797" s="4" t="s">
+        <v>497</v>
+      </c>
+      <c r="C797" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D797" s="4" t="s">
+        <v>1575</v>
+      </c>
+      <c r="E797" s="4" t="s">
+        <v>1909</v>
+      </c>
+      <c r="F797" s="2">
+        <v>46213.69305555556</v>
+      </c>
+    </row>
+    <row r="798" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A798" s="3" t="s">
+        <v>1910</v>
+      </c>
+      <c r="B798" s="4" t="s">
+        <v>1911</v>
+      </c>
+      <c r="C798" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="D798" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E798" s="4" t="s">
+        <v>1912</v>
+      </c>
+      <c r="F798" s="2">
+        <v>46212.73611111111</v>
       </c>
     </row>
   </sheetData>
@@ -22876,6 +22984,9 @@
     <hyperlink ref="A793" r:id="rId792"/>
     <hyperlink ref="A794" r:id="rId793"/>
     <hyperlink ref="A795" r:id="rId794"/>
+    <hyperlink ref="A796" r:id="rId795"/>
+    <hyperlink ref="A797" r:id="rId796"/>
+    <hyperlink ref="A798" r:id="rId797"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -22887,7 +22998,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22920,62 +23031,122 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1905</v>
+        <v>1913</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>161</v>
+        <v>27</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>424</v>
+        <v>28</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>1906</v>
+        <v>1914</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1907</v>
+        <v>1915</v>
       </c>
       <c r="F2" s="2">
-        <v>46212.72916666667</v>
+        <v>46216.007638888885</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1908</v>
+        <v>1916</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>497</v>
+        <v>325</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>294</v>
+        <v>63</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>1575</v>
+        <v>1917</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1909</v>
+        <v>1918</v>
       </c>
       <c r="F3" s="2">
-        <v>46213.69305555556</v>
+        <v>46216.59375</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>1910</v>
+        <v>1919</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>1911</v>
+        <v>1920</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>346</v>
+        <v>256</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>186</v>
+        <v>1730</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>1912</v>
+        <v>25</v>
       </c>
       <c r="F4" s="2">
-        <v>46212.73611111111</v>
+        <v>46213.70625</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1921</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>1922</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1178</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46214.711805555555</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>1923</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>1924</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>1925</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46215.46805555555</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>1926</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>1927</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>1928</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46215.464583333334</v>
       </c>
     </row>
   </sheetData>
@@ -22983,6 +23154,9 @@
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
     <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+    <hyperlink ref="A6" r:id="rId5"/>
+    <hyperlink ref="A7" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-07-14 13:00
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4027" uniqueCount="1929">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4042" uniqueCount="1937">
   <si>
     <t>link</t>
   </si>
@@ -5805,6 +5805,30 @@
   </si>
   <si>
     <t>94840020042</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/marsnenu-pag/njpjx.html</t>
+  </si>
+  <si>
+    <t>25 500 €</t>
+  </si>
+  <si>
+    <t>42640030074</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ogre-and-reg/keipenes-pag/demcc.html</t>
+  </si>
+  <si>
+    <t>74560050055</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/rozkalnu-pag/phbkc.html</t>
+  </si>
+  <si>
+    <t>12 345 €</t>
+  </si>
+  <si>
+    <t>76640020054</t>
   </si>
 </sst>
 </file>
@@ -6217,7 +6241,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F798"/>
+  <dimension ref="A1:F804"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22186,6 +22210,126 @@
       </c>
       <c r="F798" s="2">
         <v>46212.73611111111</v>
+      </c>
+    </row>
+    <row r="799" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A799" s="3" t="s">
+        <v>1913</v>
+      </c>
+      <c r="B799" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C799" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D799" s="4" t="s">
+        <v>1914</v>
+      </c>
+      <c r="E799" s="4" t="s">
+        <v>1915</v>
+      </c>
+      <c r="F799" s="2">
+        <v>46216.007638888885</v>
+      </c>
+    </row>
+    <row r="800" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A800" s="3" t="s">
+        <v>1916</v>
+      </c>
+      <c r="B800" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="C800" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D800" s="4" t="s">
+        <v>1917</v>
+      </c>
+      <c r="E800" s="4" t="s">
+        <v>1918</v>
+      </c>
+      <c r="F800" s="2">
+        <v>46216.59375</v>
+      </c>
+    </row>
+    <row r="801" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A801" s="3" t="s">
+        <v>1919</v>
+      </c>
+      <c r="B801" s="4" t="s">
+        <v>1920</v>
+      </c>
+      <c r="C801" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D801" s="4" t="s">
+        <v>1730</v>
+      </c>
+      <c r="E801" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F801" s="2">
+        <v>46213.70625</v>
+      </c>
+    </row>
+    <row r="802" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A802" s="3" t="s">
+        <v>1921</v>
+      </c>
+      <c r="B802" s="4" t="s">
+        <v>1922</v>
+      </c>
+      <c r="C802" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D802" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E802" s="4" t="s">
+        <v>1178</v>
+      </c>
+      <c r="F802" s="2">
+        <v>46214.711805555555</v>
+      </c>
+    </row>
+    <row r="803" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A803" s="3" t="s">
+        <v>1923</v>
+      </c>
+      <c r="B803" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C803" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="D803" s="4" t="s">
+        <v>1924</v>
+      </c>
+      <c r="E803" s="4" t="s">
+        <v>1925</v>
+      </c>
+      <c r="F803" s="2">
+        <v>46215.46805555555</v>
+      </c>
+    </row>
+    <row r="804" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A804" s="3" t="s">
+        <v>1926</v>
+      </c>
+      <c r="B804" s="4" t="s">
+        <v>1927</v>
+      </c>
+      <c r="C804" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="D804" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E804" s="4" t="s">
+        <v>1928</v>
+      </c>
+      <c r="F804" s="2">
+        <v>46215.464583333334</v>
       </c>
     </row>
   </sheetData>
@@ -22987,6 +23131,12 @@
     <hyperlink ref="A796" r:id="rId795"/>
     <hyperlink ref="A797" r:id="rId796"/>
     <hyperlink ref="A798" r:id="rId797"/>
+    <hyperlink ref="A799" r:id="rId798"/>
+    <hyperlink ref="A800" r:id="rId799"/>
+    <hyperlink ref="A801" r:id="rId800"/>
+    <hyperlink ref="A802" r:id="rId801"/>
+    <hyperlink ref="A803" r:id="rId802"/>
+    <hyperlink ref="A804" r:id="rId803"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -22998,7 +23148,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23031,122 +23181,62 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1913</v>
+        <v>1929</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>27</v>
+        <v>1930</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>28</v>
+        <v>63</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>1914</v>
+        <v>99</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1915</v>
+        <v>1931</v>
       </c>
       <c r="F2" s="2">
-        <v>46216.007638888885</v>
+        <v>46217.51041666667</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1916</v>
+        <v>1932</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>325</v>
+        <v>150</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>63</v>
+        <v>275</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>1917</v>
+        <v>724</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1918</v>
+        <v>1933</v>
       </c>
       <c r="F3" s="2">
-        <v>46216.59375</v>
+        <v>46217.58263888889</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>1919</v>
+        <v>1934</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>1920</v>
+        <v>1935</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>256</v>
+        <v>284</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>1730</v>
+        <v>94</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>25</v>
+        <v>1936</v>
       </c>
       <c r="F4" s="2">
-        <v>46213.70625</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1921</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>1922</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1178</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46214.711805555555</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>1923</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>392</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>1924</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>1925</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46215.46805555555</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>1926</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>1927</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>392</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>1928</v>
-      </c>
-      <c r="F7" s="2">
-        <v>46215.464583333334</v>
+        <v>46216.913888888885</v>
       </c>
     </row>
   </sheetData>
@@ -23154,9 +23244,6 @@
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
     <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A6" r:id="rId5"/>
-    <hyperlink ref="A7" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-07-15 13:03
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4042" uniqueCount="1937">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4047" uniqueCount="1938">
   <si>
     <t>link</t>
   </si>
@@ -5829,6 +5829,9 @@
   </si>
   <si>
     <t>76640020054</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/asares-pag/mkxgc.html</t>
   </si>
 </sst>
 </file>
@@ -6241,7 +6244,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F804"/>
+  <dimension ref="A1:F807"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22330,6 +22333,66 @@
       </c>
       <c r="F804" s="2">
         <v>46215.464583333334</v>
+      </c>
+    </row>
+    <row r="805" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A805" s="3" t="s">
+        <v>1929</v>
+      </c>
+      <c r="B805" s="4" t="s">
+        <v>1930</v>
+      </c>
+      <c r="C805" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D805" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E805" s="4" t="s">
+        <v>1931</v>
+      </c>
+      <c r="F805" s="2">
+        <v>46217.51041666667</v>
+      </c>
+    </row>
+    <row r="806" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A806" s="3" t="s">
+        <v>1932</v>
+      </c>
+      <c r="B806" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C806" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="D806" s="4" t="s">
+        <v>724</v>
+      </c>
+      <c r="E806" s="4" t="s">
+        <v>1933</v>
+      </c>
+      <c r="F806" s="2">
+        <v>46217.58263888889</v>
+      </c>
+    </row>
+    <row r="807" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A807" s="3" t="s">
+        <v>1934</v>
+      </c>
+      <c r="B807" s="4" t="s">
+        <v>1935</v>
+      </c>
+      <c r="C807" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D807" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="E807" s="4" t="s">
+        <v>1936</v>
+      </c>
+      <c r="F807" s="2">
+        <v>46216.913888888885</v>
       </c>
     </row>
   </sheetData>
@@ -23137,6 +23200,9 @@
     <hyperlink ref="A802" r:id="rId801"/>
     <hyperlink ref="A803" r:id="rId802"/>
     <hyperlink ref="A804" r:id="rId803"/>
+    <hyperlink ref="A805" r:id="rId804"/>
+    <hyperlink ref="A806" r:id="rId805"/>
+    <hyperlink ref="A807" r:id="rId806"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -23148,7 +23214,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23181,69 +23247,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1929</v>
+        <v>1937</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1930</v>
+        <v>576</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>63</v>
+        <v>127</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>99</v>
+        <v>272</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1931</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46217.51041666667</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1932</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>275</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>724</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1933</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46217.58263888889</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1934</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>1935</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1936</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46216.913888888885</v>
+        <v>46217.93958333333</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-07-16 13:11
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -6244,7 +6244,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F807"/>
+  <dimension ref="A1:F808"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22393,6 +22393,26 @@
       </c>
       <c r="F807" s="2">
         <v>46216.913888888885</v>
+      </c>
+    </row>
+    <row r="808" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A808" s="3" t="s">
+        <v>1937</v>
+      </c>
+      <c r="B808" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="C808" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D808" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E808" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F808" s="2">
+        <v>46217.93958333333</v>
       </c>
     </row>
   </sheetData>
@@ -23203,6 +23223,7 @@
     <hyperlink ref="A805" r:id="rId804"/>
     <hyperlink ref="A806" r:id="rId805"/>
     <hyperlink ref="A807" r:id="rId806"/>
+    <hyperlink ref="A808" r:id="rId807"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -23214,7 +23235,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23245,30 +23266,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>1937</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>576</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46217.93958333333</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-07-17 12:57
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4047" uniqueCount="1938">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4052" uniqueCount="1941">
   <si>
     <t>link</t>
   </si>
@@ -5832,6 +5832,15 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/asares-pag/mkxgc.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/tukums-and-reg/matkules-pag/hbiep.html</t>
+  </si>
+  <si>
+    <t>80 ha.</t>
+  </si>
+  <si>
+    <t>90700030320</t>
   </si>
 </sst>
 </file>
@@ -23235,7 +23244,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23266,7 +23275,30 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>1938</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>1939</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>1940</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46220.51180555555</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-07-20 13:44
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4052" uniqueCount="1941">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4102" uniqueCount="1957">
   <si>
     <t>link</t>
   </si>
@@ -5841,6 +5841,54 @@
   </si>
   <si>
     <t>90700030320</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/rugaju-pag/clomh.html</t>
+  </si>
+  <si>
+    <t>38740150102</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/bauska-and-reg/brunavas-pag/ohpcg.html</t>
+  </si>
+  <si>
+    <t>40460150033</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/raunas-pag/ofdnf.html</t>
+  </si>
+  <si>
+    <t>42760070056</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/rubenes-pag/kbxkd.html</t>
+  </si>
+  <si>
+    <t>56820030063</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/rubenes-pag/mgkkm.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kuldiga-and-reg/gudenieku-pag/cxdio.html</t>
+  </si>
+  <si>
+    <t>62500060121</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kuldiga-and-reg/gudenieku-pag/ehxlf.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/rusonas-pag/bxgkop.html</t>
+  </si>
+  <si>
+    <t>76700020029</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/tukums-and-reg/slampes-pag/oeege.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valka-and-reg/blomes-pag/kflxh.html</t>
   </si>
 </sst>
 </file>
@@ -6253,7 +6301,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F808"/>
+  <dimension ref="A1:F809"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22422,6 +22470,26 @@
       </c>
       <c r="F808" s="2">
         <v>46217.93958333333</v>
+      </c>
+    </row>
+    <row r="809" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A809" s="3" t="s">
+        <v>1938</v>
+      </c>
+      <c r="B809" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="C809" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D809" s="4" t="s">
+        <v>1939</v>
+      </c>
+      <c r="E809" s="4" t="s">
+        <v>1940</v>
+      </c>
+      <c r="F809" s="2">
+        <v>46220.51180555555</v>
       </c>
     </row>
   </sheetData>
@@ -23233,6 +23301,7 @@
     <hyperlink ref="A806" r:id="rId805"/>
     <hyperlink ref="A807" r:id="rId806"/>
     <hyperlink ref="A808" r:id="rId807"/>
+    <hyperlink ref="A809" r:id="rId808"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -23244,7 +23313,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23277,27 +23346,216 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1938</v>
+        <v>1941</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>217</v>
+        <v>189</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>1942</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46223.486805555556</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1943</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1944</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46222.91527777778</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1945</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1946</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46222.88680555555</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1947</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>971</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1948</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46223.48888888889</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>1949</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>988</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>1948</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46223.48472222222</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>1950</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>1951</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46223.47430555556</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>1952</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>1951</v>
+      </c>
+      <c r="F8" s="2">
+        <v>46223.46944444445</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>1953</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>1954</v>
+      </c>
+      <c r="F9" s="2">
+        <v>46221.66458333333</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>1955</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>376</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>1939</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>1940</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46220.51180555555</v>
+      <c r="D10" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>1239</v>
+      </c>
+      <c r="F10" s="2">
+        <v>46220.70694444445</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>1956</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>781</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>563</v>
+      </c>
+      <c r="F11" s="2">
+        <v>46222.49791666667</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+    <hyperlink ref="A6" r:id="rId5"/>
+    <hyperlink ref="A7" r:id="rId6"/>
+    <hyperlink ref="A8" r:id="rId7"/>
+    <hyperlink ref="A9" r:id="rId8"/>
+    <hyperlink ref="A10" r:id="rId9"/>
+    <hyperlink ref="A11" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-07-21 13:09
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4102" uniqueCount="1957">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4112" uniqueCount="1960">
   <si>
     <t>link</t>
   </si>
@@ -5889,6 +5889,15 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/valka-and-reg/blomes-pag/kflxh.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/dobele-and-reg/zebrenes-pag/bxpexx.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valka-and-reg/grundzales-pag/bohfp.html</t>
+  </si>
+  <si>
+    <t>94580060037</t>
   </si>
 </sst>
 </file>
@@ -6301,7 +6310,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F809"/>
+  <dimension ref="A1:F819"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22490,6 +22499,206 @@
       </c>
       <c r="F809" s="2">
         <v>46220.51180555555</v>
+      </c>
+    </row>
+    <row r="810" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A810" s="3" t="s">
+        <v>1941</v>
+      </c>
+      <c r="B810" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="C810" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D810" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E810" s="4" t="s">
+        <v>1942</v>
+      </c>
+      <c r="F810" s="2">
+        <v>46223.486805555556</v>
+      </c>
+    </row>
+    <row r="811" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A811" s="3" t="s">
+        <v>1943</v>
+      </c>
+      <c r="B811" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C811" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D811" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E811" s="4" t="s">
+        <v>1944</v>
+      </c>
+      <c r="F811" s="2">
+        <v>46222.91527777778</v>
+      </c>
+    </row>
+    <row r="812" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A812" s="3" t="s">
+        <v>1945</v>
+      </c>
+      <c r="B812" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C812" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D812" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E812" s="4" t="s">
+        <v>1946</v>
+      </c>
+      <c r="F812" s="2">
+        <v>46222.88680555555</v>
+      </c>
+    </row>
+    <row r="813" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A813" s="3" t="s">
+        <v>1947</v>
+      </c>
+      <c r="B813" s="4" t="s">
+        <v>971</v>
+      </c>
+      <c r="C813" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D813" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E813" s="4" t="s">
+        <v>1948</v>
+      </c>
+      <c r="F813" s="2">
+        <v>46223.48888888889</v>
+      </c>
+    </row>
+    <row r="814" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A814" s="3" t="s">
+        <v>1949</v>
+      </c>
+      <c r="B814" s="4" t="s">
+        <v>988</v>
+      </c>
+      <c r="C814" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D814" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="E814" s="4" t="s">
+        <v>1948</v>
+      </c>
+      <c r="F814" s="2">
+        <v>46223.48472222222</v>
+      </c>
+    </row>
+    <row r="815" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A815" s="3" t="s">
+        <v>1950</v>
+      </c>
+      <c r="B815" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C815" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="D815" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="E815" s="4" t="s">
+        <v>1951</v>
+      </c>
+      <c r="F815" s="2">
+        <v>46223.47430555556</v>
+      </c>
+    </row>
+    <row r="816" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A816" s="3" t="s">
+        <v>1952</v>
+      </c>
+      <c r="B816" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="C816" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="D816" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E816" s="4" t="s">
+        <v>1951</v>
+      </c>
+      <c r="F816" s="2">
+        <v>46223.46944444445</v>
+      </c>
+    </row>
+    <row r="817" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A817" s="3" t="s">
+        <v>1953</v>
+      </c>
+      <c r="B817" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C817" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D817" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="E817" s="4" t="s">
+        <v>1954</v>
+      </c>
+      <c r="F817" s="2">
+        <v>46221.66458333333</v>
+      </c>
+    </row>
+    <row r="818" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A818" s="3" t="s">
+        <v>1955</v>
+      </c>
+      <c r="B818" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="C818" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D818" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E818" s="4" t="s">
+        <v>1239</v>
+      </c>
+      <c r="F818" s="2">
+        <v>46220.70694444445</v>
+      </c>
+    </row>
+    <row r="819" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A819" s="3" t="s">
+        <v>1956</v>
+      </c>
+      <c r="B819" s="4" t="s">
+        <v>781</v>
+      </c>
+      <c r="C819" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="D819" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E819" s="4" t="s">
+        <v>563</v>
+      </c>
+      <c r="F819" s="2">
+        <v>46222.49791666667</v>
       </c>
     </row>
   </sheetData>
@@ -23302,6 +23511,16 @@
     <hyperlink ref="A807" r:id="rId806"/>
     <hyperlink ref="A808" r:id="rId807"/>
     <hyperlink ref="A809" r:id="rId808"/>
+    <hyperlink ref="A810" r:id="rId809"/>
+    <hyperlink ref="A811" r:id="rId810"/>
+    <hyperlink ref="A812" r:id="rId811"/>
+    <hyperlink ref="A813" r:id="rId812"/>
+    <hyperlink ref="A814" r:id="rId813"/>
+    <hyperlink ref="A815" r:id="rId814"/>
+    <hyperlink ref="A816" r:id="rId815"/>
+    <hyperlink ref="A817" r:id="rId816"/>
+    <hyperlink ref="A818" r:id="rId817"/>
+    <hyperlink ref="A819" r:id="rId818"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -23313,7 +23532,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23346,216 +23565,48 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1941</v>
+        <v>1957</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>189</v>
+        <v>31</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>28</v>
+        <v>117</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>169</v>
+        <v>1785</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1942</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46223.486805555556</v>
+        <v>46223.83541666667</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1943</v>
+        <v>1958</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>116</v>
+        <v>337</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>48</v>
+        <v>392</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>186</v>
+        <v>514</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1944</v>
+        <v>1959</v>
       </c>
       <c r="F3" s="2">
-        <v>46222.91527777778</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1945</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1946</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46222.88680555555</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1947</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>971</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1948</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46223.48888888889</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>1949</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>988</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>250</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>1948</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46223.48472222222</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>1950</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>424</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>1951</v>
-      </c>
-      <c r="F7" s="2">
-        <v>46223.47430555556</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>1952</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>449</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>424</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>1951</v>
-      </c>
-      <c r="F8" s="2">
-        <v>46223.46944444445</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>1953</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>247</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>1954</v>
-      </c>
-      <c r="F9" s="2">
-        <v>46221.66458333333</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>1955</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>376</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>1239</v>
-      </c>
-      <c r="F10" s="2">
-        <v>46220.70694444445</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>1956</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>781</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>392</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>563</v>
-      </c>
-      <c r="F11" s="2">
-        <v>46222.49791666667</v>
+        <v>46224.63333333333</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A6" r:id="rId5"/>
-    <hyperlink ref="A7" r:id="rId6"/>
-    <hyperlink ref="A8" r:id="rId7"/>
-    <hyperlink ref="A9" r:id="rId8"/>
-    <hyperlink ref="A10" r:id="rId9"/>
-    <hyperlink ref="A11" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-07-22 13:16
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4112" uniqueCount="1960">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4137" uniqueCount="1973">
   <si>
     <t>link</t>
   </si>
@@ -5898,6 +5898,45 @@
   </si>
   <si>
     <t>94580060037</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aizkraukle-and-reg/aiviekstes-pag/jblli.html</t>
+  </si>
+  <si>
+    <t>0.40 ha.</t>
+  </si>
+  <si>
+    <t>32420070013</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/bauska-and-reg/vecumnieku-pag/kiexp.html</t>
+  </si>
+  <si>
+    <t>127 000 €</t>
+  </si>
+  <si>
+    <t>40940060014</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/daugavpils/bcpem.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/aknistes-l-t/bxidmo.html</t>
+  </si>
+  <si>
+    <t>7.30 ha.</t>
+  </si>
+  <si>
+    <t>56250040129</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valka-and-reg/karku-pag/bgncij.html</t>
+  </si>
+  <si>
+    <t>73 888 €</t>
+  </si>
+  <si>
+    <t>94660050023</t>
   </si>
 </sst>
 </file>
@@ -6310,7 +6349,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F819"/>
+  <dimension ref="A1:F821"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22699,6 +22738,46 @@
       </c>
       <c r="F819" s="2">
         <v>46222.49791666667</v>
+      </c>
+    </row>
+    <row r="820" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A820" s="3" t="s">
+        <v>1957</v>
+      </c>
+      <c r="B820" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C820" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D820" s="4" t="s">
+        <v>1785</v>
+      </c>
+      <c r="E820" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F820" s="2">
+        <v>46223.83541666667</v>
+      </c>
+    </row>
+    <row r="821" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A821" s="3" t="s">
+        <v>1958</v>
+      </c>
+      <c r="B821" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="C821" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="D821" s="4" t="s">
+        <v>514</v>
+      </c>
+      <c r="E821" s="4" t="s">
+        <v>1959</v>
+      </c>
+      <c r="F821" s="2">
+        <v>46224.63333333333</v>
       </c>
     </row>
   </sheetData>
@@ -23521,6 +23600,8 @@
     <hyperlink ref="A817" r:id="rId816"/>
     <hyperlink ref="A818" r:id="rId817"/>
     <hyperlink ref="A819" r:id="rId818"/>
+    <hyperlink ref="A820" r:id="rId819"/>
+    <hyperlink ref="A821" r:id="rId820"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -23532,7 +23613,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23565,48 +23646,111 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1957</v>
+        <v>1960</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>31</v>
+        <v>536</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>117</v>
+        <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>1785</v>
+        <v>1961</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>25</v>
+        <v>1962</v>
       </c>
       <c r="F2" s="2">
-        <v>46223.83541666667</v>
+        <v>46225.507638888885</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1958</v>
+        <v>1963</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>337</v>
+        <v>1964</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>716</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1965</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46225.56319444445</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1966</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46225.51597222222</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>1967</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>988</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>1968</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1969</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46225.334027777775</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>1970</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>1971</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>392</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>514</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1959</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46224.63333333333</v>
+      <c r="D6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>1972</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46225.57083333333</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+    <hyperlink ref="A6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-07-23 13:18
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4137" uniqueCount="1973">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4142" uniqueCount="1975">
   <si>
     <t>link</t>
   </si>
@@ -5937,6 +5937,12 @@
   </si>
   <si>
     <t>94660050023</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/aluksne/kfcch.html</t>
+  </si>
+  <si>
+    <t>36760040009</t>
   </si>
 </sst>
 </file>
@@ -6349,7 +6355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F821"/>
+  <dimension ref="A1:F826"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22778,6 +22784,106 @@
       </c>
       <c r="F821" s="2">
         <v>46224.63333333333</v>
+      </c>
+    </row>
+    <row r="822" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A822" s="3" t="s">
+        <v>1960</v>
+      </c>
+      <c r="B822" s="4" t="s">
+        <v>536</v>
+      </c>
+      <c r="C822" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D822" s="4" t="s">
+        <v>1961</v>
+      </c>
+      <c r="E822" s="4" t="s">
+        <v>1962</v>
+      </c>
+      <c r="F822" s="2">
+        <v>46225.507638888885</v>
+      </c>
+    </row>
+    <row r="823" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A823" s="3" t="s">
+        <v>1963</v>
+      </c>
+      <c r="B823" s="4" t="s">
+        <v>1964</v>
+      </c>
+      <c r="C823" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D823" s="4" t="s">
+        <v>716</v>
+      </c>
+      <c r="E823" s="4" t="s">
+        <v>1965</v>
+      </c>
+      <c r="F823" s="2">
+        <v>46225.56319444445</v>
+      </c>
+    </row>
+    <row r="824" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A824" s="3" t="s">
+        <v>1966</v>
+      </c>
+      <c r="B824" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C824" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D824" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E824" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F824" s="2">
+        <v>46225.51597222222</v>
+      </c>
+    </row>
+    <row r="825" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A825" s="3" t="s">
+        <v>1967</v>
+      </c>
+      <c r="B825" s="4" t="s">
+        <v>988</v>
+      </c>
+      <c r="C825" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D825" s="4" t="s">
+        <v>1968</v>
+      </c>
+      <c r="E825" s="4" t="s">
+        <v>1969</v>
+      </c>
+      <c r="F825" s="2">
+        <v>46225.334027777775</v>
+      </c>
+    </row>
+    <row r="826" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A826" s="3" t="s">
+        <v>1970</v>
+      </c>
+      <c r="B826" s="4" t="s">
+        <v>1971</v>
+      </c>
+      <c r="C826" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="D826" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E826" s="4" t="s">
+        <v>1972</v>
+      </c>
+      <c r="F826" s="2">
+        <v>46225.57083333333</v>
       </c>
     </row>
   </sheetData>
@@ -23602,6 +23708,11 @@
     <hyperlink ref="A819" r:id="rId818"/>
     <hyperlink ref="A820" r:id="rId819"/>
     <hyperlink ref="A821" r:id="rId820"/>
+    <hyperlink ref="A822" r:id="rId821"/>
+    <hyperlink ref="A823" r:id="rId822"/>
+    <hyperlink ref="A824" r:id="rId823"/>
+    <hyperlink ref="A825" r:id="rId824"/>
+    <hyperlink ref="A826" r:id="rId825"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -23613,7 +23724,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23646,111 +23757,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1960</v>
+        <v>1973</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>536</v>
+        <v>204</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>8</v>
+        <v>435</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>1961</v>
+        <v>186</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1962</v>
+        <v>1974</v>
       </c>
       <c r="F2" s="2">
-        <v>46225.507638888885</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1963</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>1964</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>716</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1965</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46225.56319444445</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1966</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46225.51597222222</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1967</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>988</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>1968</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1969</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46225.334027777775</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>1970</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>1971</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>392</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>1972</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46225.57083333333</v>
+        <v>46226.05138888889</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-07-24 13:12
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4142" uniqueCount="1975">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4152" uniqueCount="1979">
   <si>
     <t>link</t>
   </si>
@@ -5943,6 +5943,18 @@
   </si>
   <si>
     <t>36760040009</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/amatas-pag/odhof.html</t>
+  </si>
+  <si>
+    <t>42420050354</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/maltas-pag/ekddm.html</t>
+  </si>
+  <si>
+    <t>78700010174</t>
   </si>
 </sst>
 </file>
@@ -6355,7 +6367,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F826"/>
+  <dimension ref="A1:F827"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22884,6 +22896,26 @@
       </c>
       <c r="F826" s="2">
         <v>46225.57083333333</v>
+      </c>
+    </row>
+    <row r="827" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A827" s="3" t="s">
+        <v>1973</v>
+      </c>
+      <c r="B827" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C827" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D827" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E827" s="4" t="s">
+        <v>1974</v>
+      </c>
+      <c r="F827" s="2">
+        <v>46226.05138888889</v>
       </c>
     </row>
   </sheetData>
@@ -23713,6 +23745,7 @@
     <hyperlink ref="A824" r:id="rId823"/>
     <hyperlink ref="A825" r:id="rId824"/>
     <hyperlink ref="A826" r:id="rId825"/>
+    <hyperlink ref="A827" r:id="rId826"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -23724,7 +23757,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23757,27 +23790,48 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1973</v>
+        <v>1975</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>204</v>
+        <v>467</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>435</v>
+        <v>63</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>186</v>
+        <v>75</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1974</v>
+        <v>1976</v>
       </c>
       <c r="F2" s="2">
-        <v>46226.05138888889</v>
+        <v>46227.62777777778</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1977</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>707</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1978</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46227.53055555555</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-07-27 14:05
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4152" uniqueCount="1979">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4162" uniqueCount="1983">
   <si>
     <t>link</t>
   </si>
@@ -5955,6 +5955,18 @@
   </si>
   <si>
     <t>78700010174</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/silajanu-pag/mmjem.html</t>
+  </si>
+  <si>
+    <t>76760020053</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ventspils-and-reg/ances-pag/boxdm.html</t>
+  </si>
+  <si>
+    <t>62 ha.</t>
   </si>
 </sst>
 </file>
@@ -6367,7 +6379,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F827"/>
+  <dimension ref="A1:F829"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22916,6 +22928,46 @@
       </c>
       <c r="F827" s="2">
         <v>46226.05138888889</v>
+      </c>
+    </row>
+    <row r="828" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A828" s="3" t="s">
+        <v>1975</v>
+      </c>
+      <c r="B828" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="C828" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D828" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E828" s="4" t="s">
+        <v>1976</v>
+      </c>
+      <c r="F828" s="2">
+        <v>46227.62777777778</v>
+      </c>
+    </row>
+    <row r="829" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A829" s="3" t="s">
+        <v>1977</v>
+      </c>
+      <c r="B829" s="4" t="s">
+        <v>707</v>
+      </c>
+      <c r="C829" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D829" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E829" s="4" t="s">
+        <v>1978</v>
+      </c>
+      <c r="F829" s="2">
+        <v>46227.53055555555</v>
       </c>
     </row>
   </sheetData>
@@ -23746,6 +23798,8 @@
     <hyperlink ref="A825" r:id="rId824"/>
     <hyperlink ref="A826" r:id="rId825"/>
     <hyperlink ref="A827" r:id="rId826"/>
+    <hyperlink ref="A828" r:id="rId827"/>
+    <hyperlink ref="A829" r:id="rId828"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -23790,42 +23844,42 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1975</v>
+        <v>1979</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>467</v>
+        <v>274</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>63</v>
+        <v>284</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1976</v>
+        <v>1980</v>
       </c>
       <c r="F2" s="2">
-        <v>46227.62777777778</v>
+        <v>46228.46736111111</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1977</v>
+        <v>1981</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>707</v>
+        <v>513</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>294</v>
+        <v>404</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>36</v>
+        <v>1982</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1978</v>
+        <v>25</v>
       </c>
       <c r="F3" s="2">
-        <v>46227.53055555555</v>
+        <v>46229.77986111111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-07-28 13:25
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -6379,7 +6379,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F829"/>
+  <dimension ref="A1:F831"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -22968,6 +22968,46 @@
       </c>
       <c r="F829" s="2">
         <v>46227.53055555555</v>
+      </c>
+    </row>
+    <row r="830" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A830" s="3" t="s">
+        <v>1979</v>
+      </c>
+      <c r="B830" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="C830" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D830" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E830" s="4" t="s">
+        <v>1980</v>
+      </c>
+      <c r="F830" s="2">
+        <v>46228.46736111111</v>
+      </c>
+    </row>
+    <row r="831" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A831" s="3" t="s">
+        <v>1981</v>
+      </c>
+      <c r="B831" s="4" t="s">
+        <v>513</v>
+      </c>
+      <c r="C831" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D831" s="4" t="s">
+        <v>1982</v>
+      </c>
+      <c r="E831" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F831" s="2">
+        <v>46229.77986111111</v>
       </c>
     </row>
   </sheetData>
@@ -23800,6 +23840,8 @@
     <hyperlink ref="A827" r:id="rId826"/>
     <hyperlink ref="A828" r:id="rId827"/>
     <hyperlink ref="A829" r:id="rId828"/>
+    <hyperlink ref="A830" r:id="rId829"/>
+    <hyperlink ref="A831" r:id="rId830"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -23811,7 +23853,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23842,51 +23884,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>1979</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>274</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>1980</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46228.46736111111</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1981</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>513</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>404</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>1982</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46229.77986111111</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-07-29 13:31
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4162" uniqueCount="1983">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4177" uniqueCount="1988">
   <si>
     <t>link</t>
   </si>
@@ -5967,6 +5967,21 @@
   </si>
   <si>
     <t>62 ha.</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jelgava-and-reg/jelgava/ckncp.html</t>
+  </si>
+  <si>
+    <t>54860090022</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/vestienas-pag/fkeee.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valmiera-and-reg/valmiera/bmlgb.html</t>
+  </si>
+  <si>
+    <t>Pārdod meža cirsmu</t>
   </si>
 </sst>
 </file>
@@ -23853,7 +23868,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23884,7 +23899,72 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>1983</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>1984</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46232.49375</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1985</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>1562</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46231.75486111111</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1986</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1987</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46232.60833333334</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-07-30 13:21
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4177" uniqueCount="1988">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4187" uniqueCount="1991">
   <si>
     <t>link</t>
   </si>
@@ -5982,6 +5982,15 @@
   </si>
   <si>
     <t>Pārdod meža cirsmu</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/vecpiebalgas-pag/bkdhn.html</t>
+  </si>
+  <si>
+    <t>42920050036</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/pelecu-pag/ookcl.html</t>
   </si>
 </sst>
 </file>
@@ -6394,7 +6403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F831"/>
+  <dimension ref="A1:F834"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23023,6 +23032,66 @@
       </c>
       <c r="F831" s="2">
         <v>46229.77986111111</v>
+      </c>
+    </row>
+    <row r="832" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A832" s="3" t="s">
+        <v>1983</v>
+      </c>
+      <c r="B832" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C832" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="D832" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E832" s="4" t="s">
+        <v>1984</v>
+      </c>
+      <c r="F832" s="2">
+        <v>46232.49375</v>
+      </c>
+    </row>
+    <row r="833" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A833" s="3" t="s">
+        <v>1985</v>
+      </c>
+      <c r="B833" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C833" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D833" s="4" t="s">
+        <v>1562</v>
+      </c>
+      <c r="E833" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F833" s="2">
+        <v>46231.75486111111</v>
+      </c>
+    </row>
+    <row r="834" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A834" s="3" t="s">
+        <v>1986</v>
+      </c>
+      <c r="B834" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C834" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D834" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="E834" s="4" t="s">
+        <v>1987</v>
+      </c>
+      <c r="F834" s="2">
+        <v>46232.60833333334</v>
       </c>
     </row>
   </sheetData>
@@ -23857,6 +23926,9 @@
     <hyperlink ref="A829" r:id="rId828"/>
     <hyperlink ref="A830" r:id="rId829"/>
     <hyperlink ref="A831" r:id="rId830"/>
+    <hyperlink ref="A832" r:id="rId831"/>
+    <hyperlink ref="A833" r:id="rId832"/>
+    <hyperlink ref="A834" r:id="rId833"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -23868,7 +23940,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23901,69 +23973,48 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1983</v>
+        <v>1988</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>52</v>
+        <v>666</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>518</v>
+        <v>63</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>82</v>
+        <v>1558</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1984</v>
+        <v>1989</v>
       </c>
       <c r="F2" s="2">
-        <v>46232.49375</v>
+        <v>46232.97152777778</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1985</v>
+        <v>1990</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>56</v>
+        <v>106</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>256</v>
+        <v>284</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>1562</v>
+        <v>85</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>25</v>
+        <v>912</v>
       </c>
       <c r="F3" s="2">
-        <v>46231.75486111111</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1986</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1987</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46232.60833333334</v>
+        <v>46233.49722222222</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-07-31 13:25
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -6403,7 +6403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F834"/>
+  <dimension ref="A1:F836"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23092,6 +23092,46 @@
       </c>
       <c r="F834" s="2">
         <v>46232.60833333334</v>
+      </c>
+    </row>
+    <row r="835" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A835" s="3" t="s">
+        <v>1988</v>
+      </c>
+      <c r="B835" s="4" t="s">
+        <v>666</v>
+      </c>
+      <c r="C835" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D835" s="4" t="s">
+        <v>1558</v>
+      </c>
+      <c r="E835" s="4" t="s">
+        <v>1989</v>
+      </c>
+      <c r="F835" s="2">
+        <v>46232.97152777778</v>
+      </c>
+    </row>
+    <row r="836" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A836" s="3" t="s">
+        <v>1990</v>
+      </c>
+      <c r="B836" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C836" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D836" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E836" s="4" t="s">
+        <v>912</v>
+      </c>
+      <c r="F836" s="2">
+        <v>46233.49722222222</v>
       </c>
     </row>
   </sheetData>
@@ -23929,6 +23969,8 @@
     <hyperlink ref="A832" r:id="rId831"/>
     <hyperlink ref="A833" r:id="rId832"/>
     <hyperlink ref="A834" r:id="rId833"/>
+    <hyperlink ref="A835" r:id="rId834"/>
+    <hyperlink ref="A836" r:id="rId835"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -23940,7 +23982,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23971,51 +24013,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>1988</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>666</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>1558</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>1989</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46232.97152777778</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1990</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>912</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46233.49722222222</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-08-03 14:09
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4187" uniqueCount="1991">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4197" uniqueCount="1996">
   <si>
     <t>link</t>
   </si>
@@ -5991,6 +5991,21 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/pelecu-pag/ookcl.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/andrupenes-pag/hkibg.html</t>
+  </si>
+  <si>
+    <t>60420080062</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ogre-and-reg/kegums/behdm.html</t>
+  </si>
+  <si>
+    <t>34584 m²</t>
+  </si>
+  <si>
+    <t>7409 007 0036</t>
   </si>
 </sst>
 </file>
@@ -23982,7 +23997,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24013,7 +24028,51 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>1991</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>1992</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46234.77291666667</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1993</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>1994</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1995</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46236.763194444444</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-08-04 13:31
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4197" uniqueCount="1996">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4202" uniqueCount="1998">
   <si>
     <t>link</t>
   </si>
@@ -6006,6 +6006,12 @@
   </si>
   <si>
     <t>7409 007 0036</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jelgava-and-reg/valgundes-nov/bclbm.html</t>
+  </si>
+  <si>
+    <t>54860070028</t>
   </si>
 </sst>
 </file>
@@ -6418,7 +6424,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F836"/>
+  <dimension ref="A1:F838"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23147,6 +23153,46 @@
       </c>
       <c r="F836" s="2">
         <v>46233.49722222222</v>
+      </c>
+    </row>
+    <row r="837" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A837" s="3" t="s">
+        <v>1991</v>
+      </c>
+      <c r="B837" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C837" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D837" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E837" s="4" t="s">
+        <v>1992</v>
+      </c>
+      <c r="F837" s="2">
+        <v>46234.77291666667</v>
+      </c>
+    </row>
+    <row r="838" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A838" s="3" t="s">
+        <v>1993</v>
+      </c>
+      <c r="B838" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C838" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="D838" s="4" t="s">
+        <v>1994</v>
+      </c>
+      <c r="E838" s="4" t="s">
+        <v>1995</v>
+      </c>
+      <c r="F838" s="2">
+        <v>46236.763194444444</v>
       </c>
     </row>
   </sheetData>
@@ -23986,6 +24032,8 @@
     <hyperlink ref="A834" r:id="rId833"/>
     <hyperlink ref="A835" r:id="rId834"/>
     <hyperlink ref="A836" r:id="rId835"/>
+    <hyperlink ref="A837" r:id="rId836"/>
+    <hyperlink ref="A838" r:id="rId837"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -23997,7 +24045,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24030,48 +24078,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1991</v>
+        <v>1996</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>27</v>
+        <v>88</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>146</v>
+        <v>518</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>67</v>
+        <v>82</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1992</v>
+        <v>1997</v>
       </c>
       <c r="F2" s="2">
-        <v>46234.77291666667</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1993</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>275</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>1994</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1995</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46236.763194444444</v>
+        <v>46238.620833333334</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-08-05 13:29
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4202" uniqueCount="1998">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4222" uniqueCount="2007">
   <si>
     <t>link</t>
   </si>
@@ -6012,6 +6012,33 @@
   </si>
   <si>
     <t>54860070028</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aizkraukle-and-reg/bebru-pag/boimn.html</t>
+  </si>
+  <si>
+    <t>21 800 €</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/rugaju-pag/gddxo.html</t>
+  </si>
+  <si>
+    <t>38740160011</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/gaigalavas-pag/jjnme.html</t>
+  </si>
+  <si>
+    <t>2.35 ha.</t>
+  </si>
+  <si>
+    <t>78540070451</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/tukums-and-reg/semes-pag/ilnle.html</t>
+  </si>
+  <si>
+    <t>2.34 ha.</t>
   </si>
 </sst>
 </file>
@@ -6424,7 +6451,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F838"/>
+  <dimension ref="A1:F839"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23193,6 +23220,26 @@
       </c>
       <c r="F838" s="2">
         <v>46236.763194444444</v>
+      </c>
+    </row>
+    <row r="839" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A839" s="3" t="s">
+        <v>1996</v>
+      </c>
+      <c r="B839" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C839" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="D839" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E839" s="4" t="s">
+        <v>1997</v>
+      </c>
+      <c r="F839" s="2">
+        <v>46238.620833333334</v>
       </c>
     </row>
   </sheetData>
@@ -24034,6 +24081,7 @@
     <hyperlink ref="A836" r:id="rId835"/>
     <hyperlink ref="A837" r:id="rId836"/>
     <hyperlink ref="A838" r:id="rId837"/>
+    <hyperlink ref="A839" r:id="rId838"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -24045,7 +24093,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24078,27 +24126,90 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1996</v>
+        <v>1998</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>88</v>
+        <v>1999</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>518</v>
+        <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>82</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1997</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46238.620833333334</v>
+        <v>46239.441666666666</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>2000</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>2001</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46239.6375</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>2002</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>2003</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>2004</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46238.81597222222</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>2005</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>2006</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46238.84097222222</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-08-06 13:28
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4222" uniqueCount="2007">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4232" uniqueCount="2010">
   <si>
     <t>link</t>
   </si>
@@ -6039,6 +6039,15 @@
   </si>
   <si>
     <t>2.34 ha.</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/liepaja-and-reg/rucavas-pag/negcm.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valmiera-and-reg/valmiera/hkgcd.html</t>
+  </si>
+  <si>
+    <t>96900100315</t>
   </si>
 </sst>
 </file>
@@ -6451,7 +6460,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F839"/>
+  <dimension ref="A1:F843"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23240,6 +23249,86 @@
       </c>
       <c r="F839" s="2">
         <v>46238.620833333334</v>
+      </c>
+    </row>
+    <row r="840" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A840" s="3" t="s">
+        <v>1998</v>
+      </c>
+      <c r="B840" s="4" t="s">
+        <v>1999</v>
+      </c>
+      <c r="C840" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D840" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E840" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F840" s="2">
+        <v>46239.441666666666</v>
+      </c>
+    </row>
+    <row r="841" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A841" s="3" t="s">
+        <v>2000</v>
+      </c>
+      <c r="B841" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C841" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D841" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E841" s="4" t="s">
+        <v>2001</v>
+      </c>
+      <c r="F841" s="2">
+        <v>46239.6375</v>
+      </c>
+    </row>
+    <row r="842" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A842" s="3" t="s">
+        <v>2002</v>
+      </c>
+      <c r="B842" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="C842" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D842" s="4" t="s">
+        <v>2003</v>
+      </c>
+      <c r="E842" s="4" t="s">
+        <v>2004</v>
+      </c>
+      <c r="F842" s="2">
+        <v>46238.81597222222</v>
+      </c>
+    </row>
+    <row r="843" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A843" s="3" t="s">
+        <v>2005</v>
+      </c>
+      <c r="B843" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C843" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D843" s="4" t="s">
+        <v>2006</v>
+      </c>
+      <c r="E843" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F843" s="2">
+        <v>46238.84097222222</v>
       </c>
     </row>
   </sheetData>
@@ -24082,6 +24171,10 @@
     <hyperlink ref="A837" r:id="rId836"/>
     <hyperlink ref="A838" r:id="rId837"/>
     <hyperlink ref="A839" r:id="rId838"/>
+    <hyperlink ref="A840" r:id="rId839"/>
+    <hyperlink ref="A841" r:id="rId840"/>
+    <hyperlink ref="A842" r:id="rId841"/>
+    <hyperlink ref="A843" r:id="rId842"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -24093,7 +24186,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24126,90 +24219,48 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>1998</v>
+        <v>2007</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1999</v>
+        <v>673</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>8</v>
+        <v>190</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>82</v>
+        <v>44</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>25</v>
+        <v>674</v>
       </c>
       <c r="F2" s="2">
-        <v>46239.441666666666</v>
+        <v>46240.549305555556</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>2000</v>
+        <v>2008</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>106</v>
+        <v>31</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>28</v>
+        <v>396</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>186</v>
+        <v>9</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>2001</v>
+        <v>2009</v>
       </c>
       <c r="F3" s="2">
-        <v>46239.6375</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>2002</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>268</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>2003</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>2004</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46238.81597222222</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>2005</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>376</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>2006</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46238.84097222222</v>
+        <v>46240.46875</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-08-07 12:35
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4232" uniqueCount="2010">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4247" uniqueCount="2017">
   <si>
     <t>link</t>
   </si>
@@ -6048,6 +6048,27 @@
   </si>
   <si>
     <t>96900100315</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aizkraukle-and-reg/staburaga-pag/amkcm.html</t>
+  </si>
+  <si>
+    <t>32840010201</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/annas-pag/mkjec.html</t>
+  </si>
+  <si>
+    <t>36440010037</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valka-and-reg/zvartavas-pag/bxpph.html</t>
+  </si>
+  <si>
+    <t>33400 m²</t>
+  </si>
+  <si>
+    <t>94960070020</t>
   </si>
 </sst>
 </file>
@@ -6460,7 +6481,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F843"/>
+  <dimension ref="A1:F845"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23329,6 +23350,46 @@
       </c>
       <c r="F843" s="2">
         <v>46238.84097222222</v>
+      </c>
+    </row>
+    <row r="844" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A844" s="3" t="s">
+        <v>2007</v>
+      </c>
+      <c r="B844" s="4" t="s">
+        <v>673</v>
+      </c>
+      <c r="C844" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="D844" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E844" s="4" t="s">
+        <v>674</v>
+      </c>
+      <c r="F844" s="2">
+        <v>46240.549305555556</v>
+      </c>
+    </row>
+    <row r="845" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A845" s="3" t="s">
+        <v>2008</v>
+      </c>
+      <c r="B845" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C845" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D845" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E845" s="4" t="s">
+        <v>2009</v>
+      </c>
+      <c r="F845" s="2">
+        <v>46240.46875</v>
       </c>
     </row>
   </sheetData>
@@ -24175,6 +24236,8 @@
     <hyperlink ref="A841" r:id="rId840"/>
     <hyperlink ref="A842" r:id="rId841"/>
     <hyperlink ref="A843" r:id="rId842"/>
+    <hyperlink ref="A844" r:id="rId843"/>
+    <hyperlink ref="A845" r:id="rId844"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -24186,7 +24249,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24219,48 +24282,69 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2007</v>
+        <v>2010</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>673</v>
+        <v>131</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>190</v>
+        <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>44</v>
+        <v>235</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>674</v>
+        <v>2011</v>
       </c>
       <c r="F2" s="2">
-        <v>46240.549305555556</v>
+        <v>46241.59236111111</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>2008</v>
+        <v>2012</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>31</v>
+        <v>666</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>396</v>
+        <v>435</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>9</v>
+        <v>849</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>2009</v>
+        <v>2013</v>
       </c>
       <c r="F3" s="2">
-        <v>46240.46875</v>
+        <v>46241.402083333334</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>2014</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>673</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>2015</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>2016</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46240.84861111111</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-08-10 12:38
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4247" uniqueCount="2017">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4267" uniqueCount="2028">
   <si>
     <t>link</t>
   </si>
@@ -6069,6 +6069,39 @@
   </si>
   <si>
     <t>94960070020</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/bauska-and-reg/vecumnieku-pag/khgbg.html</t>
+  </si>
+  <si>
+    <t>101 000 €</t>
+  </si>
+  <si>
+    <t>13.55 ha.</t>
+  </si>
+  <si>
+    <t>40940100001</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/nitaures-pag/hkoff.html</t>
+  </si>
+  <si>
+    <t>1.43 ha.</t>
+  </si>
+  <si>
+    <t>42680050121</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ludza-and-reg/pusmucovas-pag/mjlpo.html</t>
+  </si>
+  <si>
+    <t>68900030051</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/aronas-pag/gfglc.html</t>
+  </si>
+  <si>
+    <t>70420080041</t>
   </si>
 </sst>
 </file>
@@ -6481,7 +6514,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F845"/>
+  <dimension ref="A1:F848"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23390,6 +23423,66 @@
       </c>
       <c r="F845" s="2">
         <v>46240.46875</v>
+      </c>
+    </row>
+    <row r="846" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A846" s="3" t="s">
+        <v>2010</v>
+      </c>
+      <c r="B846" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C846" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D846" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="E846" s="4" t="s">
+        <v>2011</v>
+      </c>
+      <c r="F846" s="2">
+        <v>46241.59236111111</v>
+      </c>
+    </row>
+    <row r="847" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A847" s="3" t="s">
+        <v>2012</v>
+      </c>
+      <c r="B847" s="4" t="s">
+        <v>666</v>
+      </c>
+      <c r="C847" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D847" s="4" t="s">
+        <v>849</v>
+      </c>
+      <c r="E847" s="4" t="s">
+        <v>2013</v>
+      </c>
+      <c r="F847" s="2">
+        <v>46241.402083333334</v>
+      </c>
+    </row>
+    <row r="848" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A848" s="3" t="s">
+        <v>2014</v>
+      </c>
+      <c r="B848" s="4" t="s">
+        <v>673</v>
+      </c>
+      <c r="C848" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="D848" s="4" t="s">
+        <v>2015</v>
+      </c>
+      <c r="E848" s="4" t="s">
+        <v>2016</v>
+      </c>
+      <c r="F848" s="2">
+        <v>46240.84861111111</v>
       </c>
     </row>
   </sheetData>
@@ -24238,6 +24331,9 @@
     <hyperlink ref="A843" r:id="rId842"/>
     <hyperlink ref="A844" r:id="rId843"/>
     <hyperlink ref="A845" r:id="rId844"/>
+    <hyperlink ref="A846" r:id="rId845"/>
+    <hyperlink ref="A847" r:id="rId846"/>
+    <hyperlink ref="A848" r:id="rId847"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -24249,7 +24345,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24282,62 +24378,82 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2010</v>
+        <v>2017</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>131</v>
+        <v>2018</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>235</v>
+        <v>2019</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2011</v>
+        <v>2020</v>
       </c>
       <c r="F2" s="2">
-        <v>46241.59236111111</v>
+        <v>46243.90625</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>2012</v>
+        <v>2021</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>666</v>
+        <v>467</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>435</v>
+        <v>63</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>849</v>
+        <v>2022</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>2013</v>
+        <v>2023</v>
       </c>
       <c r="F3" s="2">
-        <v>46241.402083333334</v>
+        <v>46242.7875</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>2014</v>
+        <v>2024</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>673</v>
+        <v>204</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>392</v>
+        <v>234</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>2015</v>
+        <v>85</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>2016</v>
+        <v>2025</v>
       </c>
       <c r="F4" s="2">
-        <v>46240.84861111111</v>
+        <v>46242.33333333333</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>2026</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>1863</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>849</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>2027</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46244.52083333333</v>
       </c>
     </row>
   </sheetData>
@@ -24345,6 +24461,7 @@
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
     <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-08-11 12:35
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -6514,7 +6514,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F848"/>
+  <dimension ref="A1:F852"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23483,6 +23483,86 @@
       </c>
       <c r="F848" s="2">
         <v>46240.84861111111</v>
+      </c>
+    </row>
+    <row r="849" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A849" s="3" t="s">
+        <v>2017</v>
+      </c>
+      <c r="B849" s="4" t="s">
+        <v>2018</v>
+      </c>
+      <c r="C849" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D849" s="4" t="s">
+        <v>2019</v>
+      </c>
+      <c r="E849" s="4" t="s">
+        <v>2020</v>
+      </c>
+      <c r="F849" s="2">
+        <v>46243.90625</v>
+      </c>
+    </row>
+    <row r="850" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A850" s="3" t="s">
+        <v>2021</v>
+      </c>
+      <c r="B850" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="C850" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D850" s="4" t="s">
+        <v>2022</v>
+      </c>
+      <c r="E850" s="4" t="s">
+        <v>2023</v>
+      </c>
+      <c r="F850" s="2">
+        <v>46242.7875</v>
+      </c>
+    </row>
+    <row r="851" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A851" s="3" t="s">
+        <v>2024</v>
+      </c>
+      <c r="B851" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C851" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D851" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E851" s="4" t="s">
+        <v>2025</v>
+      </c>
+      <c r="F851" s="2">
+        <v>46242.33333333333</v>
+      </c>
+    </row>
+    <row r="852" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A852" s="3" t="s">
+        <v>2026</v>
+      </c>
+      <c r="B852" s="4" t="s">
+        <v>1863</v>
+      </c>
+      <c r="C852" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D852" s="4" t="s">
+        <v>849</v>
+      </c>
+      <c r="E852" s="4" t="s">
+        <v>2027</v>
+      </c>
+      <c r="F852" s="2">
+        <v>46244.52083333333</v>
       </c>
     </row>
   </sheetData>
@@ -24334,6 +24414,10 @@
     <hyperlink ref="A846" r:id="rId845"/>
     <hyperlink ref="A847" r:id="rId846"/>
     <hyperlink ref="A848" r:id="rId847"/>
+    <hyperlink ref="A849" r:id="rId848"/>
+    <hyperlink ref="A850" r:id="rId849"/>
+    <hyperlink ref="A851" r:id="rId850"/>
+    <hyperlink ref="A852" r:id="rId851"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -24345,7 +24429,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24376,93 +24460,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>2017</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>2018</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>2019</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>2020</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46243.90625</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>2021</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>467</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>2022</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>2023</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46242.7875</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>2024</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>2025</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46242.33333333333</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>2026</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>1863</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>849</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>2027</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46244.52083333333</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-08-12 12:38
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4267" uniqueCount="2028">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4272" uniqueCount="2030">
   <si>
     <t>link</t>
   </si>
@@ -6102,6 +6102,12 @@
   </si>
   <si>
     <t>70420080041</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jelgava-and-reg/kalnciema-l-t/fbihf.html</t>
+  </si>
+  <si>
+    <t>78 000 €</t>
   </si>
 </sst>
 </file>
@@ -24429,7 +24435,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24460,7 +24466,30 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>2028</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>2029</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>560</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46246.53125</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-08-13 12:39
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4272" uniqueCount="2030">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4287" uniqueCount="2037">
   <si>
     <t>link</t>
   </si>
@@ -6108,6 +6108,27 @@
   </si>
   <si>
     <t>78 000 €</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/ziguru-pag/gxjpj.html</t>
+  </si>
+  <si>
+    <t>10.60 ha.</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/dobele-and-reg/zebrenes-pag/bxkepd.html</t>
+  </si>
+  <si>
+    <t>46980020029</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/salas-pag/olkni.html</t>
+  </si>
+  <si>
+    <t>2.42 ha.</t>
+  </si>
+  <si>
+    <t>56860110022</t>
   </si>
 </sst>
 </file>
@@ -6520,7 +6541,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F852"/>
+  <dimension ref="A1:F853"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23569,6 +23590,26 @@
       </c>
       <c r="F852" s="2">
         <v>46244.52083333333</v>
+      </c>
+    </row>
+    <row r="853" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A853" s="3" t="s">
+        <v>2028</v>
+      </c>
+      <c r="B853" s="4" t="s">
+        <v>2029</v>
+      </c>
+      <c r="C853" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="D853" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E853" s="4" t="s">
+        <v>560</v>
+      </c>
+      <c r="F853" s="2">
+        <v>46246.53125</v>
       </c>
     </row>
   </sheetData>
@@ -24424,6 +24465,7 @@
     <hyperlink ref="A850" r:id="rId849"/>
     <hyperlink ref="A851" r:id="rId850"/>
     <hyperlink ref="A852" r:id="rId851"/>
+    <hyperlink ref="A853" r:id="rId852"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -24435,7 +24477,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24468,27 +24510,69 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2028</v>
+        <v>2030</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2029</v>
+        <v>521</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>518</v>
+        <v>28</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>67</v>
+        <v>2031</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>560</v>
+        <v>1431</v>
       </c>
       <c r="F2" s="2">
-        <v>46246.53125</v>
+        <v>46247.49166666667</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>2032</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>590</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>2033</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46247.59166666667</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>2034</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>2035</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>2036</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46247.43819444445</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-08-14 12:35
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4287" uniqueCount="2037">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4292" uniqueCount="2040">
   <si>
     <t>link</t>
   </si>
@@ -6129,6 +6129,15 @@
   </si>
   <si>
     <t>56860110022</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/gulbene-and-reg/lejasciema-pag/fgkjg.html</t>
+  </si>
+  <si>
+    <t>5 400 €</t>
+  </si>
+  <si>
+    <t>50640110005</t>
   </si>
 </sst>
 </file>
@@ -6541,7 +6550,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F853"/>
+  <dimension ref="A1:F856"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23610,6 +23619,66 @@
       </c>
       <c r="F853" s="2">
         <v>46246.53125</v>
+      </c>
+    </row>
+    <row r="854" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A854" s="3" t="s">
+        <v>2030</v>
+      </c>
+      <c r="B854" s="4" t="s">
+        <v>521</v>
+      </c>
+      <c r="C854" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D854" s="4" t="s">
+        <v>2031</v>
+      </c>
+      <c r="E854" s="4" t="s">
+        <v>1431</v>
+      </c>
+      <c r="F854" s="2">
+        <v>46247.49166666667</v>
+      </c>
+    </row>
+    <row r="855" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A855" s="3" t="s">
+        <v>2032</v>
+      </c>
+      <c r="B855" s="4" t="s">
+        <v>590</v>
+      </c>
+      <c r="C855" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D855" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E855" s="4" t="s">
+        <v>2033</v>
+      </c>
+      <c r="F855" s="2">
+        <v>46247.59166666667</v>
+      </c>
+    </row>
+    <row r="856" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A856" s="3" t="s">
+        <v>2034</v>
+      </c>
+      <c r="B856" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C856" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D856" s="4" t="s">
+        <v>2035</v>
+      </c>
+      <c r="E856" s="4" t="s">
+        <v>2036</v>
+      </c>
+      <c r="F856" s="2">
+        <v>46247.43819444445</v>
       </c>
     </row>
   </sheetData>
@@ -24466,6 +24535,9 @@
     <hyperlink ref="A851" r:id="rId850"/>
     <hyperlink ref="A852" r:id="rId851"/>
     <hyperlink ref="A853" r:id="rId852"/>
+    <hyperlink ref="A854" r:id="rId853"/>
+    <hyperlink ref="A855" r:id="rId854"/>
+    <hyperlink ref="A856" r:id="rId855"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -24477,7 +24549,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24510,69 +24582,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2030</v>
+        <v>2037</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>521</v>
+        <v>2038</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>28</v>
+        <v>124</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>2031</v>
+        <v>272</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1431</v>
+        <v>2039</v>
       </c>
       <c r="F2" s="2">
-        <v>46247.49166666667</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>2032</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>590</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>2033</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46247.59166666667</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>2034</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>2035</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>2036</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46247.43819444445</v>
+        <v>46248.46805555555</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-08-17 12:17
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4292" uniqueCount="2040">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4297" uniqueCount="2041">
   <si>
     <t>link</t>
   </si>
@@ -6138,6 +6138,9 @@
   </si>
   <si>
     <t>50640110005</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/aluksne/kblfk.html</t>
   </si>
 </sst>
 </file>
@@ -6550,7 +6553,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F856"/>
+  <dimension ref="A1:F857"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23679,6 +23682,26 @@
       </c>
       <c r="F856" s="2">
         <v>46247.43819444445</v>
+      </c>
+    </row>
+    <row r="857" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A857" s="3" t="s">
+        <v>2037</v>
+      </c>
+      <c r="B857" s="4" t="s">
+        <v>2038</v>
+      </c>
+      <c r="C857" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D857" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E857" s="4" t="s">
+        <v>2039</v>
+      </c>
+      <c r="F857" s="2">
+        <v>46248.46805555555</v>
       </c>
     </row>
   </sheetData>
@@ -24538,6 +24561,7 @@
     <hyperlink ref="A854" r:id="rId853"/>
     <hyperlink ref="A855" r:id="rId854"/>
     <hyperlink ref="A856" r:id="rId855"/>
+    <hyperlink ref="A857" r:id="rId856"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -24582,22 +24606,22 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2037</v>
+        <v>2040</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2038</v>
+        <v>599</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>124</v>
+        <v>435</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>272</v>
+        <v>253</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2039</v>
+        <v>591</v>
       </c>
       <c r="F2" s="2">
-        <v>46248.46805555555</v>
+        <v>46251.53125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-08-18 12:19
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4297" uniqueCount="2041">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4302" uniqueCount="2043">
   <si>
     <t>link</t>
   </si>
@@ -6141,6 +6141,12 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/aluksne/kblfk.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/turku-pag/hjbcb.html</t>
+  </si>
+  <si>
+    <t>76860030034</t>
   </si>
 </sst>
 </file>
@@ -6553,7 +6559,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F857"/>
+  <dimension ref="A1:F858"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23702,6 +23708,26 @@
       </c>
       <c r="F857" s="2">
         <v>46248.46805555555</v>
+      </c>
+    </row>
+    <row r="858" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A858" s="3" t="s">
+        <v>2040</v>
+      </c>
+      <c r="B858" s="4" t="s">
+        <v>599</v>
+      </c>
+      <c r="C858" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D858" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="E858" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="F858" s="2">
+        <v>46251.53125</v>
       </c>
     </row>
   </sheetData>
@@ -24562,6 +24588,7 @@
     <hyperlink ref="A855" r:id="rId854"/>
     <hyperlink ref="A856" r:id="rId855"/>
     <hyperlink ref="A857" r:id="rId856"/>
+    <hyperlink ref="A858" r:id="rId857"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -24606,22 +24633,22 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2040</v>
+        <v>2041</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>599</v>
+        <v>562</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>435</v>
+        <v>284</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>253</v>
+        <v>194</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>591</v>
+        <v>2042</v>
       </c>
       <c r="F2" s="2">
-        <v>46251.53125</v>
+        <v>46251.853472222225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-08-19 12:18
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -6559,7 +6559,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F858"/>
+  <dimension ref="A1:F859"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23728,6 +23728,26 @@
       </c>
       <c r="F858" s="2">
         <v>46251.53125</v>
+      </c>
+    </row>
+    <row r="859" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A859" s="3" t="s">
+        <v>2041</v>
+      </c>
+      <c r="B859" s="4" t="s">
+        <v>562</v>
+      </c>
+      <c r="C859" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D859" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="E859" s="4" t="s">
+        <v>2042</v>
+      </c>
+      <c r="F859" s="2">
+        <v>46251.853472222225</v>
       </c>
     </row>
   </sheetData>
@@ -24589,6 +24609,7 @@
     <hyperlink ref="A856" r:id="rId855"/>
     <hyperlink ref="A857" r:id="rId856"/>
     <hyperlink ref="A858" r:id="rId857"/>
+    <hyperlink ref="A859" r:id="rId858"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -24600,7 +24621,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24631,30 +24652,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>2041</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>562</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>2042</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46251.853472222225</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-08-20 12:20
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4302" uniqueCount="2043">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4307" uniqueCount="2044">
   <si>
     <t>link</t>
   </si>
@@ -6147,6 +6147,9 @@
   </si>
   <si>
     <t>76860030034</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/aizkalnes-pag/kljfk.html</t>
   </si>
 </sst>
 </file>
@@ -24621,7 +24624,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24652,7 +24655,30 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>2043</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46254.37569444445</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-08-21 12:20
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4307" uniqueCount="2044">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4312" uniqueCount="2046">
   <si>
     <t>link</t>
   </si>
@@ -6150,6 +6150,12 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/aizkalnes-pag/kljfk.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ludza-and-reg/malnavas-pag/ghpof.html</t>
+  </si>
+  <si>
+    <t>68680060095</t>
   </si>
 </sst>
 </file>
@@ -6562,7 +6568,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F859"/>
+  <dimension ref="A1:F860"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23751,6 +23757,26 @@
       </c>
       <c r="F859" s="2">
         <v>46251.853472222225</v>
+      </c>
+    </row>
+    <row r="860" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A860" s="3" t="s">
+        <v>2043</v>
+      </c>
+      <c r="B860" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C860" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D860" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E860" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F860" s="2">
+        <v>46254.37569444445</v>
       </c>
     </row>
   </sheetData>
@@ -24613,6 +24639,7 @@
     <hyperlink ref="A857" r:id="rId856"/>
     <hyperlink ref="A858" r:id="rId857"/>
     <hyperlink ref="A859" r:id="rId858"/>
+    <hyperlink ref="A860" r:id="rId859"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -24657,22 +24684,22 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2043</v>
+        <v>2044</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>116</v>
+        <v>161</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>284</v>
+        <v>234</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>36</v>
+        <v>212</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>25</v>
+        <v>2045</v>
       </c>
       <c r="F2" s="2">
-        <v>46254.37569444445</v>
+        <v>46255.47083333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-08-24 12:21
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4312" uniqueCount="2046">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4327" uniqueCount="2052">
   <si>
     <t>link</t>
   </si>
@@ -6156,6 +6156,24 @@
   </si>
   <si>
     <t>68680060095</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/vectilzas-pag/ekjex.html</t>
+  </si>
+  <si>
+    <t>38900050014</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/ilukste/inheh.html</t>
+  </si>
+  <si>
+    <t>7.35 ha.</t>
+  </si>
+  <si>
+    <t>44880010170</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ventspils-and-reg/ances-pag/eochi.html</t>
   </si>
 </sst>
 </file>
@@ -6568,7 +6586,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F860"/>
+  <dimension ref="A1:F861"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23777,6 +23795,26 @@
       </c>
       <c r="F860" s="2">
         <v>46254.37569444445</v>
+      </c>
+    </row>
+    <row r="861" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A861" s="3" t="s">
+        <v>2044</v>
+      </c>
+      <c r="B861" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C861" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D861" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="E861" s="4" t="s">
+        <v>2045</v>
+      </c>
+      <c r="F861" s="2">
+        <v>46255.47083333333</v>
       </c>
     </row>
   </sheetData>
@@ -24640,6 +24678,7 @@
     <hyperlink ref="A858" r:id="rId857"/>
     <hyperlink ref="A859" r:id="rId858"/>
     <hyperlink ref="A860" r:id="rId859"/>
+    <hyperlink ref="A861" r:id="rId860"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -24651,7 +24690,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24684,27 +24723,69 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2044</v>
+        <v>2046</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>161</v>
+        <v>437</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>234</v>
+        <v>28</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>212</v>
+        <v>67</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2045</v>
+        <v>2047</v>
       </c>
       <c r="F2" s="2">
-        <v>46255.47083333333</v>
+        <v>46256.75069444445</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>2048</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>2049</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>2050</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46257.788194444445</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>2051</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>513</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>1982</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46256.94027777778</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-08-25 12:21
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -6586,7 +6586,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F861"/>
+  <dimension ref="A1:F864"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23815,6 +23815,66 @@
       </c>
       <c r="F861" s="2">
         <v>46255.47083333333</v>
+      </c>
+    </row>
+    <row r="862" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A862" s="3" t="s">
+        <v>2046</v>
+      </c>
+      <c r="B862" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="C862" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D862" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E862" s="4" t="s">
+        <v>2047</v>
+      </c>
+      <c r="F862" s="2">
+        <v>46256.75069444445</v>
+      </c>
+    </row>
+    <row r="863" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A863" s="3" t="s">
+        <v>2048</v>
+      </c>
+      <c r="B863" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C863" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D863" s="4" t="s">
+        <v>2049</v>
+      </c>
+      <c r="E863" s="4" t="s">
+        <v>2050</v>
+      </c>
+      <c r="F863" s="2">
+        <v>46257.788194444445</v>
+      </c>
+    </row>
+    <row r="864" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A864" s="3" t="s">
+        <v>2051</v>
+      </c>
+      <c r="B864" s="4" t="s">
+        <v>513</v>
+      </c>
+      <c r="C864" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D864" s="4" t="s">
+        <v>1982</v>
+      </c>
+      <c r="E864" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F864" s="2">
+        <v>46256.94027777778</v>
       </c>
     </row>
   </sheetData>
@@ -24679,6 +24739,9 @@
     <hyperlink ref="A859" r:id="rId858"/>
     <hyperlink ref="A860" r:id="rId859"/>
     <hyperlink ref="A861" r:id="rId860"/>
+    <hyperlink ref="A862" r:id="rId861"/>
+    <hyperlink ref="A863" r:id="rId862"/>
+    <hyperlink ref="A864" r:id="rId863"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -24690,7 +24753,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24721,72 +24784,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>2046</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>437</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>2047</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46256.75069444445</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>2048</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>2049</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>2050</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46257.788194444445</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>2051</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>513</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>404</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>1982</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46256.94027777778</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-08-26 12:23
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4327" uniqueCount="2052">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4332" uniqueCount="2054">
   <si>
     <t>link</t>
   </si>
@@ -6174,6 +6174,12 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/ventspils-and-reg/ances-pag/eochi.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valka-and-reg/valka/kcbxi.html</t>
+  </si>
+  <si>
+    <t>1 m²</t>
   </si>
 </sst>
 </file>
@@ -24753,7 +24759,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24784,7 +24790,30 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>2052</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>969</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>2053</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46259.75</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-08-27 21:22
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4332" uniqueCount="2054">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4352" uniqueCount="2061">
   <si>
     <t>link</t>
   </si>
@@ -6180,6 +6180,27 @@
   </si>
   <si>
     <t>1 m²</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/demenes-pag/mjjej.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/tukums-and-reg/matkules-pag/ocgce.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/tukums-and-reg/zentenes-pag/fdmed.html</t>
+  </si>
+  <si>
+    <t>92 500 €</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valmiera-and-reg/burtnieku-pag/jdodx.html</t>
+  </si>
+  <si>
+    <t>36 ha.</t>
+  </si>
+  <si>
+    <t>96480150014</t>
   </si>
 </sst>
 </file>
@@ -6592,7 +6613,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F864"/>
+  <dimension ref="A1:F865"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23881,6 +23902,26 @@
       </c>
       <c r="F864" s="2">
         <v>46256.94027777778</v>
+      </c>
+    </row>
+    <row r="865" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A865" s="3" t="s">
+        <v>2052</v>
+      </c>
+      <c r="B865" s="4" t="s">
+        <v>969</v>
+      </c>
+      <c r="C865" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="D865" s="4" t="s">
+        <v>2053</v>
+      </c>
+      <c r="E865" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F865" s="2">
+        <v>46259.75</v>
       </c>
     </row>
   </sheetData>
@@ -24748,6 +24789,7 @@
     <hyperlink ref="A862" r:id="rId861"/>
     <hyperlink ref="A863" r:id="rId862"/>
     <hyperlink ref="A864" r:id="rId863"/>
+    <hyperlink ref="A865" r:id="rId864"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -24759,7 +24801,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24792,27 +24834,90 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2052</v>
+        <v>2054</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>969</v>
+        <v>161</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>392</v>
+        <v>74</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>2053</v>
+        <v>67</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46259.75</v>
+        <v>46261.925</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>2055</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>1939</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1940</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46261.51111111111</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>2056</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>2057</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46261.37222222222</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>2058</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>1557</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>2059</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>2060</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46261.67708333333</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-08-28 21:34
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4352" uniqueCount="2061">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4362" uniqueCount="2066">
   <si>
     <t>link</t>
   </si>
@@ -6201,6 +6201,21 @@
   </si>
   <si>
     <t>96480150014</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/liepaja-and-reg/embutes-pag/kodbp.html</t>
+  </si>
+  <si>
+    <t>64540040106</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/other/aedpx.html</t>
+  </si>
+  <si>
+    <t>280 €</t>
+  </si>
+  <si>
+    <t>100 m²</t>
   </si>
 </sst>
 </file>
@@ -6613,7 +6628,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F865"/>
+  <dimension ref="A1:F869"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -23922,6 +23937,86 @@
       </c>
       <c r="F865" s="2">
         <v>46259.75</v>
+      </c>
+    </row>
+    <row r="866" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A866" s="3" t="s">
+        <v>2054</v>
+      </c>
+      <c r="B866" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C866" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D866" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E866" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F866" s="2">
+        <v>46261.925</v>
+      </c>
+    </row>
+    <row r="867" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A867" s="3" t="s">
+        <v>2055</v>
+      </c>
+      <c r="B867" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="C867" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D867" s="4" t="s">
+        <v>1939</v>
+      </c>
+      <c r="E867" s="4" t="s">
+        <v>1940</v>
+      </c>
+      <c r="F867" s="2">
+        <v>46261.51111111111</v>
+      </c>
+    </row>
+    <row r="868" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A868" s="3" t="s">
+        <v>2056</v>
+      </c>
+      <c r="B868" s="4" t="s">
+        <v>2057</v>
+      </c>
+      <c r="C868" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D868" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E868" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F868" s="2">
+        <v>46261.37222222222</v>
+      </c>
+    </row>
+    <row r="869" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A869" s="3" t="s">
+        <v>2058</v>
+      </c>
+      <c r="B869" s="4" t="s">
+        <v>1557</v>
+      </c>
+      <c r="C869" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D869" s="4" t="s">
+        <v>2059</v>
+      </c>
+      <c r="E869" s="4" t="s">
+        <v>2060</v>
+      </c>
+      <c r="F869" s="2">
+        <v>46261.67708333333</v>
       </c>
     </row>
   </sheetData>
@@ -24790,6 +24885,10 @@
     <hyperlink ref="A863" r:id="rId862"/>
     <hyperlink ref="A864" r:id="rId863"/>
     <hyperlink ref="A865" r:id="rId864"/>
+    <hyperlink ref="A866" r:id="rId865"/>
+    <hyperlink ref="A867" r:id="rId866"/>
+    <hyperlink ref="A868" r:id="rId867"/>
+    <hyperlink ref="A869" r:id="rId868"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -24801,7 +24900,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24834,90 +24933,48 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2054</v>
+        <v>2061</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>161</v>
+        <v>1735</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>74</v>
+        <v>190</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>67</v>
+        <v>9</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>25</v>
+        <v>2062</v>
       </c>
       <c r="F2" s="2">
-        <v>46261.925</v>
+        <v>46262.38541666667</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>2055</v>
+        <v>2063</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>217</v>
+        <v>2064</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>376</v>
+        <v>25</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>1939</v>
+        <v>2065</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>1940</v>
+        <v>25</v>
       </c>
       <c r="F3" s="2">
-        <v>46261.51111111111</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>2056</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>2057</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>376</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46261.37222222222</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>2058</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>1557</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>2059</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>2060</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46261.67708333333</v>
+        <v>46262.63125</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-08-31 18:18
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4362" uniqueCount="2066">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4372" uniqueCount="2073">
   <si>
     <t>link</t>
   </si>
@@ -6216,6 +6216,27 @@
   </si>
   <si>
     <t>100 m²</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/drustu-pag/bghdk.html</t>
+  </si>
+  <si>
+    <t>145 000 €</t>
+  </si>
+  <si>
+    <t>42480090127</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valmiera-and-reg/diklu-pag/fkjih.html</t>
+  </si>
+  <si>
+    <t>180 000 €</t>
+  </si>
+  <si>
+    <t>42 ha.</t>
+  </si>
+  <si>
+    <t>9652-004-0063</t>
   </si>
 </sst>
 </file>
@@ -6628,7 +6649,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F869"/>
+  <dimension ref="A1:F871"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24017,6 +24038,46 @@
       </c>
       <c r="F869" s="2">
         <v>46261.67708333333</v>
+      </c>
+    </row>
+    <row r="870" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A870" s="3" t="s">
+        <v>2061</v>
+      </c>
+      <c r="B870" s="4" t="s">
+        <v>1735</v>
+      </c>
+      <c r="C870" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="D870" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E870" s="4" t="s">
+        <v>2062</v>
+      </c>
+      <c r="F870" s="2">
+        <v>46262.38541666667</v>
+      </c>
+    </row>
+    <row r="871" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A871" s="3" t="s">
+        <v>2063</v>
+      </c>
+      <c r="B871" s="4" t="s">
+        <v>2064</v>
+      </c>
+      <c r="C871" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D871" s="4" t="s">
+        <v>2065</v>
+      </c>
+      <c r="E871" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F871" s="2">
+        <v>46262.63125</v>
       </c>
     </row>
   </sheetData>
@@ -24889,6 +24950,8 @@
     <hyperlink ref="A867" r:id="rId866"/>
     <hyperlink ref="A868" r:id="rId867"/>
     <hyperlink ref="A869" r:id="rId868"/>
+    <hyperlink ref="A870" r:id="rId869"/>
+    <hyperlink ref="A871" r:id="rId870"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -24933,42 +24996,42 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2061</v>
+        <v>2066</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1735</v>
+        <v>2067</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>190</v>
+        <v>63</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>9</v>
+        <v>478</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2062</v>
+        <v>2068</v>
       </c>
       <c r="F2" s="2">
-        <v>46262.38541666667</v>
+        <v>46263.75902777778</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>2063</v>
+        <v>2069</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>2064</v>
+        <v>2070</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>25</v>
+        <v>396</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>2065</v>
+        <v>2071</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>25</v>
+        <v>2072</v>
       </c>
       <c r="F3" s="2">
-        <v>46262.63125</v>
+        <v>46263.28194444445</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-09-01 15:39
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4372" uniqueCount="2073">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4382" uniqueCount="2080">
   <si>
     <t>link</t>
   </si>
@@ -6237,6 +6237,27 @@
   </si>
   <si>
     <t>9652-004-0063</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aizkraukle-and-reg/skriveru-pag/ejmhx.html</t>
+  </si>
+  <si>
+    <t>5.04 ha.</t>
+  </si>
+  <si>
+    <t>32820030053</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ogre-and-reg/birzgales-pag/lmelc.html</t>
+  </si>
+  <si>
+    <t>79 900 €</t>
+  </si>
+  <si>
+    <t>6.56 ha.</t>
+  </si>
+  <si>
+    <t>74440070157</t>
   </si>
 </sst>
 </file>
@@ -6649,7 +6670,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F871"/>
+  <dimension ref="A1:F873"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24078,6 +24099,46 @@
       </c>
       <c r="F871" s="2">
         <v>46262.63125</v>
+      </c>
+    </row>
+    <row r="872" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A872" s="3" t="s">
+        <v>2066</v>
+      </c>
+      <c r="B872" s="4" t="s">
+        <v>2067</v>
+      </c>
+      <c r="C872" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D872" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="E872" s="4" t="s">
+        <v>2068</v>
+      </c>
+      <c r="F872" s="2">
+        <v>46263.75902777778</v>
+      </c>
+    </row>
+    <row r="873" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A873" s="3" t="s">
+        <v>2069</v>
+      </c>
+      <c r="B873" s="4" t="s">
+        <v>2070</v>
+      </c>
+      <c r="C873" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D873" s="4" t="s">
+        <v>2071</v>
+      </c>
+      <c r="E873" s="4" t="s">
+        <v>2072</v>
+      </c>
+      <c r="F873" s="2">
+        <v>46263.28194444445</v>
       </c>
     </row>
   </sheetData>
@@ -24952,6 +25013,8 @@
     <hyperlink ref="A869" r:id="rId868"/>
     <hyperlink ref="A870" r:id="rId869"/>
     <hyperlink ref="A871" r:id="rId870"/>
+    <hyperlink ref="A872" r:id="rId871"/>
+    <hyperlink ref="A873" r:id="rId872"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -24996,42 +25059,42 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2066</v>
+        <v>2073</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2067</v>
+        <v>116</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>63</v>
+        <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>478</v>
+        <v>2074</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2068</v>
+        <v>2075</v>
       </c>
       <c r="F2" s="2">
-        <v>46263.75902777778</v>
+        <v>46266.77291666667</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>2069</v>
+        <v>2076</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>2070</v>
+        <v>2077</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>396</v>
+        <v>275</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>2071</v>
+        <v>2078</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>2072</v>
+        <v>2079</v>
       </c>
       <c r="F3" s="2">
-        <v>46263.28194444445</v>
+        <v>46266.70972222222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-09-02 15:27
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4382" uniqueCount="2080">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4392" uniqueCount="2084">
   <si>
     <t>link</t>
   </si>
@@ -6258,6 +6258,18 @@
   </si>
   <si>
     <t>74440070157</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/gulbene-and-reg/lejasciema-pag/bpnjmh.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ludza-and-reg/cirmas-pag/hkdmn.html</t>
+  </si>
+  <si>
+    <t>9.80 ha.</t>
+  </si>
+  <si>
+    <t>6850-002-0107</t>
   </si>
 </sst>
 </file>
@@ -6670,7 +6682,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F873"/>
+  <dimension ref="A1:F875"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24139,6 +24151,46 @@
       </c>
       <c r="F873" s="2">
         <v>46263.28194444445</v>
+      </c>
+    </row>
+    <row r="874" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A874" s="3" t="s">
+        <v>2073</v>
+      </c>
+      <c r="B874" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C874" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D874" s="4" t="s">
+        <v>2074</v>
+      </c>
+      <c r="E874" s="4" t="s">
+        <v>2075</v>
+      </c>
+      <c r="F874" s="2">
+        <v>46266.77291666667</v>
+      </c>
+    </row>
+    <row r="875" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A875" s="3" t="s">
+        <v>2076</v>
+      </c>
+      <c r="B875" s="4" t="s">
+        <v>2077</v>
+      </c>
+      <c r="C875" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="D875" s="4" t="s">
+        <v>2078</v>
+      </c>
+      <c r="E875" s="4" t="s">
+        <v>2079</v>
+      </c>
+      <c r="F875" s="2">
+        <v>46266.70972222222</v>
       </c>
     </row>
   </sheetData>
@@ -25015,6 +25067,8 @@
     <hyperlink ref="A871" r:id="rId870"/>
     <hyperlink ref="A872" r:id="rId871"/>
     <hyperlink ref="A873" r:id="rId872"/>
+    <hyperlink ref="A874" r:id="rId873"/>
+    <hyperlink ref="A875" r:id="rId874"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25059,42 +25113,42 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2073</v>
+        <v>2080</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>116</v>
+        <v>52</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>8</v>
+        <v>124</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>2074</v>
+        <v>59</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2075</v>
+        <v>895</v>
       </c>
       <c r="F2" s="2">
-        <v>46266.77291666667</v>
+        <v>46266.865277777775</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>2076</v>
+        <v>2081</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>2077</v>
+        <v>1019</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>275</v>
+        <v>234</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>2078</v>
+        <v>2082</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>2079</v>
+        <v>2083</v>
       </c>
       <c r="F3" s="2">
-        <v>46266.70972222222</v>
+        <v>46266.81805555556</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-09-03 15:21
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -6682,7 +6682,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F875"/>
+  <dimension ref="A1:F877"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24191,6 +24191,46 @@
       </c>
       <c r="F875" s="2">
         <v>46266.70972222222</v>
+      </c>
+    </row>
+    <row r="876" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A876" s="3" t="s">
+        <v>2080</v>
+      </c>
+      <c r="B876" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C876" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D876" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E876" s="4" t="s">
+        <v>895</v>
+      </c>
+      <c r="F876" s="2">
+        <v>46266.865277777775</v>
+      </c>
+    </row>
+    <row r="877" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A877" s="3" t="s">
+        <v>2081</v>
+      </c>
+      <c r="B877" s="4" t="s">
+        <v>1019</v>
+      </c>
+      <c r="C877" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D877" s="4" t="s">
+        <v>2082</v>
+      </c>
+      <c r="E877" s="4" t="s">
+        <v>2083</v>
+      </c>
+      <c r="F877" s="2">
+        <v>46266.81805555556</v>
       </c>
     </row>
   </sheetData>
@@ -25069,6 +25109,8 @@
     <hyperlink ref="A873" r:id="rId872"/>
     <hyperlink ref="A874" r:id="rId873"/>
     <hyperlink ref="A875" r:id="rId874"/>
+    <hyperlink ref="A876" r:id="rId875"/>
+    <hyperlink ref="A877" r:id="rId876"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25080,7 +25122,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25111,51 +25153,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>2080</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>895</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46266.865277777775</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>2081</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>1019</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>2082</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>2083</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46266.81805555556</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-09-04 15:15
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4392" uniqueCount="2084">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4397" uniqueCount="2087">
   <si>
     <t>link</t>
   </si>
@@ -6270,6 +6270,15 @@
   </si>
   <si>
     <t>6850-002-0107</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/dzelzavas-pag/gfigd.html</t>
+  </si>
+  <si>
+    <t>14.79 ha.</t>
+  </si>
+  <si>
+    <t>70500030164</t>
   </si>
 </sst>
 </file>
@@ -25122,7 +25131,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25153,7 +25162,30 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>2084</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>745</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>2085</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>2086</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46269.35486111111</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-09-07 16:44
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4397" uniqueCount="2087">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4407" uniqueCount="2093">
   <si>
     <t>link</t>
   </si>
@@ -6279,6 +6279,24 @@
   </si>
   <si>
     <t>70500030164</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/nitaures-pag/iihhg.html</t>
+  </si>
+  <si>
+    <t>56000 m²</t>
+  </si>
+  <si>
+    <t>42680090041</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/ligatne/hjhdg.html</t>
+  </si>
+  <si>
+    <t>235000 m²</t>
+  </si>
+  <si>
+    <t>4262 0010113</t>
   </si>
 </sst>
 </file>
@@ -6691,7 +6709,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F877"/>
+  <dimension ref="A1:F878"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24240,6 +24258,26 @@
       </c>
       <c r="F877" s="2">
         <v>46266.81805555556</v>
+      </c>
+    </row>
+    <row r="878" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A878" s="3" t="s">
+        <v>2084</v>
+      </c>
+      <c r="B878" s="4" t="s">
+        <v>745</v>
+      </c>
+      <c r="C878" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D878" s="4" t="s">
+        <v>2085</v>
+      </c>
+      <c r="E878" s="4" t="s">
+        <v>2086</v>
+      </c>
+      <c r="F878" s="2">
+        <v>46269.35486111111</v>
       </c>
     </row>
   </sheetData>
@@ -25120,6 +25158,7 @@
     <hyperlink ref="A875" r:id="rId874"/>
     <hyperlink ref="A876" r:id="rId875"/>
     <hyperlink ref="A877" r:id="rId876"/>
+    <hyperlink ref="A878" r:id="rId877"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25131,7 +25170,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25164,27 +25203,48 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2084</v>
+        <v>2087</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>745</v>
+        <v>31</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>256</v>
+        <v>63</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>2085</v>
+        <v>2088</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2086</v>
+        <v>2089</v>
       </c>
       <c r="F2" s="2">
-        <v>46269.35486111111</v>
+        <v>46270.96666666667</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>2090</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>673</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>2091</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>2092</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46270.959027777775</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-09-08 15:29
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4407" uniqueCount="2093">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4412" uniqueCount="2096">
   <si>
     <t>link</t>
   </si>
@@ -6297,6 +6297,15 @@
   </si>
   <si>
     <t>4262 0010113</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/liepaja-and-reg/sakas-pag/fjjef.html</t>
+  </si>
+  <si>
+    <t>82 000 €</t>
+  </si>
+  <si>
+    <t>64860020012</t>
   </si>
 </sst>
 </file>
@@ -6709,7 +6718,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F878"/>
+  <dimension ref="A1:F880"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24278,6 +24287,46 @@
       </c>
       <c r="F878" s="2">
         <v>46269.35486111111</v>
+      </c>
+    </row>
+    <row r="879" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A879" s="3" t="s">
+        <v>2087</v>
+      </c>
+      <c r="B879" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C879" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D879" s="4" t="s">
+        <v>2088</v>
+      </c>
+      <c r="E879" s="4" t="s">
+        <v>2089</v>
+      </c>
+      <c r="F879" s="2">
+        <v>46270.96666666667</v>
+      </c>
+    </row>
+    <row r="880" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A880" s="3" t="s">
+        <v>2090</v>
+      </c>
+      <c r="B880" s="4" t="s">
+        <v>673</v>
+      </c>
+      <c r="C880" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D880" s="4" t="s">
+        <v>2091</v>
+      </c>
+      <c r="E880" s="4" t="s">
+        <v>2092</v>
+      </c>
+      <c r="F880" s="2">
+        <v>46270.959027777775</v>
       </c>
     </row>
   </sheetData>
@@ -25159,6 +25208,8 @@
     <hyperlink ref="A876" r:id="rId875"/>
     <hyperlink ref="A877" r:id="rId876"/>
     <hyperlink ref="A878" r:id="rId877"/>
+    <hyperlink ref="A879" r:id="rId878"/>
+    <hyperlink ref="A880" r:id="rId879"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25170,7 +25221,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25203,48 +25254,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2087</v>
+        <v>2093</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>31</v>
+        <v>2094</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>63</v>
+        <v>190</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>2088</v>
+        <v>75</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2089</v>
+        <v>2095</v>
       </c>
       <c r="F2" s="2">
-        <v>46270.96666666667</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>2090</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>673</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>2091</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>2092</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46270.959027777775</v>
+        <v>46273.683333333334</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-09-09 15:25
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -6718,7 +6718,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F880"/>
+  <dimension ref="A1:F881"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24327,6 +24327,26 @@
       </c>
       <c r="F880" s="2">
         <v>46270.959027777775</v>
+      </c>
+    </row>
+    <row r="881" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A881" s="3" t="s">
+        <v>2093</v>
+      </c>
+      <c r="B881" s="4" t="s">
+        <v>2094</v>
+      </c>
+      <c r="C881" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="D881" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E881" s="4" t="s">
+        <v>2095</v>
+      </c>
+      <c r="F881" s="2">
+        <v>46273.683333333334</v>
       </c>
     </row>
   </sheetData>
@@ -25210,6 +25230,7 @@
     <hyperlink ref="A878" r:id="rId877"/>
     <hyperlink ref="A879" r:id="rId878"/>
     <hyperlink ref="A880" r:id="rId879"/>
+    <hyperlink ref="A881" r:id="rId880"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25221,7 +25242,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25252,30 +25273,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>2093</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>2094</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>2095</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46273.683333333334</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-09-10 15:20
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4412" uniqueCount="2096">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4417" uniqueCount="2100">
   <si>
     <t>link</t>
   </si>
@@ -6306,6 +6306,18 @@
   </si>
   <si>
     <t>64860020012</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/sarkanu-pag/idpoj.html</t>
+  </si>
+  <si>
+    <t>30 400 €</t>
+  </si>
+  <si>
+    <t>5.20 ha.</t>
+  </si>
+  <si>
+    <t>70900010015</t>
   </si>
 </sst>
 </file>
@@ -25242,7 +25254,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25273,7 +25285,30 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>2096</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>2097</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>2098</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>2099</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46275.40347222222</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-09-11 15:21
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4417" uniqueCount="2100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4422" uniqueCount="2103">
   <si>
     <t>link</t>
   </si>
@@ -6318,6 +6318,15 @@
   </si>
   <si>
     <t>70900010015</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/ziemera-pag/bxjnbn.html</t>
+  </si>
+  <si>
+    <t>18.80 ha.</t>
+  </si>
+  <si>
+    <t>3696-005-0125</t>
   </si>
 </sst>
 </file>
@@ -6730,7 +6739,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F881"/>
+  <dimension ref="A1:F882"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24359,6 +24368,26 @@
       </c>
       <c r="F881" s="2">
         <v>46273.683333333334</v>
+      </c>
+    </row>
+    <row r="882" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A882" s="3" t="s">
+        <v>2096</v>
+      </c>
+      <c r="B882" s="4" t="s">
+        <v>2097</v>
+      </c>
+      <c r="C882" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D882" s="4" t="s">
+        <v>2098</v>
+      </c>
+      <c r="E882" s="4" t="s">
+        <v>2099</v>
+      </c>
+      <c r="F882" s="2">
+        <v>46275.40347222222</v>
       </c>
     </row>
   </sheetData>
@@ -25243,6 +25272,7 @@
     <hyperlink ref="A879" r:id="rId878"/>
     <hyperlink ref="A880" r:id="rId879"/>
     <hyperlink ref="A881" r:id="rId880"/>
+    <hyperlink ref="A882" r:id="rId881"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25287,22 +25317,22 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2096</v>
+        <v>2100</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2097</v>
+        <v>533</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>256</v>
+        <v>435</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>2098</v>
+        <v>2101</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2099</v>
+        <v>2102</v>
       </c>
       <c r="F2" s="2">
-        <v>46275.40347222222</v>
+        <v>46276.69861111111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>